<commit_message>
Atualização de dados: Controle Resumo - Base BSW (5).xlsx (07/05/2026 15:16)
</commit_message>
<xml_diff>
--- a/data/dados_atuais.xlsx
+++ b/data/dados_atuais.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://delgadiadema.sharepoint.com/sites/GestoEstratgica/Documentos Compartilhados/Controle Master/BSW/Novo controle (Em processo)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="675" documentId="1_{DDE4A242-D13A-46DE-8B65-653B9F6ECEB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01440C8C-64C3-470E-963D-5741F6CE805C}"/>
+  <xr:revisionPtr revIDLastSave="689" documentId="1_{DDE4A242-D13A-46DE-8B65-653B9F6ECEB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8F3BA450-5B28-412E-82C4-E944558592F1}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3E398004-7492-4AA0-94C2-EA9B761AAA49}"/>
   </bookViews>
@@ -321,7 +321,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6233" uniqueCount="1406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6243" uniqueCount="1408">
   <si>
     <t>Código
 Bobina Mâe</t>
@@ -4658,6 +4658,24 @@
   <si>
     <t>Produtos com processo de corte laser com reduções significativas no peso bruto unitário. Aumento da quantidade de peças / chapa.
 Em análise a redução do comprimento da chapa, mantendo a quantidade de peças / chapa.</t>
+  </si>
+  <si>
+    <t>DJ000059Z / 060Z</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Redução no passo do blank. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>AGUARDANDO RETORNO DO FORNECEDOR EM RELAÇÃO À MP.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -5407,7 +5425,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>0.37680005792085014</c:v>
+                  <c:v>0.38521698042732067</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6325,7 +6343,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>0.24010429823778848</c:v>
+                  <c:v>0.26354378919303767</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6984,7 +7002,7 @@
                   <c:v>885025.4800000001</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>20671.96</c:v>
+                  <c:v>38173.78</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -7279,7 +7297,7 @@
                 <c:formatCode>_("R$"* #,##0.00_);_("R$"* \(#,##0.00\);_("R$"* "-"??_);_(@_)</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>905697.44000000006</c:v>
+                  <c:v>923199.26000000013</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7651,7 +7669,7 @@
                   <c:v>1322.6778035000002</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>392.45735950000005</c:v>
+                  <c:v>430.76987950000006</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -13459,7 +13477,7 @@
       <c r="AL5" s="1"/>
       <c r="AM5" s="1"/>
     </row>
-    <row r="6" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
         <v>39</v>
       </c>
@@ -13753,7 +13771,7 @@
       <c r="AL8" s="1"/>
       <c r="AM8" s="1"/>
     </row>
-    <row r="9" spans="1:39" s="26" customFormat="1" ht="132.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:39" s="26" customFormat="1" ht="132.6" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
         <v>48</v>
       </c>
@@ -14089,7 +14107,7 @@
       <c r="AL11" s="1"/>
       <c r="AM11" s="1"/>
     </row>
-    <row r="12" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
         <v>56</v>
       </c>
@@ -14919,7 +14937,7 @@
       <c r="AL19" s="1"/>
       <c r="AM19" s="1"/>
     </row>
-    <row r="20" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
         <v>61</v>
       </c>
@@ -15027,7 +15045,7 @@
         <v>1400</v>
       </c>
     </row>
-    <row r="21" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
         <v>67</v>
       </c>
@@ -15751,7 +15769,7 @@
       <c r="AL27" s="1"/>
       <c r="AM27" s="1"/>
     </row>
-    <row r="28" spans="1:39" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:39" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A28" s="22" t="s">
         <v>72</v>
       </c>
@@ -15861,7 +15879,7 @@
         <v>1405</v>
       </c>
     </row>
-    <row r="29" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="22" t="s">
         <v>77</v>
       </c>
@@ -16041,7 +16059,7 @@
       <c r="AL30" s="1"/>
       <c r="AM30" s="1"/>
     </row>
-    <row r="31" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>81</v>
       </c>
@@ -16112,28 +16130,48 @@
         <f>AVERAGE(U31:X31)</f>
         <v>38.312520000000006</v>
       </c>
-      <c r="Z31" s="10"/>
-      <c r="AA31" s="10"/>
-      <c r="AB31" s="10"/>
-      <c r="AC31" s="10"/>
-      <c r="AD31" s="10"/>
-      <c r="AE31" s="10"/>
-      <c r="AF31" s="10"/>
+      <c r="Z31" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AA31" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AB31" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AC31" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AD31" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AE31" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AF31" s="10" t="s">
+        <v>693</v>
+      </c>
       <c r="AG31" s="38">
         <f>COUNTIF(Z31:AF31,"X")/7</f>
-        <v>0</v>
-      </c>
-      <c r="AH31" s="51" t="str">
+        <v>1</v>
+      </c>
+      <c r="AH31" s="51">
         <f>IF(AG31=100%,Y31," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="AI31" s="64"/>
-      <c r="AJ31" s="1"/>
+        <v>38.312520000000006</v>
+      </c>
+      <c r="AI31" s="64">
+        <v>2</v>
+      </c>
+      <c r="AJ31" s="1" t="s">
+        <v>1406</v>
+      </c>
       <c r="AK31" s="65">
-        <v>0</v>
+        <v>17501.82</v>
       </c>
       <c r="AL31" s="1"/>
-      <c r="AM31" s="1"/>
+      <c r="AM31" s="1" t="s">
+        <v>1398</v>
+      </c>
     </row>
     <row r="32" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="22" t="s">
@@ -16307,7 +16345,7 @@
       <c r="AL33" s="1"/>
       <c r="AM33" s="1"/>
     </row>
-    <row r="34" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="22" t="s">
         <v>86</v>
       </c>
@@ -16399,7 +16437,9 @@
         <v>0</v>
       </c>
       <c r="AL34" s="1"/>
-      <c r="AM34" s="1"/>
+      <c r="AM34" s="1" t="s">
+        <v>1407</v>
+      </c>
     </row>
     <row r="35" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="19" t="s">
@@ -16669,7 +16709,7 @@
       <c r="AL37" s="1"/>
       <c r="AM37" s="1"/>
     </row>
-    <row r="38" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="22" t="s">
         <v>89</v>
       </c>
@@ -16939,7 +16979,7 @@
       <c r="AL40" s="1"/>
       <c r="AM40" s="1"/>
     </row>
-    <row r="41" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="22" t="s">
         <v>95</v>
       </c>
@@ -17031,7 +17071,7 @@
       <c r="AL41" s="1"/>
       <c r="AM41" s="1"/>
     </row>
-    <row r="42" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="22" t="s">
         <v>97</v>
       </c>
@@ -17125,7 +17165,7 @@
       <c r="AL42" s="1"/>
       <c r="AM42" s="1"/>
     </row>
-    <row r="43" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="22" t="s">
         <v>100</v>
       </c>
@@ -17307,7 +17347,7 @@
       <c r="AL44" s="1"/>
       <c r="AM44" s="1"/>
     </row>
-    <row r="45" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="22" t="s">
         <v>103</v>
       </c>
@@ -17401,7 +17441,7 @@
       <c r="AL45" s="1"/>
       <c r="AM45" s="1"/>
     </row>
-    <row r="46" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="22" t="s">
         <v>109</v>
       </c>
@@ -17493,7 +17533,7 @@
       <c r="AL46" s="1"/>
       <c r="AM46" s="1"/>
     </row>
-    <row r="47" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="22" t="s">
         <v>113</v>
       </c>
@@ -17585,7 +17625,7 @@
       <c r="AL47" s="1"/>
       <c r="AM47" s="1"/>
     </row>
-    <row r="48" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="22" t="s">
         <v>117</v>
       </c>
@@ -17855,7 +17895,7 @@
       <c r="AL50" s="1"/>
       <c r="AM50" s="1"/>
     </row>
-    <row r="51" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A51" s="22" t="s">
         <v>121</v>
       </c>
@@ -18035,7 +18075,7 @@
       <c r="AL52" s="1"/>
       <c r="AM52" s="1"/>
     </row>
-    <row r="53" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A53" s="22" t="s">
         <v>124</v>
       </c>
@@ -18213,7 +18253,7 @@
       <c r="AL54" s="1"/>
       <c r="AM54" s="1"/>
     </row>
-    <row r="55" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A55" s="22" t="s">
         <v>126</v>
       </c>
@@ -18395,7 +18435,7 @@
       <c r="AL56" s="1"/>
       <c r="AM56" s="1"/>
     </row>
-    <row r="57" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A57" s="22" t="s">
         <v>127</v>
       </c>
@@ -18487,7 +18527,7 @@
       <c r="AL57" s="1"/>
       <c r="AM57" s="1"/>
     </row>
-    <row r="58" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A58" s="22" t="s">
         <v>129</v>
       </c>
@@ -18669,7 +18709,7 @@
       <c r="AL59" s="1"/>
       <c r="AM59" s="1"/>
     </row>
-    <row r="60" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A60" s="22" t="s">
         <v>131</v>
       </c>
@@ -18941,7 +18981,7 @@
       <c r="AL62" s="1"/>
       <c r="AM62" s="1"/>
     </row>
-    <row r="63" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A63" s="22" t="s">
         <v>134</v>
       </c>
@@ -19211,7 +19251,7 @@
       <c r="AL65" s="1"/>
       <c r="AM65" s="1"/>
     </row>
-    <row r="66" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A66" s="22" t="s">
         <v>137</v>
       </c>
@@ -19569,7 +19609,7 @@
       <c r="AL69" s="1"/>
       <c r="AM69" s="1"/>
     </row>
-    <row r="70" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A70" s="22" t="s">
         <v>139</v>
       </c>
@@ -19663,7 +19703,7 @@
       <c r="AL70" s="1"/>
       <c r="AM70" s="1"/>
     </row>
-    <row r="71" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A71" s="22" t="s">
         <v>140</v>
       </c>
@@ -19755,7 +19795,7 @@
       <c r="AL71" s="1"/>
       <c r="AM71" s="1"/>
     </row>
-    <row r="72" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A72" s="22" t="s">
         <v>143</v>
       </c>
@@ -19847,7 +19887,7 @@
       <c r="AL72" s="1"/>
       <c r="AM72" s="1"/>
     </row>
-    <row r="73" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A73" s="22" t="s">
         <v>147</v>
       </c>
@@ -20111,7 +20151,7 @@
       <c r="AL75" s="1"/>
       <c r="AM75" s="1"/>
     </row>
-    <row r="76" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A76" s="22" t="s">
         <v>151</v>
       </c>
@@ -20295,7 +20335,7 @@
       <c r="AL77" s="1"/>
       <c r="AM77" s="1"/>
     </row>
-    <row r="78" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A78" s="22" t="s">
         <v>157</v>
       </c>
@@ -20477,7 +20517,7 @@
       <c r="AL79" s="1"/>
       <c r="AM79" s="1"/>
     </row>
-    <row r="80" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A80" s="22" t="s">
         <v>161</v>
       </c>
@@ -20743,7 +20783,7 @@
       <c r="AL82" s="1"/>
       <c r="AM82" s="1"/>
     </row>
-    <row r="83" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A83" s="22" t="s">
         <v>162</v>
       </c>
@@ -20835,7 +20875,7 @@
       <c r="AL83" s="1"/>
       <c r="AM83" s="1"/>
     </row>
-    <row r="84" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A84" s="22" t="s">
         <v>165</v>
       </c>
@@ -21287,7 +21327,7 @@
       <c r="AL88" s="1"/>
       <c r="AM88" s="1"/>
     </row>
-    <row r="89" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A89" s="22" t="s">
         <v>171</v>
       </c>
@@ -21559,7 +21599,7 @@
       <c r="AL91" s="1"/>
       <c r="AM91" s="1"/>
     </row>
-    <row r="92" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A92" s="22" t="s">
         <v>174</v>
       </c>
@@ -21655,7 +21695,7 @@
       <c r="AL92" s="1"/>
       <c r="AM92" s="1"/>
     </row>
-    <row r="93" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A93" s="22" t="s">
         <v>176</v>
       </c>
@@ -21745,7 +21785,7 @@
       <c r="AL93" s="1"/>
       <c r="AM93" s="1"/>
     </row>
-    <row r="94" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A94" s="22" t="s">
         <v>178</v>
       </c>
@@ -22107,7 +22147,7 @@
       <c r="AL97" s="1"/>
       <c r="AM97" s="1"/>
     </row>
-    <row r="98" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A98" s="22" t="s">
         <v>180</v>
       </c>
@@ -22199,7 +22239,7 @@
       <c r="AL98" s="1"/>
       <c r="AM98" s="1"/>
     </row>
-    <row r="99" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A99" s="22" t="s">
         <v>184</v>
       </c>
@@ -22381,7 +22421,7 @@
       <c r="AL100" s="1"/>
       <c r="AM100" s="1"/>
     </row>
-    <row r="101" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A101" s="22" t="s">
         <v>188</v>
       </c>
@@ -22895,7 +22935,7 @@
       <c r="AL106" s="1"/>
       <c r="AM106" s="1"/>
     </row>
-    <row r="107" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A107" s="22" t="s">
         <v>191</v>
       </c>
@@ -22987,7 +23027,7 @@
       <c r="AL107" s="1"/>
       <c r="AM107" s="1"/>
     </row>
-    <row r="108" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A108" s="22" t="s">
         <v>197</v>
       </c>
@@ -23789,7 +23829,7 @@
       <c r="AL116" s="1"/>
       <c r="AM116" s="1"/>
     </row>
-    <row r="117" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A117" s="22" t="s">
         <v>199</v>
       </c>
@@ -23881,7 +23921,7 @@
       <c r="AL117" s="1"/>
       <c r="AM117" s="1"/>
     </row>
-    <row r="118" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A118" s="22" t="s">
         <v>201</v>
       </c>
@@ -23973,7 +24013,7 @@
       <c r="AL118" s="1"/>
       <c r="AM118" s="1"/>
     </row>
-    <row r="119" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A119" s="22" t="s">
         <v>204</v>
       </c>
@@ -24155,7 +24195,7 @@
       <c r="AL120" s="1"/>
       <c r="AM120" s="1"/>
     </row>
-    <row r="121" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A121" s="22" t="s">
         <v>207</v>
       </c>
@@ -24247,7 +24287,7 @@
       <c r="AL121" s="1"/>
       <c r="AM121" s="1"/>
     </row>
-    <row r="122" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A122" s="22" t="s">
         <v>210</v>
       </c>
@@ -24771,7 +24811,7 @@
       <c r="AL127" s="1"/>
       <c r="AM127" s="1"/>
     </row>
-    <row r="128" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A128" s="22" t="s">
         <v>212</v>
       </c>
@@ -24953,7 +24993,7 @@
       <c r="AL129" s="1"/>
       <c r="AM129" s="1"/>
     </row>
-    <row r="130" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A130" s="22" t="s">
         <v>216</v>
       </c>
@@ -25225,7 +25265,7 @@
       <c r="AL132" s="1"/>
       <c r="AM132" s="1"/>
     </row>
-    <row r="133" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A133" s="22" t="s">
         <v>221</v>
       </c>
@@ -25493,7 +25533,7 @@
       <c r="AL135" s="1"/>
       <c r="AM135" s="1"/>
     </row>
-    <row r="136" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A136" s="22" t="s">
         <v>223</v>
       </c>
@@ -25585,7 +25625,7 @@
       <c r="AL136" s="1"/>
       <c r="AM136" s="1"/>
     </row>
-    <row r="137" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A137" s="22" t="s">
         <v>225</v>
       </c>
@@ -25929,7 +25969,7 @@
       <c r="AL140" s="1"/>
       <c r="AM140" s="1"/>
     </row>
-    <row r="141" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A141" s="22" t="s">
         <v>227</v>
       </c>
@@ -26197,7 +26237,7 @@
       <c r="AL143" s="1"/>
       <c r="AM143" s="1"/>
     </row>
-    <row r="144" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A144" s="22" t="s">
         <v>228</v>
       </c>
@@ -26375,7 +26415,7 @@
       <c r="AL145" s="1"/>
       <c r="AM145" s="1"/>
     </row>
-    <row r="146" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A146" s="22" t="s">
         <v>232</v>
       </c>
@@ -26467,7 +26507,7 @@
       <c r="AL146" s="1"/>
       <c r="AM146" s="1"/>
     </row>
-    <row r="147" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A147" s="22" t="s">
         <v>234</v>
       </c>
@@ -26559,7 +26599,7 @@
       <c r="AL147" s="1"/>
       <c r="AM147" s="1"/>
     </row>
-    <row r="148" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A148" s="22" t="s">
         <v>236</v>
       </c>
@@ -26909,7 +26949,7 @@
       <c r="AL151" s="1"/>
       <c r="AM151" s="1"/>
     </row>
-    <row r="152" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A152" s="22" t="s">
         <v>240</v>
       </c>
@@ -27089,7 +27129,7 @@
       <c r="AL153" s="1"/>
       <c r="AM153" s="1"/>
     </row>
-    <row r="154" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A154" s="22" t="s">
         <v>243</v>
       </c>
@@ -27181,7 +27221,7 @@
       <c r="AL154" s="1"/>
       <c r="AM154" s="1"/>
     </row>
-    <row r="155" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A155" s="22" t="s">
         <v>245</v>
       </c>
@@ -27359,7 +27399,7 @@
       <c r="AL156" s="1"/>
       <c r="AM156" s="1"/>
     </row>
-    <row r="157" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A157" s="22" t="s">
         <v>246</v>
       </c>
@@ -27623,7 +27663,7 @@
       <c r="AL159" s="1"/>
       <c r="AM159" s="1"/>
     </row>
-    <row r="160" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A160" s="22" t="s">
         <v>249</v>
       </c>
@@ -27715,7 +27755,7 @@
       <c r="AL160" s="1"/>
       <c r="AM160" s="1"/>
     </row>
-    <row r="161" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A161" s="22" t="s">
         <v>251</v>
       </c>
@@ -27981,7 +28021,7 @@
       <c r="AL163" s="1"/>
       <c r="AM163" s="1"/>
     </row>
-    <row r="164" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A164" s="22" t="s">
         <v>253</v>
       </c>
@@ -28689,7 +28729,7 @@
       <c r="AL171" s="1"/>
       <c r="AM171" s="1"/>
     </row>
-    <row r="172" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A172" s="22" t="s">
         <v>256</v>
       </c>
@@ -28961,7 +29001,7 @@
       <c r="AL174" s="1"/>
       <c r="AM174" s="1"/>
     </row>
-    <row r="175" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A175" s="22" t="s">
         <v>258</v>
       </c>
@@ -29051,7 +29091,7 @@
       <c r="AL175" s="1"/>
       <c r="AM175" s="1"/>
     </row>
-    <row r="176" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A176" s="22" t="s">
         <v>261</v>
       </c>
@@ -29143,7 +29183,7 @@
       <c r="AL176" s="1"/>
       <c r="AM176" s="1"/>
     </row>
-    <row r="177" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A177" s="22" t="s">
         <v>265</v>
       </c>
@@ -29321,7 +29361,7 @@
       <c r="AL178" s="1"/>
       <c r="AM178" s="1"/>
     </row>
-    <row r="179" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A179" s="22" t="s">
         <v>268</v>
       </c>
@@ -29411,7 +29451,7 @@
       <c r="AL179" s="1"/>
       <c r="AM179" s="1"/>
     </row>
-    <row r="180" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A180" s="22" t="s">
         <v>270</v>
       </c>
@@ -29593,7 +29633,7 @@
       <c r="AL181" s="1"/>
       <c r="AM181" s="1"/>
     </row>
-    <row r="182" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A182" s="22" t="s">
         <v>272</v>
       </c>
@@ -29863,7 +29903,7 @@
       <c r="AL184" s="1"/>
       <c r="AM184" s="1"/>
     </row>
-    <row r="185" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A185" s="22" t="s">
         <v>275</v>
       </c>
@@ -29955,7 +29995,7 @@
       <c r="AL185" s="1"/>
       <c r="AM185" s="1"/>
     </row>
-    <row r="186" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A186" s="22" t="s">
         <v>278</v>
       </c>
@@ -30463,7 +30503,7 @@
       <c r="AL191" s="1"/>
       <c r="AM191" s="1"/>
     </row>
-    <row r="192" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A192" s="22" t="s">
         <v>281</v>
       </c>
@@ -30643,7 +30683,7 @@
       <c r="AL193" s="1"/>
       <c r="AM193" s="1"/>
     </row>
-    <row r="194" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A194" s="22" t="s">
         <v>283</v>
       </c>
@@ -31085,7 +31125,7 @@
       <c r="AL198" s="1"/>
       <c r="AM198" s="1"/>
     </row>
-    <row r="199" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A199" s="22" t="s">
         <v>285</v>
       </c>
@@ -31265,7 +31305,7 @@
       <c r="AL200" s="1"/>
       <c r="AM200" s="1"/>
     </row>
-    <row r="201" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A201" s="22" t="s">
         <v>287</v>
       </c>
@@ -31515,7 +31555,7 @@
       <c r="AL203" s="1"/>
       <c r="AM203" s="1"/>
     </row>
-    <row r="204" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A204" s="22" t="s">
         <v>289</v>
       </c>
@@ -31945,7 +31985,7 @@
       <c r="AL208" s="1"/>
       <c r="AM208" s="1"/>
     </row>
-    <row r="209" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A209" s="22" t="s">
         <v>292</v>
       </c>
@@ -32037,7 +32077,7 @@
       <c r="AL209" s="1"/>
       <c r="AM209" s="1"/>
     </row>
-    <row r="210" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A210" s="22" t="s">
         <v>294</v>
       </c>
@@ -32129,7 +32169,7 @@
       <c r="AL210" s="1"/>
       <c r="AM210" s="1"/>
     </row>
-    <row r="211" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A211" s="22" t="s">
         <v>299</v>
       </c>
@@ -32463,7 +32503,7 @@
       <c r="AL214" s="1"/>
       <c r="AM214" s="1"/>
     </row>
-    <row r="215" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A215" s="22" t="s">
         <v>303</v>
       </c>
@@ -32551,7 +32591,7 @@
       <c r="AL215" s="1"/>
       <c r="AM215" s="1"/>
     </row>
-    <row r="216" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A216" s="22" t="s">
         <v>307</v>
       </c>
@@ -32715,7 +32755,7 @@
       <c r="AL217" s="1"/>
       <c r="AM217" s="1"/>
     </row>
-    <row r="218" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A218" s="22" t="s">
         <v>310</v>
       </c>
@@ -32893,7 +32933,7 @@
       <c r="AL219" s="1"/>
       <c r="AM219" s="1"/>
     </row>
-    <row r="220" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A220" s="22" t="s">
         <v>312</v>
       </c>
@@ -34899,7 +34939,7 @@
       <c r="AL244" s="1"/>
       <c r="AM244" s="1"/>
     </row>
-    <row r="245" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A245" s="22" t="s">
         <v>315</v>
       </c>
@@ -36117,7 +36157,7 @@
       <c r="AL259" s="1"/>
       <c r="AM259" s="1"/>
     </row>
-    <row r="260" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A260" s="22" t="s">
         <v>318</v>
       </c>
@@ -36297,7 +36337,7 @@
       <c r="AL261" s="1"/>
       <c r="AM261" s="1"/>
     </row>
-    <row r="262" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A262" s="3" t="s">
         <v>320</v>
       </c>
@@ -36389,7 +36429,7 @@
       <c r="AL262" s="1"/>
       <c r="AM262" s="1"/>
     </row>
-    <row r="263" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A263" s="22" t="s">
         <v>324</v>
       </c>
@@ -36475,7 +36515,7 @@
       <c r="AL263" s="1"/>
       <c r="AM263" s="1"/>
     </row>
-    <row r="264" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A264" s="22" t="s">
         <v>325</v>
       </c>
@@ -36891,7 +36931,7 @@
       <c r="AL268" s="1"/>
       <c r="AM268" s="1"/>
     </row>
-    <row r="269" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A269" s="22" t="s">
         <v>327</v>
       </c>
@@ -37781,7 +37821,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="280" spans="1:39" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:39" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A280" s="22" t="s">
         <v>330</v>
       </c>
@@ -37871,7 +37911,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="281" spans="1:39" s="26" customFormat="1" ht="122.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:39" s="26" customFormat="1" ht="122.4" x14ac:dyDescent="0.3">
       <c r="A281" s="22" t="s">
         <v>333</v>
       </c>
@@ -38561,7 +38601,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="289" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A289" s="22" t="s">
         <v>336</v>
       </c>
@@ -39029,7 +39069,7 @@
       <c r="AL294" s="1"/>
       <c r="AM294" s="1"/>
     </row>
-    <row r="295" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A295" s="22" t="s">
         <v>337</v>
       </c>
@@ -39269,7 +39309,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="298" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A298" s="22" t="s">
         <v>339</v>
       </c>
@@ -39679,7 +39719,7 @@
       <c r="AL302" s="1"/>
       <c r="AM302" s="1"/>
     </row>
-    <row r="303" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A303" s="22" t="s">
         <v>341</v>
       </c>
@@ -39929,7 +39969,7 @@
       <c r="AL305" s="1"/>
       <c r="AM305" s="1"/>
     </row>
-    <row r="306" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A306" s="22" t="s">
         <v>343</v>
       </c>
@@ -40015,7 +40055,7 @@
       <c r="AL306" s="1"/>
       <c r="AM306" s="1"/>
     </row>
-    <row r="307" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A307" s="22" t="s">
         <v>344</v>
       </c>
@@ -40107,7 +40147,7 @@
       <c r="AL307" s="1"/>
       <c r="AM307" s="1"/>
     </row>
-    <row r="308" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A308" s="22" t="s">
         <v>346</v>
       </c>
@@ -40197,7 +40237,7 @@
       <c r="AL308" s="1"/>
       <c r="AM308" s="1"/>
     </row>
-    <row r="309" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A309" s="22" t="s">
         <v>348</v>
       </c>
@@ -40515,7 +40555,7 @@
       <c r="AL312" s="1"/>
       <c r="AM312" s="1"/>
     </row>
-    <row r="313" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A313" s="22" t="s">
         <v>350</v>
       </c>
@@ -40761,7 +40801,7 @@
       <c r="AL315" s="1"/>
       <c r="AM315" s="1"/>
     </row>
-    <row r="316" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A316" s="22" t="s">
         <v>352</v>
       </c>
@@ -41177,7 +41217,7 @@
       <c r="AL320" s="1"/>
       <c r="AM320" s="1"/>
     </row>
-    <row r="321" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A321" s="3" t="s">
         <v>354</v>
       </c>
@@ -41441,7 +41481,7 @@
       <c r="AL323" s="1"/>
       <c r="AM323" s="1"/>
     </row>
-    <row r="324" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A324" s="22" t="s">
         <v>356</v>
       </c>
@@ -41689,7 +41729,7 @@
       <c r="AL326" s="1"/>
       <c r="AM326" s="1"/>
     </row>
-    <row r="327" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A327" s="22" t="s">
         <v>358</v>
       </c>
@@ -41849,7 +41889,7 @@
       <c r="AL328" s="1"/>
       <c r="AM328" s="1"/>
     </row>
-    <row r="329" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A329" s="22" t="s">
         <v>362</v>
       </c>
@@ -41941,7 +41981,7 @@
       <c r="AL329" s="1"/>
       <c r="AM329" s="1"/>
     </row>
-    <row r="330" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A330" s="22" t="s">
         <v>364</v>
       </c>
@@ -42485,7 +42525,7 @@
       <c r="AL336" s="1"/>
       <c r="AM336" s="1"/>
     </row>
-    <row r="337" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A337" s="22" t="s">
         <v>366</v>
       </c>
@@ -42967,7 +43007,7 @@
       <c r="AL342" s="1"/>
       <c r="AM342" s="1"/>
     </row>
-    <row r="343" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A343" s="22" t="s">
         <v>368</v>
       </c>
@@ -43213,7 +43253,7 @@
       <c r="AL345" s="1"/>
       <c r="AM345" s="1"/>
     </row>
-    <row r="346" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A346" s="22" t="s">
         <v>370</v>
       </c>
@@ -43779,7 +43819,7 @@
       <c r="AL352" s="1"/>
       <c r="AM352" s="1"/>
     </row>
-    <row r="353" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A353" s="22" t="s">
         <v>372</v>
       </c>
@@ -44039,7 +44079,7 @@
       <c r="AL355" s="1"/>
       <c r="AM355" s="1"/>
     </row>
-    <row r="356" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A356" s="22" t="s">
         <v>373</v>
       </c>
@@ -44375,7 +44415,7 @@
       <c r="AL359" s="1"/>
       <c r="AM359" s="1"/>
     </row>
-    <row r="360" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A360" s="22" t="s">
         <v>375</v>
       </c>
@@ -44463,7 +44503,7 @@
       <c r="AL360" s="1"/>
       <c r="AM360" s="1"/>
     </row>
-    <row r="361" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A361" s="22" t="s">
         <v>378</v>
       </c>
@@ -45423,7 +45463,7 @@
       <c r="AL372" s="1"/>
       <c r="AM372" s="1"/>
     </row>
-    <row r="373" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A373" s="22" t="s">
         <v>380</v>
       </c>
@@ -45745,7 +45785,7 @@
       <c r="AL376" s="1"/>
       <c r="AM376" s="1"/>
     </row>
-    <row r="377" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A377" s="22" t="s">
         <v>383</v>
       </c>
@@ -45827,7 +45867,7 @@
       <c r="AL377" s="1"/>
       <c r="AM377" s="1"/>
     </row>
-    <row r="378" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A378" s="22" t="s">
         <v>384</v>
       </c>
@@ -46477,7 +46517,7 @@
       <c r="AL385" s="1"/>
       <c r="AM385" s="1"/>
     </row>
-    <row r="386" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A386" s="22" t="s">
         <v>385</v>
       </c>
@@ -46785,7 +46825,7 @@
       <c r="AL389" s="1"/>
       <c r="AM389" s="1"/>
     </row>
-    <row r="390" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A390" s="22" t="s">
         <v>387</v>
       </c>
@@ -46877,7 +46917,7 @@
       <c r="AL390" s="1"/>
       <c r="AM390" s="1"/>
     </row>
-    <row r="391" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="391" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A391" s="22" t="s">
         <v>389</v>
       </c>
@@ -46959,7 +46999,7 @@
       <c r="AL391" s="1"/>
       <c r="AM391" s="1"/>
     </row>
-    <row r="392" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A392" s="22" t="s">
         <v>390</v>
       </c>
@@ -47263,7 +47303,7 @@
       <c r="AL395" s="1"/>
       <c r="AM395" s="1"/>
     </row>
-    <row r="396" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A396" s="22" t="s">
         <v>392</v>
       </c>
@@ -47657,7 +47697,7 @@
       <c r="AL400" s="1"/>
       <c r="AM400" s="1"/>
     </row>
-    <row r="401" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A401" s="22" t="s">
         <v>394</v>
       </c>
@@ -47829,7 +47869,7 @@
       <c r="AL402" s="1"/>
       <c r="AM402" s="1"/>
     </row>
-    <row r="403" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A403" s="22" t="s">
         <v>396</v>
       </c>
@@ -47911,7 +47951,7 @@
       <c r="AL403" s="1"/>
       <c r="AM403" s="1"/>
     </row>
-    <row r="404" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A404" s="22" t="s">
         <v>397</v>
       </c>
@@ -48299,7 +48339,7 @@
       <c r="AL408" s="1"/>
       <c r="AM408" s="1"/>
     </row>
-    <row r="409" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="409" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A409" s="15" t="s">
         <v>400</v>
       </c>
@@ -48623,7 +48663,7 @@
       <c r="AL412" s="1"/>
       <c r="AM412" s="1"/>
     </row>
-    <row r="413" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="413" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A413" s="15" t="s">
         <v>402</v>
       </c>
@@ -48795,7 +48835,7 @@
       <c r="AL414" s="1"/>
       <c r="AM414" s="1"/>
     </row>
-    <row r="415" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="415" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A415" s="15" t="s">
         <v>403</v>
       </c>
@@ -48879,7 +48919,7 @@
       <c r="AL415" s="1"/>
       <c r="AM415" s="1"/>
     </row>
-    <row r="416" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="416" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A416" s="15" t="s">
         <v>404</v>
       </c>
@@ -49031,7 +49071,7 @@
       <c r="AL417" s="1"/>
       <c r="AM417" s="1"/>
     </row>
-    <row r="418" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="418" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A418" s="15" t="s">
         <v>405</v>
       </c>
@@ -49435,7 +49475,7 @@
       <c r="AL422" s="1"/>
       <c r="AM422" s="1"/>
     </row>
-    <row r="423" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="423" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A423" s="15" t="s">
         <v>406</v>
       </c>
@@ -49525,7 +49565,7 @@
       <c r="AL423" s="1"/>
       <c r="AM423" s="1"/>
     </row>
-    <row r="424" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="424" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A424" s="15" t="s">
         <v>409</v>
       </c>
@@ -49609,7 +49649,7 @@
       <c r="AL424" s="1"/>
       <c r="AM424" s="1"/>
     </row>
-    <row r="425" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="425" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A425" s="15" t="s">
         <v>410</v>
       </c>
@@ -49693,7 +49733,7 @@
       <c r="AL425" s="1"/>
       <c r="AM425" s="1"/>
     </row>
-    <row r="426" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="426" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A426" s="15" t="s">
         <v>411</v>
       </c>
@@ -49777,7 +49817,7 @@
       <c r="AL426" s="1"/>
       <c r="AM426" s="1"/>
     </row>
-    <row r="427" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="427" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A427" s="15" t="s">
         <v>412</v>
       </c>
@@ -49955,7 +49995,7 @@
       <c r="AL428" s="1"/>
       <c r="AM428" s="1"/>
     </row>
-    <row r="429" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="429" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A429" s="15" t="s">
         <v>416</v>
       </c>
@@ -50039,7 +50079,7 @@
       <c r="AL429" s="1"/>
       <c r="AM429" s="1"/>
     </row>
-    <row r="430" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="430" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A430" s="15" t="s">
         <v>418</v>
       </c>
@@ -50125,7 +50165,7 @@
       <c r="AL430" s="1"/>
       <c r="AM430" s="1"/>
     </row>
-    <row r="431" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="431" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A431" s="15" t="s">
         <v>421</v>
       </c>
@@ -50215,7 +50255,7 @@
       <c r="AL431" s="1"/>
       <c r="AM431" s="1"/>
     </row>
-    <row r="432" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="432" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A432" s="15" t="s">
         <v>423</v>
       </c>
@@ -50301,7 +50341,7 @@
       <c r="AL432" s="1"/>
       <c r="AM432" s="1"/>
     </row>
-    <row r="433" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="433" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A433" s="15" t="s">
         <v>426</v>
       </c>
@@ -50391,7 +50431,7 @@
       <c r="AL433" s="1"/>
       <c r="AM433" s="1"/>
     </row>
-    <row r="434" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="434" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A434" s="15" t="s">
         <v>428</v>
       </c>
@@ -50481,7 +50521,7 @@
       <c r="AL434" s="1"/>
       <c r="AM434" s="1"/>
     </row>
-    <row r="435" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="435" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A435" s="15" t="s">
         <v>430</v>
       </c>
@@ -50565,7 +50605,7 @@
       <c r="AL435" s="1"/>
       <c r="AM435" s="1"/>
     </row>
-    <row r="436" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="436" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A436" s="15" t="s">
         <v>432</v>
       </c>
@@ -50655,7 +50695,7 @@
       <c r="AL436" s="1"/>
       <c r="AM436" s="1"/>
     </row>
-    <row r="437" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="437" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A437" s="15" t="s">
         <v>435</v>
       </c>
@@ -50741,7 +50781,7 @@
       <c r="AL437" s="1"/>
       <c r="AM437" s="1"/>
     </row>
-    <row r="438" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="438" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A438" s="15" t="s">
         <v>437</v>
       </c>
@@ -50827,7 +50867,7 @@
       <c r="AL438" s="1"/>
       <c r="AM438" s="1"/>
     </row>
-    <row r="439" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="439" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A439" s="15" t="s">
         <v>439</v>
       </c>
@@ -50913,7 +50953,7 @@
       <c r="AL439" s="1"/>
       <c r="AM439" s="1"/>
     </row>
-    <row r="440" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="440" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A440" s="15" t="s">
         <v>441</v>
       </c>
@@ -50999,7 +51039,7 @@
       <c r="AL440" s="1"/>
       <c r="AM440" s="1"/>
     </row>
-    <row r="441" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="441" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A441" s="15" t="s">
         <v>444</v>
       </c>
@@ -51085,7 +51125,7 @@
       <c r="AL441" s="1"/>
       <c r="AM441" s="1"/>
     </row>
-    <row r="442" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="442" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A442" s="15" t="s">
         <v>446</v>
       </c>
@@ -51171,7 +51211,7 @@
       <c r="AL442" s="1"/>
       <c r="AM442" s="1"/>
     </row>
-    <row r="443" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="443" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A443" s="15" t="s">
         <v>448</v>
       </c>
@@ -51257,7 +51297,7 @@
       <c r="AL443" s="1"/>
       <c r="AM443" s="1"/>
     </row>
-    <row r="444" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="444" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A444" s="15" t="s">
         <v>450</v>
       </c>
@@ -51343,7 +51383,7 @@
       <c r="AL444" s="1"/>
       <c r="AM444" s="1"/>
     </row>
-    <row r="445" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="445" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A445" s="15" t="s">
         <v>452</v>
       </c>
@@ -51429,7 +51469,7 @@
       <c r="AL445" s="1"/>
       <c r="AM445" s="1"/>
     </row>
-    <row r="446" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="446" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A446" s="15" t="s">
         <v>454</v>
       </c>
@@ -51519,7 +51559,7 @@
       <c r="AL446" s="1"/>
       <c r="AM446" s="1"/>
     </row>
-    <row r="447" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="447" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A447" s="15" t="s">
         <v>457</v>
       </c>
@@ -51605,7 +51645,7 @@
       <c r="AL447" s="1"/>
       <c r="AM447" s="1"/>
     </row>
-    <row r="448" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="448" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A448" s="15" t="s">
         <v>459</v>
       </c>
@@ -51691,7 +51731,7 @@
       <c r="AL448" s="1"/>
       <c r="AM448" s="1"/>
     </row>
-    <row r="449" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="449" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A449" s="15" t="s">
         <v>461</v>
       </c>
@@ -51777,7 +51817,7 @@
       <c r="AL449" s="1"/>
       <c r="AM449" s="1"/>
     </row>
-    <row r="450" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="450" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A450" s="15" t="s">
         <v>463</v>
       </c>
@@ -51863,7 +51903,7 @@
       <c r="AL450" s="1"/>
       <c r="AM450" s="1"/>
     </row>
-    <row r="451" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="451" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A451" s="15" t="s">
         <v>465</v>
       </c>
@@ -51949,7 +51989,7 @@
       <c r="AL451" s="1"/>
       <c r="AM451" s="1"/>
     </row>
-    <row r="452" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="452" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A452" s="15" t="s">
         <v>467</v>
       </c>
@@ -52035,7 +52075,7 @@
       <c r="AL452" s="1"/>
       <c r="AM452" s="1"/>
     </row>
-    <row r="453" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="453" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A453" s="15" t="s">
         <v>469</v>
       </c>
@@ -52121,7 +52161,7 @@
       <c r="AL453" s="1"/>
       <c r="AM453" s="1"/>
     </row>
-    <row r="454" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="454" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A454" s="15" t="s">
         <v>471</v>
       </c>
@@ -52207,7 +52247,7 @@
       <c r="AL454" s="1"/>
       <c r="AM454" s="1"/>
     </row>
-    <row r="455" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="455" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A455" s="15" t="s">
         <v>473</v>
       </c>
@@ -52293,7 +52333,7 @@
       <c r="AL455" s="1"/>
       <c r="AM455" s="1"/>
     </row>
-    <row r="456" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="456" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A456" s="15" t="s">
         <v>475</v>
       </c>
@@ -52379,7 +52419,7 @@
       <c r="AL456" s="1"/>
       <c r="AM456" s="1"/>
     </row>
-    <row r="457" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="457" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A457" s="15" t="s">
         <v>477</v>
       </c>
@@ -52465,7 +52505,7 @@
       <c r="AL457" s="1"/>
       <c r="AM457" s="1"/>
     </row>
-    <row r="458" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="458" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A458" s="15" t="s">
         <v>479</v>
       </c>
@@ -52551,7 +52591,7 @@
       <c r="AL458" s="1"/>
       <c r="AM458" s="1"/>
     </row>
-    <row r="459" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="459" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A459" s="15" t="s">
         <v>481</v>
       </c>
@@ -52623,7 +52663,7 @@
       <c r="AL459" s="1"/>
       <c r="AM459" s="1"/>
     </row>
-    <row r="460" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="460" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A460" s="15" t="s">
         <v>482</v>
       </c>
@@ -52709,7 +52749,7 @@
       <c r="AL460" s="1"/>
       <c r="AM460" s="1"/>
     </row>
-    <row r="461" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="461" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A461" s="15" t="s">
         <v>485</v>
       </c>
@@ -52793,7 +52833,7 @@
       <c r="AL461" s="1"/>
       <c r="AM461" s="1"/>
     </row>
-    <row r="462" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="462" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A462" s="15" t="s">
         <v>487</v>
       </c>
@@ -52883,7 +52923,7 @@
       <c r="AL462" s="1"/>
       <c r="AM462" s="1"/>
     </row>
-    <row r="463" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="463" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A463" s="15" t="s">
         <v>488</v>
       </c>
@@ -52969,7 +53009,7 @@
       <c r="AL463" s="1"/>
       <c r="AM463" s="1"/>
     </row>
-    <row r="464" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="464" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A464" s="15" t="s">
         <v>492</v>
       </c>
@@ -53061,7 +53101,7 @@
       <c r="AL464" s="1"/>
       <c r="AM464" s="1"/>
     </row>
-    <row r="465" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="465" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A465" s="15" t="s">
         <v>495</v>
       </c>
@@ -53153,7 +53193,7 @@
       <c r="AL465" s="1"/>
       <c r="AM465" s="1"/>
     </row>
-    <row r="466" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="466" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A466" s="15" t="s">
         <v>498</v>
       </c>
@@ -53243,7 +53283,7 @@
       <c r="AL466" s="1"/>
       <c r="AM466" s="1"/>
     </row>
-    <row r="467" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="467" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A467" s="15" t="s">
         <v>500</v>
       </c>
@@ -53329,7 +53369,7 @@
       <c r="AL467" s="1"/>
       <c r="AM467" s="1"/>
     </row>
-    <row r="468" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="468" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A468" s="15" t="s">
         <v>501</v>
       </c>
@@ -53415,7 +53455,7 @@
       <c r="AL468" s="1"/>
       <c r="AM468" s="1"/>
     </row>
-    <row r="469" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="469" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A469" s="15" t="s">
         <v>503</v>
       </c>
@@ -53501,7 +53541,7 @@
       <c r="AL469" s="1"/>
       <c r="AM469" s="1"/>
     </row>
-    <row r="470" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="470" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A470" s="15" t="s">
         <v>506</v>
       </c>
@@ -53587,7 +53627,7 @@
       <c r="AL470" s="1"/>
       <c r="AM470" s="1"/>
     </row>
-    <row r="471" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="471" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A471" s="15" t="s">
         <v>508</v>
       </c>
@@ -53673,7 +53713,7 @@
       <c r="AL471" s="1"/>
       <c r="AM471" s="1"/>
     </row>
-    <row r="472" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="472" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A472" s="15" t="s">
         <v>511</v>
       </c>
@@ -53759,7 +53799,7 @@
       <c r="AL472" s="1"/>
       <c r="AM472" s="1"/>
     </row>
-    <row r="473" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="473" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A473" s="15" t="s">
         <v>514</v>
       </c>
@@ -53843,7 +53883,7 @@
       <c r="AL473" s="1"/>
       <c r="AM473" s="1"/>
     </row>
-    <row r="474" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="474" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A474" s="15" t="s">
         <v>516</v>
       </c>
@@ -53929,7 +53969,7 @@
       <c r="AL474" s="1"/>
       <c r="AM474" s="1"/>
     </row>
-    <row r="475" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="475" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A475" s="15" t="s">
         <v>518</v>
       </c>
@@ -54013,7 +54053,7 @@
       <c r="AL475" s="1"/>
       <c r="AM475" s="1"/>
     </row>
-    <row r="476" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="476" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A476" s="15" t="s">
         <v>520</v>
       </c>
@@ -54099,7 +54139,7 @@
       <c r="AL476" s="1"/>
       <c r="AM476" s="1"/>
     </row>
-    <row r="477" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="477" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A477" s="15" t="s">
         <v>522</v>
       </c>
@@ -54185,7 +54225,7 @@
       <c r="AL477" s="1"/>
       <c r="AM477" s="1"/>
     </row>
-    <row r="478" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="478" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A478" s="15" t="s">
         <v>525</v>
       </c>
@@ -54271,7 +54311,7 @@
       <c r="AL478" s="1"/>
       <c r="AM478" s="1"/>
     </row>
-    <row r="479" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="479" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A479" s="15" t="s">
         <v>528</v>
       </c>
@@ -54357,7 +54397,7 @@
       <c r="AL479" s="1"/>
       <c r="AM479" s="1"/>
     </row>
-    <row r="480" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="480" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A480" s="15" t="s">
         <v>531</v>
       </c>
@@ -54443,7 +54483,7 @@
       <c r="AL480" s="1"/>
       <c r="AM480" s="1"/>
     </row>
-    <row r="481" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="481" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A481" s="15" t="s">
         <v>535</v>
       </c>
@@ -54529,7 +54569,7 @@
       <c r="AL481" s="1"/>
       <c r="AM481" s="1"/>
     </row>
-    <row r="482" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="482" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A482" s="15" t="s">
         <v>537</v>
       </c>
@@ -54615,7 +54655,7 @@
       <c r="AL482" s="1"/>
       <c r="AM482" s="1"/>
     </row>
-    <row r="483" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="483" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A483" s="15" t="s">
         <v>539</v>
       </c>
@@ -54701,7 +54741,7 @@
       <c r="AL483" s="1"/>
       <c r="AM483" s="1"/>
     </row>
-    <row r="484" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="484" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A484" s="15" t="s">
         <v>541</v>
       </c>
@@ -54785,7 +54825,7 @@
       <c r="AL484" s="1"/>
       <c r="AM484" s="1"/>
     </row>
-    <row r="485" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="485" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A485" s="15" t="s">
         <v>543</v>
       </c>
@@ -54871,7 +54911,7 @@
       <c r="AL485" s="1"/>
       <c r="AM485" s="1"/>
     </row>
-    <row r="486" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="486" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A486" s="15" t="s">
         <v>546</v>
       </c>
@@ -54961,7 +55001,7 @@
       <c r="AL486" s="1"/>
       <c r="AM486" s="1"/>
     </row>
-    <row r="487" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="487" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A487" s="15" t="s">
         <v>547</v>
       </c>
@@ -55047,7 +55087,7 @@
       <c r="AL487" s="1"/>
       <c r="AM487" s="1"/>
     </row>
-    <row r="488" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="488" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A488" s="15" t="s">
         <v>548</v>
       </c>
@@ -55133,7 +55173,7 @@
       <c r="AL488" s="1"/>
       <c r="AM488" s="1"/>
     </row>
-    <row r="489" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="489" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A489" s="15" t="s">
         <v>550</v>
       </c>
@@ -55219,7 +55259,7 @@
       <c r="AL489" s="1"/>
       <c r="AM489" s="1"/>
     </row>
-    <row r="490" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="490" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A490" s="15" t="s">
         <v>551</v>
       </c>
@@ -55309,7 +55349,7 @@
       <c r="AL490" s="1"/>
       <c r="AM490" s="1"/>
     </row>
-    <row r="491" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="491" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A491" s="15" t="s">
         <v>552</v>
       </c>
@@ -55395,7 +55435,7 @@
       <c r="AL491" s="1"/>
       <c r="AM491" s="1"/>
     </row>
-    <row r="492" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="492" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A492" s="15" t="s">
         <v>555</v>
       </c>
@@ -55481,7 +55521,7 @@
       <c r="AL492" s="1"/>
       <c r="AM492" s="1"/>
     </row>
-    <row r="493" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="493" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A493" s="15" t="s">
         <v>557</v>
       </c>
@@ -55567,7 +55607,7 @@
       <c r="AL493" s="1"/>
       <c r="AM493" s="1"/>
     </row>
-    <row r="494" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="494" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A494" s="15" t="s">
         <v>559</v>
       </c>
@@ -55653,7 +55693,7 @@
       <c r="AL494" s="1"/>
       <c r="AM494" s="1"/>
     </row>
-    <row r="495" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="495" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A495" s="15" t="s">
         <v>561</v>
       </c>
@@ -55739,7 +55779,7 @@
       <c r="AL495" s="1"/>
       <c r="AM495" s="1"/>
     </row>
-    <row r="496" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="496" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A496" s="15" t="s">
         <v>563</v>
       </c>
@@ -55825,7 +55865,7 @@
       <c r="AL496" s="1"/>
       <c r="AM496" s="1"/>
     </row>
-    <row r="497" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="497" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A497" s="15" t="s">
         <v>565</v>
       </c>
@@ -55911,7 +55951,7 @@
       <c r="AL497" s="1"/>
       <c r="AM497" s="1"/>
     </row>
-    <row r="498" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="498" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A498" s="15" t="s">
         <v>567</v>
       </c>
@@ -55997,7 +56037,7 @@
       <c r="AL498" s="1"/>
       <c r="AM498" s="1"/>
     </row>
-    <row r="499" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="499" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A499" s="15" t="s">
         <v>570</v>
       </c>
@@ -56085,7 +56125,7 @@
       <c r="AL499" s="1"/>
       <c r="AM499" s="1"/>
     </row>
-    <row r="500" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="500" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A500" s="15" t="s">
         <v>573</v>
       </c>
@@ -56169,7 +56209,7 @@
       <c r="AL500" s="1"/>
       <c r="AM500" s="1"/>
     </row>
-    <row r="501" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="501" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A501" s="15" t="s">
         <v>575</v>
       </c>
@@ -56255,7 +56295,7 @@
       <c r="AL501" s="1"/>
       <c r="AM501" s="1"/>
     </row>
-    <row r="502" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="502" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A502" s="15" t="s">
         <v>578</v>
       </c>
@@ -56339,7 +56379,7 @@
       <c r="AL502" s="1"/>
       <c r="AM502" s="1"/>
     </row>
-    <row r="503" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="503" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A503" s="15" t="s">
         <v>580</v>
       </c>
@@ -56423,7 +56463,7 @@
       <c r="AL503" s="1"/>
       <c r="AM503" s="1"/>
     </row>
-    <row r="504" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="504" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A504" s="15" t="s">
         <v>582</v>
       </c>
@@ -56503,7 +56543,7 @@
       <c r="AL504" s="1"/>
       <c r="AM504" s="1"/>
     </row>
-    <row r="505" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="505" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A505" s="15" t="s">
         <v>583</v>
       </c>
@@ -56587,7 +56627,7 @@
       <c r="AL505" s="1"/>
       <c r="AM505" s="1"/>
     </row>
-    <row r="506" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="506" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A506" s="15" t="s">
         <v>586</v>
       </c>
@@ -56671,7 +56711,7 @@
       <c r="AL506" s="1"/>
       <c r="AM506" s="1"/>
     </row>
-    <row r="507" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="507" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A507" s="15" t="s">
         <v>589</v>
       </c>
@@ -56755,7 +56795,7 @@
       <c r="AL507" s="1"/>
       <c r="AM507" s="1"/>
     </row>
-    <row r="508" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="508" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A508" s="15" t="s">
         <v>591</v>
       </c>
@@ -56843,7 +56883,7 @@
       <c r="AL508" s="1"/>
       <c r="AM508" s="1"/>
     </row>
-    <row r="509" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="509" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A509" s="15" t="s">
         <v>593</v>
       </c>
@@ -56925,7 +56965,7 @@
       <c r="AL509" s="1"/>
       <c r="AM509" s="1"/>
     </row>
-    <row r="510" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="510" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A510" s="15" t="s">
         <v>595</v>
       </c>
@@ -57011,7 +57051,7 @@
       <c r="AL510" s="1"/>
       <c r="AM510" s="1"/>
     </row>
-    <row r="511" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="511" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A511" s="15" t="s">
         <v>597</v>
       </c>
@@ -57097,7 +57137,7 @@
       <c r="AL511" s="1"/>
       <c r="AM511" s="1"/>
     </row>
-    <row r="512" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="512" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A512" s="15" t="s">
         <v>600</v>
       </c>
@@ -57181,7 +57221,7 @@
       <c r="AL512" s="1"/>
       <c r="AM512" s="1"/>
     </row>
-    <row r="513" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="513" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A513" s="15" t="s">
         <v>602</v>
       </c>
@@ -57263,7 +57303,7 @@
       <c r="AL513" s="1"/>
       <c r="AM513" s="1"/>
     </row>
-    <row r="514" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="514" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A514" s="15" t="s">
         <v>603</v>
       </c>
@@ -57347,7 +57387,7 @@
       <c r="AL514" s="1"/>
       <c r="AM514" s="1"/>
     </row>
-    <row r="515" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="515" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A515" s="15" t="s">
         <v>605</v>
       </c>
@@ -57431,7 +57471,7 @@
       <c r="AL515" s="1"/>
       <c r="AM515" s="1"/>
     </row>
-    <row r="516" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="516" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A516" s="15" t="s">
         <v>607</v>
       </c>
@@ -57511,7 +57551,7 @@
       <c r="AL516" s="1"/>
       <c r="AM516" s="1"/>
     </row>
-    <row r="517" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="517" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A517" s="15" t="s">
         <v>608</v>
       </c>
@@ -57681,7 +57721,7 @@
       <c r="AL518" s="1"/>
       <c r="AM518" s="1"/>
     </row>
-    <row r="519" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="519" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A519" s="15" t="s">
         <v>611</v>
       </c>
@@ -57767,7 +57807,7 @@
       <c r="AL519" s="1"/>
       <c r="AM519" s="1"/>
     </row>
-    <row r="520" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="520" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A520" s="15" t="s">
         <v>614</v>
       </c>
@@ -57853,7 +57893,7 @@
       <c r="AL520" s="1"/>
       <c r="AM520" s="1"/>
     </row>
-    <row r="521" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="521" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A521" s="15" t="s">
         <v>616</v>
       </c>
@@ -57939,7 +57979,7 @@
       <c r="AL521" s="1"/>
       <c r="AM521" s="1"/>
     </row>
-    <row r="522" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="522" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A522" s="15" t="s">
         <v>619</v>
       </c>
@@ -58029,7 +58069,7 @@
       <c r="AL522" s="1"/>
       <c r="AM522" s="1"/>
     </row>
-    <row r="523" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="523" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A523" s="15" t="s">
         <v>622</v>
       </c>
@@ -58119,7 +58159,7 @@
       <c r="AL523" s="1"/>
       <c r="AM523" s="1"/>
     </row>
-    <row r="524" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="524" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A524" s="15" t="s">
         <v>624</v>
       </c>
@@ -58209,7 +58249,7 @@
       <c r="AL524" s="1"/>
       <c r="AM524" s="1"/>
     </row>
-    <row r="525" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="525" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A525" s="15" t="s">
         <v>626</v>
       </c>
@@ -58295,7 +58335,7 @@
       <c r="AL525" s="1"/>
       <c r="AM525" s="1"/>
     </row>
-    <row r="526" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="526" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A526" s="15" t="s">
         <v>628</v>
       </c>
@@ -58381,7 +58421,7 @@
       <c r="AL526" s="1"/>
       <c r="AM526" s="1"/>
     </row>
-    <row r="527" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="527" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A527" s="15" t="s">
         <v>630</v>
       </c>
@@ -58471,7 +58511,7 @@
       <c r="AL527" s="1"/>
       <c r="AM527" s="1"/>
     </row>
-    <row r="528" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="528" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A528" s="15" t="s">
         <v>632</v>
       </c>
@@ -58557,7 +58597,7 @@
       <c r="AL528" s="1"/>
       <c r="AM528" s="1"/>
     </row>
-    <row r="529" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="529" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A529" s="15" t="s">
         <v>634</v>
       </c>
@@ -58641,7 +58681,7 @@
       <c r="AL529" s="1"/>
       <c r="AM529" s="1"/>
     </row>
-    <row r="530" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="530" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A530" s="15" t="s">
         <v>636</v>
       </c>
@@ -58727,7 +58767,7 @@
       <c r="AL530" s="1"/>
       <c r="AM530" s="1"/>
     </row>
-    <row r="531" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="531" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A531" s="15" t="s">
         <v>638</v>
       </c>
@@ -58813,7 +58853,7 @@
       <c r="AL531" s="1"/>
       <c r="AM531" s="1"/>
     </row>
-    <row r="532" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="532" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A532" s="15" t="s">
         <v>640</v>
       </c>
@@ -58899,7 +58939,7 @@
       <c r="AL532" s="1"/>
       <c r="AM532" s="1"/>
     </row>
-    <row r="533" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="533" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A533" s="15" t="s">
         <v>642</v>
       </c>
@@ -58985,7 +59025,7 @@
       <c r="AL533" s="1"/>
       <c r="AM533" s="1"/>
     </row>
-    <row r="534" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="534" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A534" s="15" t="s">
         <v>644</v>
       </c>
@@ -59071,7 +59111,7 @@
       <c r="AL534" s="1"/>
       <c r="AM534" s="1"/>
     </row>
-    <row r="535" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="535" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A535" s="15" t="s">
         <v>645</v>
       </c>
@@ -59155,7 +59195,7 @@
       <c r="AL535" s="1"/>
       <c r="AM535" s="1"/>
     </row>
-    <row r="536" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="536" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A536" s="15" t="s">
         <v>647</v>
       </c>
@@ -59239,7 +59279,7 @@
       <c r="AL536" s="1"/>
       <c r="AM536" s="1"/>
     </row>
-    <row r="537" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="537" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A537" s="15" t="s">
         <v>649</v>
       </c>
@@ -59323,7 +59363,7 @@
       <c r="AL537" s="1"/>
       <c r="AM537" s="1"/>
     </row>
-    <row r="538" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="538" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A538" s="15" t="s">
         <v>651</v>
       </c>
@@ -59407,7 +59447,7 @@
       <c r="AL538" s="1"/>
       <c r="AM538" s="1"/>
     </row>
-    <row r="539" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="539" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A539" s="15" t="s">
         <v>653</v>
       </c>
@@ -59493,7 +59533,7 @@
       <c r="AL539" s="1"/>
       <c r="AM539" s="1"/>
     </row>
-    <row r="540" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="540" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A540" s="15" t="s">
         <v>655</v>
       </c>
@@ -59579,7 +59619,7 @@
       <c r="AL540" s="1"/>
       <c r="AM540" s="1"/>
     </row>
-    <row r="541" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="541" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A541" s="15" t="s">
         <v>657</v>
       </c>
@@ -59665,7 +59705,7 @@
       <c r="AL541" s="1"/>
       <c r="AM541" s="1"/>
     </row>
-    <row r="542" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="542" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A542" s="15" t="s">
         <v>659</v>
       </c>
@@ -59751,7 +59791,7 @@
       <c r="AL542" s="1"/>
       <c r="AM542" s="1"/>
     </row>
-    <row r="543" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="543" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A543" s="15" t="s">
         <v>661</v>
       </c>
@@ -59837,7 +59877,7 @@
       <c r="AL543" s="1"/>
       <c r="AM543" s="1"/>
     </row>
-    <row r="544" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="544" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A544" s="15" t="s">
         <v>663</v>
       </c>
@@ -59921,7 +59961,7 @@
       <c r="AL544" s="1"/>
       <c r="AM544" s="1"/>
     </row>
-    <row r="545" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="545" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A545" s="15" t="s">
         <v>664</v>
       </c>
@@ -60001,7 +60041,7 @@
       <c r="AL545" s="1"/>
       <c r="AM545" s="1"/>
     </row>
-    <row r="546" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="546" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A546" s="15" t="s">
         <v>665</v>
       </c>
@@ -60081,7 +60121,7 @@
       <c r="AL546" s="1"/>
       <c r="AM546" s="1"/>
     </row>
-    <row r="547" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="547" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A547" s="15" t="s">
         <v>666</v>
       </c>
@@ -60157,7 +60197,7 @@
       <c r="AL547" s="1"/>
       <c r="AM547" s="1"/>
     </row>
-    <row r="548" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="548" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A548" s="15" t="s">
         <v>668</v>
       </c>
@@ -60237,7 +60277,7 @@
       <c r="AL548" s="1"/>
       <c r="AM548" s="1"/>
     </row>
-    <row r="549" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="549" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A549" s="15" t="s">
         <v>669</v>
       </c>
@@ -60317,7 +60357,7 @@
       <c r="AL549" s="1"/>
       <c r="AM549" s="1"/>
     </row>
-    <row r="550" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="550" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A550" s="15" t="s">
         <v>670</v>
       </c>
@@ -60397,7 +60437,7 @@
       <c r="AL550" s="1"/>
       <c r="AM550" s="1"/>
     </row>
-    <row r="551" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="551" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A551" s="15" t="s">
         <v>671</v>
       </c>
@@ -60477,7 +60517,7 @@
       <c r="AL551" s="1"/>
       <c r="AM551" s="1"/>
     </row>
-    <row r="552" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="552" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A552" s="15" t="s">
         <v>672</v>
       </c>
@@ -60557,7 +60597,7 @@
       <c r="AL552" s="1"/>
       <c r="AM552" s="1"/>
     </row>
-    <row r="553" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="553" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A553" s="15" t="s">
         <v>674</v>
       </c>
@@ -60637,7 +60677,7 @@
       <c r="AL553" s="1"/>
       <c r="AM553" s="1"/>
     </row>
-    <row r="554" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="554" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A554" s="15" t="s">
         <v>675</v>
       </c>
@@ -60717,7 +60757,7 @@
       <c r="AL554" s="1"/>
       <c r="AM554" s="1"/>
     </row>
-    <row r="555" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="555" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A555" s="15" t="s">
         <v>676</v>
       </c>
@@ -60797,7 +60837,7 @@
       <c r="AL555" s="1"/>
       <c r="AM555" s="1"/>
     </row>
-    <row r="556" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="556" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A556" s="31" t="s">
         <v>677</v>
       </c>
@@ -60877,7 +60917,7 @@
       <c r="AL556" s="1"/>
       <c r="AM556" s="1"/>
     </row>
-    <row r="557" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="557" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A557" s="15" t="s">
         <v>678</v>
       </c>
@@ -60957,7 +60997,7 @@
       <c r="AL557" s="1"/>
       <c r="AM557" s="1"/>
     </row>
-    <row r="558" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="558" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A558" s="15" t="s">
         <v>679</v>
       </c>
@@ -61037,7 +61077,7 @@
       <c r="AL558" s="1"/>
       <c r="AM558" s="1"/>
     </row>
-    <row r="559" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="559" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A559" s="15" t="s">
         <v>680</v>
       </c>
@@ -61117,7 +61157,7 @@
       <c r="AL559" s="1"/>
       <c r="AM559" s="1"/>
     </row>
-    <row r="560" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="560" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A560" s="15" t="s">
         <v>681</v>
       </c>
@@ -61197,7 +61237,7 @@
       <c r="AL560" s="1"/>
       <c r="AM560" s="1"/>
     </row>
-    <row r="561" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="561" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A561" s="15" t="s">
         <v>682</v>
       </c>
@@ -61277,7 +61317,7 @@
       <c r="AL561" s="1"/>
       <c r="AM561" s="1"/>
     </row>
-    <row r="562" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="562" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A562" s="15" t="s">
         <v>683</v>
       </c>
@@ -72904,12 +72944,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A2:AL707" xr:uid="{2AA437EE-405D-4A43-9EB9-23F1BEB36011}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="6,00"/>
-        <filter val="6,30"/>
-      </filters>
-    </filterColumn>
     <filterColumn colId="17">
       <filters>
         <filter val="Diadema"/>
@@ -73058,15 +73092,15 @@
       </c>
       <c r="D3" s="52">
         <f>SUMIF(Controle!R:R,Formulas!A3,Controle!AH:AH)</f>
-        <v>392.45735950000005</v>
+        <v>430.76987950000006</v>
       </c>
       <c r="E3" s="49">
         <f t="shared" ref="E3:E5" si="0">D3/C3</f>
-        <v>0.24010429823778848</v>
+        <v>0.26354378919303767</v>
       </c>
       <c r="F3" s="66">
         <f>SUMIF(Controle!$R:$R,Formulas!A3,Controle!$AK:$AK)</f>
-        <v>20671.96</v>
+        <v>38173.78</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -73133,15 +73167,15 @@
       </c>
       <c r="D6" s="55">
         <f t="shared" si="1"/>
-        <v>1715.1351630000004</v>
+        <v>1753.4476830000003</v>
       </c>
       <c r="E6" s="56">
         <f>D6/C6</f>
-        <v>0.37680005792085014</v>
+        <v>0.38521698042732067</v>
       </c>
       <c r="F6" s="67">
         <f t="shared" si="1"/>
-        <v>905697.44000000006</v>
+        <v>923199.26000000013</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -73179,7 +73213,7 @@
       </c>
       <c r="E10" s="66">
         <f>SUMIF(Controle!$L:$L,A10,Controle!$AK:$AK)</f>
-        <v>345413.89</v>
+        <v>362915.71</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -73849,7 +73883,7 @@
       </c>
       <c r="E42" s="68">
         <f>SUM(E10:E41)</f>
-        <v>905697.44</v>
+        <v>923199.26</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualização de dados: Controle Resumo - Base BSW (6).xlsx (07/05/2026 17:28)
</commit_message>
<xml_diff>
--- a/data/dados_atuais.xlsx
+++ b/data/dados_atuais.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://delgadiadema.sharepoint.com/sites/GestoEstratgica/Documentos Compartilhados/Controle Master/BSW/Novo controle (Em processo)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="689" documentId="1_{DDE4A242-D13A-46DE-8B65-653B9F6ECEB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8F3BA450-5B28-412E-82C4-E944558592F1}"/>
+  <xr:revisionPtr revIDLastSave="760" documentId="1_{DDE4A242-D13A-46DE-8B65-653B9F6ECEB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC19E163-D936-4F25-812E-A708E260AC2E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3E398004-7492-4AA0-94C2-EA9B761AAA49}"/>
   </bookViews>
@@ -321,7 +321,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6243" uniqueCount="1408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6278" uniqueCount="1421">
   <si>
     <t>Código
 Bobina Mâe</t>
@@ -4677,6 +4677,71 @@
       <t>AGUARDANDO RETORNO DO FORNECEDOR EM RELAÇÃO À MP.</t>
     </r>
   </si>
+  <si>
+    <t>VW00581Z / 582Z</t>
+  </si>
+  <si>
+    <t>GM000390Z / GM000391Z / GM000392Z / GM000393Z / DJ000131Z / DJ000132Z</t>
+  </si>
+  <si>
+    <t>VW000745Z / 746Z</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>GM000378Z / 379Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>/ GM000396Z / 397Z / GM000380Z / 381Z</t>
+    </r>
+  </si>
+  <si>
+    <t>Redução no passo do blank. Aguardando validação da Controladoria.</t>
+  </si>
+  <si>
+    <t>VW000585Z / 586Z</t>
+  </si>
+  <si>
+    <t>VW000506Z / VW000522AA / VW000597Z / VW000815Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> DA000489AA / DA000490AA</t>
+  </si>
+  <si>
+    <t>VW000887AA / VW000888AA</t>
+  </si>
+  <si>
+    <t>DA000475AA / DA000476AA / DA000477AA / DA000478AA / DA000479AA</t>
+  </si>
+  <si>
+    <t>VB000347LA / DA000496Z / DA000498Z / DA000499Z / DA000501Z / DA000500Z / DA000502Z / DA000506Z / DA000530Z / DA000531</t>
+  </si>
+  <si>
+    <t>DJ000049Z / DJ000050Z / DJ000232Z / DJ000233Z</t>
+  </si>
+  <si>
+    <t>DA000213Z</t>
+  </si>
 </sst>
 </file>
 
@@ -4687,7 +4752,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4792,6 +4857,18 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -4889,7 +4966,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5095,6 +5172,18 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -5425,7 +5514,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>0.38521698042732067</c:v>
+                  <c:v>0.39198599504207626</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6343,7 +6432,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>0.26354378919303767</c:v>
+                  <c:v>0.28239417740993544</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7002,7 +7091,7 @@
                   <c:v>885025.4800000001</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>38173.78</c:v>
+                  <c:v>50984.49</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -7297,7 +7386,7 @@
                 <c:formatCode>_("R$"* #,##0.00_);_("R$"* \(#,##0.00\);_("R$"* "-"??_);_(@_)</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>923199.26000000013</c:v>
+                  <c:v>936009.97000000009</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7669,7 +7758,7 @@
                   <c:v>1322.6778035000002</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>430.76987950000006</c:v>
+                  <c:v>461.58137950000003</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -15963,8 +16052,12 @@
         <f>IF(AG29=100%,Y29," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="AI29" s="64"/>
-      <c r="AJ29" s="1"/>
+      <c r="AI29" s="64">
+        <v>2</v>
+      </c>
+      <c r="AJ29" s="1" t="s">
+        <v>1410</v>
+      </c>
       <c r="AK29" s="65">
         <v>0</v>
       </c>
@@ -16416,25 +16509,39 @@
         <f>AVERAGE(U34:X34)</f>
         <v>36.241950000000003</v>
       </c>
-      <c r="Z34" s="10"/>
-      <c r="AA34" s="10"/>
-      <c r="AB34" s="10"/>
-      <c r="AC34" s="10"/>
+      <c r="Z34" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AA34" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AB34" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AC34" s="10" t="s">
+        <v>693</v>
+      </c>
       <c r="AD34" s="10"/>
       <c r="AE34" s="10"/>
-      <c r="AF34" s="10"/>
+      <c r="AF34" s="10" t="s">
+        <v>693</v>
+      </c>
       <c r="AG34" s="38">
         <f>COUNTIF(Z34:AF34,"X")/7</f>
-        <v>0</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="AH34" s="51" t="str">
         <f>IF(AG34=100%,Y34," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="AI34" s="64"/>
-      <c r="AJ34" s="1"/>
+      <c r="AI34" s="64">
+        <v>2</v>
+      </c>
+      <c r="AJ34" s="1" t="s">
+        <v>1408</v>
+      </c>
       <c r="AK34" s="65">
-        <v>0</v>
+        <v>12810.71</v>
       </c>
       <c r="AL34" s="1"/>
       <c r="AM34" s="1" t="s">
@@ -16709,7 +16816,7 @@
       <c r="AL37" s="1"/>
       <c r="AM37" s="1"/>
     </row>
-    <row r="38" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:39" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A38" s="22" t="s">
         <v>89</v>
       </c>
@@ -16776,28 +16883,44 @@
         <f>AVERAGE(U38:X38)</f>
         <v>33.56026</v>
       </c>
-      <c r="Z38" s="10"/>
-      <c r="AA38" s="10"/>
-      <c r="AB38" s="10"/>
-      <c r="AC38" s="10"/>
+      <c r="Z38" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AA38" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AB38" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AC38" s="10" t="s">
+        <v>693</v>
+      </c>
       <c r="AD38" s="10"/>
       <c r="AE38" s="10"/>
-      <c r="AF38" s="10"/>
+      <c r="AF38" s="10" t="s">
+        <v>693</v>
+      </c>
       <c r="AG38" s="38">
         <f>COUNTIF(Z38:AF38,"X")/7</f>
-        <v>0</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="AH38" s="51" t="str">
         <f>IF(AG38=100%,Y38," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="AI38" s="64"/>
-      <c r="AJ38" s="1"/>
+      <c r="AI38" s="64">
+        <v>6</v>
+      </c>
+      <c r="AJ38" s="2" t="s">
+        <v>1411</v>
+      </c>
       <c r="AK38" s="65">
         <v>0</v>
       </c>
       <c r="AL38" s="1"/>
-      <c r="AM38" s="1"/>
+      <c r="AM38" s="1" t="s">
+        <v>1412</v>
+      </c>
     </row>
     <row r="39" spans="1:39" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="19" t="s">
@@ -17063,15 +17186,19 @@
         <f>IF(AG41=100%,Y41," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="AI41" s="64"/>
-      <c r="AJ41" s="1"/>
+      <c r="AI41" s="64">
+        <v>2</v>
+      </c>
+      <c r="AJ41" s="19" t="s">
+        <v>1413</v>
+      </c>
       <c r="AK41" s="65">
         <v>0</v>
       </c>
       <c r="AL41" s="1"/>
       <c r="AM41" s="1"/>
     </row>
-    <row r="42" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:39" s="26" customFormat="1" ht="30.6" x14ac:dyDescent="0.3">
       <c r="A42" s="22" t="s">
         <v>97</v>
       </c>
@@ -17142,30 +17269,44 @@
         <f>AVERAGE(U42:X42)</f>
         <v>31.700772499999999</v>
       </c>
-      <c r="Z42" s="10"/>
-      <c r="AA42" s="10"/>
-      <c r="AB42" s="10"/>
-      <c r="AC42" s="10"/>
+      <c r="Z42" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AA42" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AB42" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AC42" s="10" t="s">
+        <v>693</v>
+      </c>
       <c r="AD42" s="10"/>
       <c r="AE42" s="10"/>
-      <c r="AF42" s="10"/>
+      <c r="AF42" s="10" t="s">
+        <v>693</v>
+      </c>
       <c r="AG42" s="38">
         <f>COUNTIF(Z42:AF42,"X")/7</f>
-        <v>0</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="AH42" s="51" t="str">
         <f>IF(AG42=100%,Y42," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="AI42" s="64"/>
-      <c r="AJ42" s="1"/>
+      <c r="AI42" s="64">
+        <v>6</v>
+      </c>
+      <c r="AJ42" s="77" t="s">
+        <v>1409</v>
+      </c>
       <c r="AK42" s="65">
         <v>0</v>
       </c>
       <c r="AL42" s="1"/>
       <c r="AM42" s="1"/>
     </row>
-    <row r="43" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:39" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A43" s="22" t="s">
         <v>100</v>
       </c>
@@ -17249,8 +17390,12 @@
         <f>IF(AG43=100%,Y43," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="AI43" s="64"/>
-      <c r="AJ43" s="1"/>
+      <c r="AI43" s="64">
+        <v>4</v>
+      </c>
+      <c r="AJ43" s="19" t="s">
+        <v>1414</v>
+      </c>
       <c r="AK43" s="65">
         <v>0</v>
       </c>
@@ -17418,30 +17563,48 @@
         <f>AVERAGE(U45:X45)</f>
         <v>30.811499999999995</v>
       </c>
-      <c r="Z45" s="10"/>
-      <c r="AA45" s="10"/>
-      <c r="AB45" s="10"/>
-      <c r="AC45" s="10"/>
-      <c r="AD45" s="10"/>
-      <c r="AE45" s="10"/>
-      <c r="AF45" s="10"/>
+      <c r="Z45" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AA45" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AB45" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AC45" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AD45" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AE45" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AF45" s="10" t="s">
+        <v>693</v>
+      </c>
       <c r="AG45" s="38">
         <f>COUNTIF(Z45:AF45,"X")/7</f>
-        <v>0</v>
-      </c>
-      <c r="AH45" s="51" t="str">
+        <v>1</v>
+      </c>
+      <c r="AH45" s="51">
         <f>IF(AG45=100%,Y45," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="AI45" s="64"/>
-      <c r="AJ45" s="1"/>
+        <v>30.811499999999995</v>
+      </c>
+      <c r="AI45" s="64">
+        <v>2</v>
+      </c>
+      <c r="AJ45" s="78" t="s">
+        <v>1415</v>
+      </c>
       <c r="AK45" s="65">
         <v>0</v>
       </c>
       <c r="AL45" s="1"/>
       <c r="AM45" s="1"/>
     </row>
-    <row r="46" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:39" s="26" customFormat="1" ht="51" x14ac:dyDescent="0.3">
       <c r="A46" s="22" t="s">
         <v>109</v>
       </c>
@@ -17525,15 +17688,19 @@
         <f>IF(AG46=100%,Y46," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="AI46" s="64"/>
-      <c r="AJ46" s="1"/>
+      <c r="AI46" s="64">
+        <v>10</v>
+      </c>
+      <c r="AJ46" s="79" t="s">
+        <v>1418</v>
+      </c>
       <c r="AK46" s="65">
         <v>0</v>
       </c>
       <c r="AL46" s="1"/>
       <c r="AM46" s="1"/>
     </row>
-    <row r="47" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:39" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A47" s="22" t="s">
         <v>113</v>
       </c>
@@ -17617,8 +17784,12 @@
         <f>IF(AG47=100%,Y47," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="AI47" s="64"/>
-      <c r="AJ47" s="1"/>
+      <c r="AI47" s="64">
+        <v>4</v>
+      </c>
+      <c r="AJ47" s="80" t="s">
+        <v>1419</v>
+      </c>
       <c r="AK47" s="65">
         <v>0</v>
       </c>
@@ -17709,8 +17880,12 @@
         <f>IF(AG48=100%,Y48," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="AI48" s="64"/>
-      <c r="AJ48" s="1"/>
+      <c r="AI48" s="64">
+        <v>1</v>
+      </c>
+      <c r="AJ48" s="80" t="s">
+        <v>1420</v>
+      </c>
       <c r="AK48" s="65">
         <v>0</v>
       </c>
@@ -17979,8 +18154,12 @@
         <f>IF(AG51=100%,Y51," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="AI51" s="64"/>
-      <c r="AJ51" s="1"/>
+      <c r="AI51" s="64">
+        <v>2</v>
+      </c>
+      <c r="AJ51" s="2" t="s">
+        <v>1416</v>
+      </c>
       <c r="AK51" s="65">
         <v>0</v>
       </c>
@@ -18075,7 +18254,7 @@
       <c r="AL52" s="1"/>
       <c r="AM52" s="1"/>
     </row>
-    <row r="53" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:39" s="26" customFormat="1" ht="30.6" x14ac:dyDescent="0.3">
       <c r="A53" s="22" t="s">
         <v>124</v>
       </c>
@@ -18157,8 +18336,12 @@
         <f>IF(AG53=100%,Y53," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="AI53" s="64"/>
-      <c r="AJ53" s="1"/>
+      <c r="AI53" s="64">
+        <v>5</v>
+      </c>
+      <c r="AJ53" s="2" t="s">
+        <v>1417</v>
+      </c>
       <c r="AK53" s="65">
         <v>0</v>
       </c>
@@ -73092,15 +73275,15 @@
       </c>
       <c r="D3" s="52">
         <f>SUMIF(Controle!R:R,Formulas!A3,Controle!AH:AH)</f>
-        <v>430.76987950000006</v>
+        <v>461.58137950000003</v>
       </c>
       <c r="E3" s="49">
         <f t="shared" ref="E3:E5" si="0">D3/C3</f>
-        <v>0.26354378919303767</v>
+        <v>0.28239417740993544</v>
       </c>
       <c r="F3" s="66">
         <f>SUMIF(Controle!$R:$R,Formulas!A3,Controle!$AK:$AK)</f>
-        <v>38173.78</v>
+        <v>50984.49</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -73167,15 +73350,15 @@
       </c>
       <c r="D6" s="55">
         <f t="shared" si="1"/>
-        <v>1753.4476830000003</v>
+        <v>1784.2591830000001</v>
       </c>
       <c r="E6" s="56">
         <f>D6/C6</f>
-        <v>0.38521698042732067</v>
+        <v>0.39198599504207626</v>
       </c>
       <c r="F6" s="67">
         <f t="shared" si="1"/>
-        <v>923199.26000000013</v>
+        <v>936009.97000000009</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -73318,7 +73501,7 @@
       </c>
       <c r="E15" s="66">
         <f>SUMIF(Controle!$L:$L,A15,Controle!$AK:$AK)</f>
-        <v>0</v>
+        <v>12810.71</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -73883,7 +74066,7 @@
       </c>
       <c r="E42" s="68">
         <f>SUM(E10:E41)</f>
-        <v>923199.26</v>
+        <v>936009.97</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualização de dados: Controle Resumo - Base BSW (7).xlsx (07/05/2026 19:07)
</commit_message>
<xml_diff>
--- a/data/dados_atuais.xlsx
+++ b/data/dados_atuais.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://delgadiadema.sharepoint.com/sites/GestoEstratgica/Documentos Compartilhados/Controle Master/BSW/Novo controle (Em processo)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="760" documentId="1_{DDE4A242-D13A-46DE-8B65-653B9F6ECEB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC19E163-D936-4F25-812E-A708E260AC2E}"/>
+  <xr:revisionPtr revIDLastSave="835" documentId="1_{DDE4A242-D13A-46DE-8B65-653B9F6ECEB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DEAF20B0-9399-4F8A-8409-22F9172E6583}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3E398004-7492-4AA0-94C2-EA9B761AAA49}"/>
   </bookViews>
   <sheets>
     <sheet name="Controle" sheetId="1" r:id="rId1"/>
-    <sheet name="Formulas" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="Planilha1" sheetId="3" r:id="rId2"/>
+    <sheet name="Formulas" sheetId="2" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Controle!$A$2:$AL$707</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Formulas!$A$9:$D$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Formulas!$A$9:$D$41</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -321,7 +322,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6278" uniqueCount="1421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6327" uniqueCount="1427">
   <si>
     <t>Código
 Bobina Mâe</t>
@@ -4741,6 +4742,59 @@
   </si>
   <si>
     <t>DA000213Z</t>
+  </si>
+  <si>
+    <t>MB003601Z</t>
+  </si>
+  <si>
+    <t>GM000408Z / GM000409Z</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>VB000346LA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> / DA000480Z / </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="8"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>MB003597LA / MB003598LA / MB003594LA / MB003595LA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> / MB003607LA / MB003608LA / MB002301LA / MB003563Z / MB003564Z / MB003540Z / MB003541Z</t>
+    </r>
+  </si>
+  <si>
+    <t>DA000491AA / DA000492AA</t>
+  </si>
+  <si>
+    <t>MB002289Z / MB002290Z</t>
+  </si>
+  <si>
+    <t>MB002446LA / MB003670LA / MB003671LA</t>
   </si>
 </sst>
 </file>
@@ -4966,7 +5020,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5183,6 +5237,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="15" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5514,7 +5583,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>0.39198599504207626</c:v>
+                  <c:v>0.41414588085673165</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6432,7 +6501,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>0.28239417740993544</c:v>
+                  <c:v>0.34410514632080136</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7758,7 +7827,7 @@
                   <c:v>1322.6778035000002</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>461.58137950000003</c:v>
+                  <c:v>562.44972749999999</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -18687,23 +18756,41 @@
         <f>AVERAGE(U57:X57)</f>
         <v>25.433042499999999</v>
       </c>
-      <c r="Z57" s="10"/>
-      <c r="AA57" s="10"/>
-      <c r="AB57" s="10"/>
-      <c r="AC57" s="10"/>
-      <c r="AD57" s="10"/>
-      <c r="AE57" s="10"/>
-      <c r="AF57" s="10"/>
+      <c r="Z57" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AA57" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AB57" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AC57" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AD57" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AE57" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AF57" s="10" t="s">
+        <v>693</v>
+      </c>
       <c r="AG57" s="38">
         <f>COUNTIF(Z57:AF57,"X")/7</f>
-        <v>0</v>
-      </c>
-      <c r="AH57" s="51" t="str">
+        <v>1</v>
+      </c>
+      <c r="AH57" s="51">
         <f>IF(AG57=100%,Y57," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="AI57" s="64"/>
-      <c r="AJ57" s="1"/>
+        <v>25.433042499999999</v>
+      </c>
+      <c r="AI57" s="64">
+        <v>1</v>
+      </c>
+      <c r="AJ57" s="81" t="s">
+        <v>1421</v>
+      </c>
       <c r="AK57" s="65">
         <v>0</v>
       </c>
@@ -19863,23 +19950,41 @@
         <f>AVERAGE(U70:X70)</f>
         <v>21.069427500000003</v>
       </c>
-      <c r="Z70" s="10"/>
-      <c r="AA70" s="10"/>
-      <c r="AB70" s="10"/>
-      <c r="AC70" s="10"/>
-      <c r="AD70" s="10"/>
-      <c r="AE70" s="10"/>
-      <c r="AF70" s="10"/>
+      <c r="Z70" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AA70" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AB70" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AC70" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AD70" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AE70" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AF70" s="10" t="s">
+        <v>693</v>
+      </c>
       <c r="AG70" s="38">
         <f>COUNTIF(Z70:AF70,"X")/7</f>
-        <v>0</v>
-      </c>
-      <c r="AH70" s="51" t="str">
+        <v>1</v>
+      </c>
+      <c r="AH70" s="51">
         <f>IF(AG70=100%,Y70," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="AI70" s="64"/>
-      <c r="AJ70" s="1"/>
+        <v>21.069427500000003</v>
+      </c>
+      <c r="AI70" s="64">
+        <v>2</v>
+      </c>
+      <c r="AJ70" s="82" t="s">
+        <v>1422</v>
+      </c>
       <c r="AK70" s="65">
         <v>0</v>
       </c>
@@ -19955,7 +20060,9 @@
         <f>AVERAGE(U71:X71)</f>
         <v>21.0627</v>
       </c>
-      <c r="Z71" s="10"/>
+      <c r="Z71" s="10" t="s">
+        <v>693</v>
+      </c>
       <c r="AA71" s="10"/>
       <c r="AB71" s="10"/>
       <c r="AC71" s="10"/>
@@ -19964,7 +20071,7 @@
       <c r="AF71" s="10"/>
       <c r="AG71" s="38">
         <f>COUNTIF(Z71:AF71,"X")/7</f>
-        <v>0</v>
+        <v>0.14285714285714285</v>
       </c>
       <c r="AH71" s="51" t="str">
         <f>IF(AG71=100%,Y71," ")</f>
@@ -20403,20 +20510,34 @@
         <f>AVERAGE(U76:X76)</f>
         <v>18.897327999999998</v>
       </c>
-      <c r="Z76" s="10"/>
-      <c r="AA76" s="10"/>
-      <c r="AB76" s="10"/>
-      <c r="AC76" s="10"/>
-      <c r="AD76" s="10"/>
-      <c r="AE76" s="10"/>
-      <c r="AF76" s="10"/>
+      <c r="Z76" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AA76" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AB76" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AC76" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AD76" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AE76" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AF76" s="10" t="s">
+        <v>693</v>
+      </c>
       <c r="AG76" s="38">
         <f>COUNTIF(Z76:AF76,"X")/7</f>
-        <v>0</v>
-      </c>
-      <c r="AH76" s="51" t="str">
+        <v>1</v>
+      </c>
+      <c r="AH76" s="51">
         <f>IF(AG76=100%,Y76," ")</f>
-        <v xml:space="preserve"> </v>
+        <v>18.897327999999998</v>
       </c>
       <c r="AI76" s="64"/>
       <c r="AJ76" s="1"/>
@@ -21782,7 +21903,7 @@
       <c r="AL91" s="1"/>
       <c r="AM91" s="1"/>
     </row>
-    <row r="92" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:39" s="26" customFormat="1" ht="71.400000000000006" x14ac:dyDescent="0.3">
       <c r="A92" s="22" t="s">
         <v>174</v>
       </c>
@@ -21855,23 +21976,41 @@
         <f>AVERAGE(U92:X92)</f>
         <v>14.416340000000002</v>
       </c>
-      <c r="Z92" s="10"/>
-      <c r="AA92" s="10"/>
-      <c r="AB92" s="10"/>
-      <c r="AC92" s="10"/>
-      <c r="AD92" s="10"/>
-      <c r="AE92" s="10"/>
-      <c r="AF92" s="10"/>
+      <c r="Z92" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AA92" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AB92" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AC92" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AD92" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AE92" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AF92" s="10" t="s">
+        <v>693</v>
+      </c>
       <c r="AG92" s="38">
         <f>COUNTIF(Z92:AF92,"X")/7</f>
-        <v>0</v>
-      </c>
-      <c r="AH92" s="51" t="str">
+        <v>1</v>
+      </c>
+      <c r="AH92" s="51">
         <f>IF(AG92=100%,Y92," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="AI92" s="64"/>
-      <c r="AJ92" s="1"/>
+        <v>14.416340000000002</v>
+      </c>
+      <c r="AI92" s="64">
+        <v>13</v>
+      </c>
+      <c r="AJ92" s="83" t="s">
+        <v>1423</v>
+      </c>
       <c r="AK92" s="65">
         <v>0</v>
       </c>
@@ -22039,23 +22178,41 @@
         <f>AVERAGE(U94:X94)</f>
         <v>14.171620000000001</v>
       </c>
-      <c r="Z94" s="10"/>
-      <c r="AA94" s="10"/>
-      <c r="AB94" s="10"/>
-      <c r="AC94" s="10"/>
-      <c r="AD94" s="10"/>
-      <c r="AE94" s="10"/>
-      <c r="AF94" s="10"/>
+      <c r="Z94" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AA94" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AB94" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AC94" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AD94" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AE94" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AF94" s="10" t="s">
+        <v>693</v>
+      </c>
       <c r="AG94" s="38">
         <f>COUNTIF(Z94:AF94,"X")/7</f>
-        <v>0</v>
-      </c>
-      <c r="AH94" s="51" t="str">
+        <v>1</v>
+      </c>
+      <c r="AH94" s="51">
         <f>IF(AG94=100%,Y94," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="AI94" s="64"/>
-      <c r="AJ94" s="1"/>
+        <v>14.171620000000001</v>
+      </c>
+      <c r="AI94" s="64">
+        <v>2</v>
+      </c>
+      <c r="AJ94" s="82" t="s">
+        <v>1424</v>
+      </c>
       <c r="AK94" s="65">
         <v>0</v>
       </c>
@@ -25337,23 +25494,39 @@
         <f>AVERAGE(U131:X131)</f>
         <v>6.8805899999999998</v>
       </c>
-      <c r="Z131" s="10"/>
-      <c r="AA131" s="10"/>
-      <c r="AB131" s="10"/>
-      <c r="AC131" s="10"/>
-      <c r="AD131" s="10"/>
-      <c r="AE131" s="10"/>
-      <c r="AF131" s="10"/>
+      <c r="Z131" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AA131" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AB131" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AC131" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AD131" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AE131" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="AF131" s="10" t="s">
+        <v>693</v>
+      </c>
       <c r="AG131" s="38">
         <f>COUNTIF(Z131:AF131,"X")/7</f>
-        <v>0</v>
-      </c>
-      <c r="AH131" s="51" t="str">
+        <v>1</v>
+      </c>
+      <c r="AH131" s="51">
         <f>IF(AG131=100%,Y131," ")</f>
-        <v xml:space="preserve"> </v>
+        <v>6.8805899999999998</v>
       </c>
       <c r="AI131" s="64"/>
-      <c r="AJ131" s="1"/>
+      <c r="AJ131" s="81" t="s">
+        <v>1425</v>
+      </c>
       <c r="AK131" s="65">
         <v>0</v>
       </c>
@@ -26420,7 +26593,7 @@
       <c r="AL143" s="1"/>
       <c r="AM143" s="1"/>
     </row>
-    <row r="144" spans="1:39" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:39" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A144" s="22" t="s">
         <v>228</v>
       </c>
@@ -26505,7 +26678,9 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="AI144" s="64"/>
-      <c r="AJ144" s="1"/>
+      <c r="AJ144" s="82" t="s">
+        <v>1426</v>
+      </c>
       <c r="AK144" s="65">
         <v>0</v>
       </c>
@@ -26591,7 +26766,7 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="AI145" s="64"/>
-      <c r="AJ145" s="1"/>
+      <c r="AJ145" s="84"/>
       <c r="AK145" s="65">
         <v>0</v>
       </c>
@@ -26683,7 +26858,7 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="AI146" s="64"/>
-      <c r="AJ146" s="1"/>
+      <c r="AJ146" s="85"/>
       <c r="AK146" s="65">
         <v>0</v>
       </c>
@@ -26775,7 +26950,7 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="AI147" s="64"/>
-      <c r="AJ147" s="1"/>
+      <c r="AJ147" s="81"/>
       <c r="AK147" s="65">
         <v>0</v>
       </c>
@@ -73203,6 +73378,21 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{179A2EE8-1335-4D6B-B158-248E4A1AFF5C}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D813743-8135-4F32-BACA-A0CD44F9427F}">
   <dimension ref="A1:F44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -73275,11 +73465,11 @@
       </c>
       <c r="D3" s="52">
         <f>SUMIF(Controle!R:R,Formulas!A3,Controle!AH:AH)</f>
-        <v>461.58137950000003</v>
+        <v>562.44972749999999</v>
       </c>
       <c r="E3" s="49">
         <f t="shared" ref="E3:E5" si="0">D3/C3</f>
-        <v>0.28239417740993544</v>
+        <v>0.34410514632080136</v>
       </c>
       <c r="F3" s="66">
         <f>SUMIF(Controle!$R:$R,Formulas!A3,Controle!$AK:$AK)</f>
@@ -73350,11 +73540,11 @@
       </c>
       <c r="D6" s="55">
         <f t="shared" si="1"/>
-        <v>1784.2591830000001</v>
+        <v>1885.1275310000001</v>
       </c>
       <c r="E6" s="56">
         <f>D6/C6</f>
-        <v>0.39198599504207626</v>
+        <v>0.41414588085673165</v>
       </c>
       <c r="F6" s="67">
         <f t="shared" si="1"/>

</xml_diff>

<commit_message>
Atualização de dados: Controle Resumo - Base BSW (26).xlsx (15/05/2026 14:57)
</commit_message>
<xml_diff>
--- a/data/dados_atuais.xlsx
+++ b/data/dados_atuais.xlsx
@@ -5,20 +5,21 @@
   <workbookPr codeName="EsteLivro"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gabriel.souza.DELGADIADEMA\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://delgadiadema.sharepoint.com/sites/GestoEstratgica/Documentos Compartilhados/Controle Master/BSW/Novo controle (Em processo)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5759F119-FAB5-4931-8352-76DE5B42E428}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2078" documentId="1_{DDE4A242-D13A-46DE-8B65-653B9F6ECEB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C9D8836-533B-48DD-A7BC-4E47E2A31386}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3E398004-7492-4AA0-94C2-EA9B761AAA49}"/>
+    <workbookView minimized="1" xWindow="3696" yWindow="3696" windowWidth="17280" windowHeight="8880" xr2:uid="{3E398004-7492-4AA0-94C2-EA9B761AAA49}"/>
   </bookViews>
   <sheets>
     <sheet name="Controle" sheetId="1" r:id="rId1"/>
     <sheet name="Formulas" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Controle!$A$2:$AN$710</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Controle!$A$2:$AN$711</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Formulas!$A$9:$D$41</definedName>
+    <definedName name="_FiltrarBaseDados" localSheetId="0" hidden="1">Controle!$A$2:$AL$710</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -212,16 +213,16 @@
     </comment>
     <comment ref="A555" authorId="3" shapeId="0" xr:uid="{33C328EB-7B56-47E9-A787-F392CA006902}">
       <text>
-        <t>[Comentário por tópicos]
-A sua versão do Excel permite-lhe ler este comentário por tópicos. No entanto, as edições feitas ao comentário serão removidas se o ficheiro for aberto numa versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
+        <t>[Comentário encadeado]
+Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
 Comentário:
     Utilizando material 1,60x417</t>
       </text>
     </comment>
     <comment ref="A564" authorId="4" shapeId="0" xr:uid="{C01DA7E7-015C-4D77-8E50-06C386F35AF3}">
       <text>
-        <t>[Comentário por tópicos]
-A sua versão do Excel permite-lhe ler este comentário por tópicos. No entanto, as edições feitas ao comentário serão removidas se o ficheiro for aberto numa versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
+        <t>[Comentário encadeado]
+Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
 Comentário:
     Temos na Fitametal 
 BOZ0070TJ1350 - 10249kg</t>
@@ -253,16 +254,16 @@
     </comment>
     <comment ref="A574" authorId="6" shapeId="0" xr:uid="{67F1D739-35C9-474A-BA1D-BDA6C83EF4A4}">
       <text>
-        <t>[Comentário por tópicos]
-A sua versão do Excel permite-lhe ler este comentário por tópicos. No entanto, as edições feitas ao comentário serão removidas se o ficheiro for aberto numa versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
+        <t>[Comentário encadeado]
+Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
 Comentário:
     CORTAR SLEETER DE MATERIAL SEMELHANTE DEVIDO AO BAIXO VOLUME TEMOS O MESMO MATERIAL COM OUTRAS LARGURAS</t>
       </text>
     </comment>
     <comment ref="A575" authorId="7" shapeId="0" xr:uid="{9641E501-4748-445C-B1A5-D0E296582A82}">
       <text>
-        <t>[Comentário por tópicos]
-A sua versão do Excel permite-lhe ler este comentário por tópicos. No entanto, as edições feitas ao comentário serão removidas se o ficheiro for aberto numa versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
+        <t>[Comentário encadeado]
+Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
 Comentário:
     Usar material BOZ0060HU1000 como material alternativo</t>
       </text>
@@ -5532,7 +5533,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 10 2" xfId="3" xr:uid="{1B383F52-B05A-44D9-B6C7-8BD991E51E85}"/>
     <cellStyle name="Normal 4" xfId="2" xr:uid="{F191687B-6134-4FCE-8079-A034ADDB0F30}"/>
-    <cellStyle name="Percentagem" xfId="4" builtinId="5"/>
+    <cellStyle name="Porcentagem" xfId="4" builtinId="5"/>
     <cellStyle name="Vírgula" xfId="1" builtinId="3"/>
   </cellStyles>
   <dxfs count="5">
@@ -5603,7 +5604,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="pt-PT"/>
+  <c:lang val="pt-BR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -5968,7 +5969,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="pt-PT"/>
+  <c:lang val="pt-BR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -6274,7 +6275,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="pt-PT"/>
+  <c:lang val="pt-BR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -6580,7 +6581,7 @@
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="pt-PT"/>
+  <c:lang val="pt-BR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -6886,7 +6887,7 @@
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="pt-PT"/>
+  <c:lang val="pt-BR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -7192,7 +7193,7 @@
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="pt-PT"/>
+  <c:lang val="pt-BR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -7547,7 +7548,7 @@
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="pt-PT"/>
+  <c:lang val="pt-BR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -7840,7 +7841,7 @@
 <file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="pt-PT"/>
+  <c:lang val="pt-BR"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -13574,7 +13575,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:40" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:40" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
         <v>40</v>
       </c>
@@ -13689,7 +13690,7 @@
       </c>
       <c r="AN3" s="83"/>
     </row>
-    <row r="4" spans="1:40" s="26" customFormat="1" ht="132.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:40" s="26" customFormat="1" ht="132.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
         <v>53</v>
       </c>
@@ -13806,7 +13807,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="5" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
         <v>63</v>
       </c>
@@ -13923,7 +13924,7 @@
         <v>46143</v>
       </c>
     </row>
-    <row r="6" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
         <v>70</v>
       </c>
@@ -14032,7 +14033,7 @@
       </c>
       <c r="AN6" s="83"/>
     </row>
-    <row r="7" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
         <v>78</v>
       </c>
@@ -14147,7 +14148,7 @@
       </c>
       <c r="AN7" s="83"/>
     </row>
-    <row r="8" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
         <v>85</v>
       </c>
@@ -14244,7 +14245,7 @@
       <c r="AM8" s="1"/>
       <c r="AN8" s="83"/>
     </row>
-    <row r="9" spans="1:40" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:40" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
         <v>90</v>
       </c>
@@ -14361,7 +14362,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="10" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>97</v>
       </c>
@@ -14478,7 +14479,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="11" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
         <v>103</v>
       </c>
@@ -14591,7 +14592,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="12" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
         <v>108</v>
       </c>
@@ -14688,7 +14689,7 @@
       <c r="AM12" s="1"/>
       <c r="AN12" s="83"/>
     </row>
-    <row r="13" spans="1:40" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:40" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
         <v>111</v>
       </c>
@@ -14787,7 +14788,7 @@
       <c r="AM13" s="1"/>
       <c r="AN13" s="83"/>
     </row>
-    <row r="14" spans="1:40" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:40" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
         <v>115</v>
       </c>
@@ -14892,7 +14893,7 @@
       <c r="AM14" s="1"/>
       <c r="AN14" s="83"/>
     </row>
-    <row r="15" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
         <v>118</v>
       </c>
@@ -14985,7 +14986,7 @@
       <c r="AM15" s="1"/>
       <c r="AN15" s="83"/>
     </row>
-    <row r="16" spans="1:40" s="26" customFormat="1" ht="30.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:40" s="26" customFormat="1" ht="30.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
         <v>122</v>
       </c>
@@ -15102,7 +15103,7 @@
         <v>46235</v>
       </c>
     </row>
-    <row r="17" spans="1:40" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:40" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
         <v>127</v>
       </c>
@@ -15199,7 +15200,7 @@
       <c r="AM17" s="1"/>
       <c r="AN17" s="83"/>
     </row>
-    <row r="18" spans="1:40" s="26" customFormat="1" ht="51" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:40" s="26" customFormat="1" ht="51" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
         <v>132</v>
       </c>
@@ -15296,7 +15297,7 @@
       <c r="AM18" s="1"/>
       <c r="AN18" s="83"/>
     </row>
-    <row r="19" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
         <v>137</v>
       </c>
@@ -15395,7 +15396,7 @@
       </c>
       <c r="AN19" s="83"/>
     </row>
-    <row r="20" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
         <v>142</v>
       </c>
@@ -15492,7 +15493,7 @@
       <c r="AM20" s="1"/>
       <c r="AN20" s="83"/>
     </row>
-    <row r="21" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
         <v>147</v>
       </c>
@@ -15607,7 +15608,7 @@
         <v>46143</v>
       </c>
     </row>
-    <row r="22" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
         <v>154</v>
       </c>
@@ -15700,7 +15701,7 @@
       <c r="AM22" s="1"/>
       <c r="AN22" s="83"/>
     </row>
-    <row r="23" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
         <v>156</v>
       </c>
@@ -15815,7 +15816,7 @@
         <v>46143</v>
       </c>
     </row>
-    <row r="24" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="22" t="s">
         <v>160</v>
       </c>
@@ -15908,7 +15909,7 @@
       <c r="AM24" s="1"/>
       <c r="AN24" s="83"/>
     </row>
-    <row r="25" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="22" t="s">
         <v>161</v>
       </c>
@@ -16001,7 +16002,7 @@
       <c r="AM25" s="1"/>
       <c r="AN25" s="83"/>
     </row>
-    <row r="26" spans="1:40" s="26" customFormat="1" ht="30.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:40" s="26" customFormat="1" ht="30.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="22" t="s">
         <v>163</v>
       </c>
@@ -16096,7 +16097,7 @@
       <c r="AM26" s="1"/>
       <c r="AN26" s="83"/>
     </row>
-    <row r="27" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="22" t="s">
         <v>166</v>
       </c>
@@ -16189,7 +16190,7 @@
       <c r="AM27" s="1"/>
       <c r="AN27" s="83"/>
     </row>
-    <row r="28" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="22" t="s">
         <v>169</v>
       </c>
@@ -16284,7 +16285,7 @@
       <c r="AM28" s="62"/>
       <c r="AN28" s="83"/>
     </row>
-    <row r="29" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="22" t="s">
         <v>172</v>
       </c>
@@ -16379,7 +16380,7 @@
       <c r="AM29" s="1"/>
       <c r="AN29" s="83"/>
     </row>
-    <row r="30" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="22" t="s">
         <v>175</v>
       </c>
@@ -16472,7 +16473,7 @@
       <c r="AM30" s="1"/>
       <c r="AN30" s="83"/>
     </row>
-    <row r="31" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="22" t="s">
         <v>179</v>
       </c>
@@ -16559,7 +16560,7 @@
       <c r="AM31" s="1"/>
       <c r="AN31" s="83"/>
     </row>
-    <row r="32" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="22" t="s">
         <v>181</v>
       </c>
@@ -16676,7 +16677,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="33" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="22" t="s">
         <v>184</v>
       </c>
@@ -16791,7 +16792,7 @@
         <v>46143</v>
       </c>
     </row>
-    <row r="34" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="22" t="s">
         <v>190</v>
       </c>
@@ -16884,7 +16885,7 @@
       <c r="AM34" s="1"/>
       <c r="AN34" s="83"/>
     </row>
-    <row r="35" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="22" t="s">
         <v>194</v>
       </c>
@@ -17001,7 +17002,7 @@
         <v>46235</v>
       </c>
     </row>
-    <row r="36" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="22" t="s">
         <v>200</v>
       </c>
@@ -17096,7 +17097,7 @@
       <c r="AM36" s="1"/>
       <c r="AN36" s="83"/>
     </row>
-    <row r="37" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="22" t="s">
         <v>201</v>
       </c>
@@ -17183,7 +17184,7 @@
       <c r="AM37" s="1"/>
       <c r="AN37" s="83"/>
     </row>
-    <row r="38" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="22" t="s">
         <v>204</v>
       </c>
@@ -17284,7 +17285,7 @@
       <c r="AM38" s="1"/>
       <c r="AN38" s="83"/>
     </row>
-    <row r="39" spans="1:40" s="26" customFormat="1" ht="71.400000000000006" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:40" s="26" customFormat="1" ht="71.400000000000006" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="22" t="s">
         <v>207</v>
       </c>
@@ -17403,7 +17404,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="40" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="22" t="s">
         <v>211</v>
       </c>
@@ -17496,7 +17497,7 @@
       <c r="AM40" s="1"/>
       <c r="AN40" s="83"/>
     </row>
-    <row r="41" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="22" t="s">
         <v>214</v>
       </c>
@@ -17589,7 +17590,7 @@
       <c r="AM41" s="1"/>
       <c r="AN41" s="83"/>
     </row>
-    <row r="42" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="22" t="s">
         <v>217</v>
       </c>
@@ -17682,7 +17683,7 @@
       <c r="AM42" s="1"/>
       <c r="AN42" s="83"/>
     </row>
-    <row r="43" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="22" t="s">
         <v>221</v>
       </c>
@@ -17775,7 +17776,7 @@
       <c r="AM43" s="1"/>
       <c r="AN43" s="83"/>
     </row>
-    <row r="44" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="22" t="s">
         <v>225</v>
       </c>
@@ -17892,7 +17893,7 @@
         <v>46143</v>
       </c>
     </row>
-    <row r="45" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="22" t="s">
         <v>230</v>
       </c>
@@ -18005,7 +18006,7 @@
         <v>46143</v>
       </c>
     </row>
-    <row r="46" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="22" t="s">
         <v>234</v>
       </c>
@@ -18098,7 +18099,7 @@
       <c r="AM46" s="1"/>
       <c r="AN46" s="83"/>
     </row>
-    <row r="47" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="22" t="s">
         <v>241</v>
       </c>
@@ -18191,7 +18192,7 @@
       <c r="AM47" s="1"/>
       <c r="AN47" s="83"/>
     </row>
-    <row r="48" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="22" t="s">
         <v>244</v>
       </c>
@@ -18284,7 +18285,7 @@
       <c r="AM48" s="1"/>
       <c r="AN48" s="83"/>
     </row>
-    <row r="49" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="22" t="s">
         <v>246</v>
       </c>
@@ -18377,7 +18378,7 @@
       <c r="AM49" s="1"/>
       <c r="AN49" s="83"/>
     </row>
-    <row r="50" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="22" t="s">
         <v>248</v>
       </c>
@@ -18470,7 +18471,7 @@
       <c r="AM50" s="1"/>
       <c r="AN50" s="83"/>
     </row>
-    <row r="51" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="22" t="s">
         <v>251</v>
       </c>
@@ -18563,7 +18564,7 @@
       <c r="AM51" s="1"/>
       <c r="AN51" s="83"/>
     </row>
-    <row r="52" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="22" t="s">
         <v>254</v>
       </c>
@@ -18656,7 +18657,7 @@
       <c r="AM52" s="1"/>
       <c r="AN52" s="83"/>
     </row>
-    <row r="53" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="22" t="s">
         <v>257</v>
       </c>
@@ -18749,7 +18750,7 @@
       <c r="AM53" s="1"/>
       <c r="AN53" s="83"/>
     </row>
-    <row r="54" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="22" t="s">
         <v>259</v>
       </c>
@@ -18842,7 +18843,7 @@
       <c r="AM54" s="1"/>
       <c r="AN54" s="83"/>
     </row>
-    <row r="55" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="22" t="s">
         <v>263</v>
       </c>
@@ -18935,7 +18936,7 @@
       <c r="AM55" s="1"/>
       <c r="AN55" s="83"/>
     </row>
-    <row r="56" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="22" t="s">
         <v>266</v>
       </c>
@@ -19052,7 +19053,7 @@
         <v>46143</v>
       </c>
     </row>
-    <row r="57" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="22" t="s">
         <v>270</v>
       </c>
@@ -19145,7 +19146,7 @@
       <c r="AM57" s="1"/>
       <c r="AN57" s="83"/>
     </row>
-    <row r="58" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="22" t="s">
         <v>271</v>
       </c>
@@ -19238,7 +19239,7 @@
       <c r="AM58" s="1"/>
       <c r="AN58" s="83"/>
     </row>
-    <row r="59" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="22" t="s">
         <v>273</v>
       </c>
@@ -19331,7 +19332,7 @@
       <c r="AM59" s="1"/>
       <c r="AN59" s="83"/>
     </row>
-    <row r="60" spans="1:40" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:40" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="22" t="s">
         <v>275</v>
       </c>
@@ -19442,7 +19443,7 @@
       </c>
       <c r="AN60" s="83"/>
     </row>
-    <row r="61" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="22" t="s">
         <v>281</v>
       </c>
@@ -19555,7 +19556,7 @@
         <v>46054</v>
       </c>
     </row>
-    <row r="62" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="22" t="s">
         <v>287</v>
       </c>
@@ -19648,7 +19649,7 @@
       <c r="AM62" s="1"/>
       <c r="AN62" s="83"/>
     </row>
-    <row r="63" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="22" t="s">
         <v>289</v>
       </c>
@@ -19741,7 +19742,7 @@
       <c r="AM63" s="1"/>
       <c r="AN63" s="83"/>
     </row>
-    <row r="64" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="22" t="s">
         <v>292</v>
       </c>
@@ -19834,7 +19835,7 @@
       <c r="AM64" s="1"/>
       <c r="AN64" s="83"/>
     </row>
-    <row r="65" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" s="22" t="s">
         <v>294</v>
       </c>
@@ -19929,7 +19930,7 @@
       <c r="AM65" s="1"/>
       <c r="AN65" s="83"/>
     </row>
-    <row r="66" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="22" t="s">
         <v>296</v>
       </c>
@@ -20024,7 +20025,7 @@
       <c r="AM66" s="1"/>
       <c r="AN66" s="83"/>
     </row>
-    <row r="67" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="22" t="s">
         <v>298</v>
       </c>
@@ -20113,7 +20114,7 @@
       <c r="AM67" s="1"/>
       <c r="AN67" s="83"/>
     </row>
-    <row r="68" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="22" t="s">
         <v>299</v>
       </c>
@@ -20206,7 +20207,7 @@
       <c r="AM68" s="1"/>
       <c r="AN68" s="83"/>
     </row>
-    <row r="69" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="22" t="s">
         <v>301</v>
       </c>
@@ -20301,7 +20302,7 @@
       <c r="AM69" s="1"/>
       <c r="AN69" s="83"/>
     </row>
-    <row r="70" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="22" t="s">
         <v>304</v>
       </c>
@@ -20394,7 +20395,7 @@
       <c r="AM70" s="1"/>
       <c r="AN70" s="83"/>
     </row>
-    <row r="71" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="22" t="s">
         <v>306</v>
       </c>
@@ -20487,7 +20488,7 @@
       <c r="AM71" s="1"/>
       <c r="AN71" s="83"/>
     </row>
-    <row r="72" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="22" t="s">
         <v>309</v>
       </c>
@@ -20582,7 +20583,7 @@
       <c r="AM72" s="1"/>
       <c r="AN72" s="83"/>
     </row>
-    <row r="73" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="22" t="s">
         <v>312</v>
       </c>
@@ -20675,7 +20676,7 @@
       <c r="AM73" s="1"/>
       <c r="AN73" s="83"/>
     </row>
-    <row r="74" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" s="22" t="s">
         <v>314</v>
       </c>
@@ -20768,7 +20769,7 @@
       <c r="AM74" s="1"/>
       <c r="AN74" s="83"/>
     </row>
-    <row r="75" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" s="22" t="s">
         <v>316</v>
       </c>
@@ -20859,7 +20860,7 @@
       <c r="AM75" s="1"/>
       <c r="AN75" s="83"/>
     </row>
-    <row r="76" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" s="22" t="s">
         <v>319</v>
       </c>
@@ -20952,7 +20953,7 @@
       <c r="AM76" s="1"/>
       <c r="AN76" s="83"/>
     </row>
-    <row r="77" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" s="22" t="s">
         <v>323</v>
       </c>
@@ -21043,7 +21044,7 @@
       <c r="AM77" s="1"/>
       <c r="AN77" s="83"/>
     </row>
-    <row r="78" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" s="22" t="s">
         <v>325</v>
       </c>
@@ -21156,7 +21157,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="79" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" s="22" t="s">
         <v>329</v>
       </c>
@@ -21249,7 +21250,7 @@
       <c r="AM79" s="1"/>
       <c r="AN79" s="83"/>
     </row>
-    <row r="80" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" s="22" t="s">
         <v>332</v>
       </c>
@@ -21362,7 +21363,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="81" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="22" t="s">
         <v>336</v>
       </c>
@@ -21457,7 +21458,7 @@
       <c r="AM81" s="1"/>
       <c r="AN81" s="83"/>
     </row>
-    <row r="82" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" s="22" t="s">
         <v>338</v>
       </c>
@@ -21550,7 +21551,7 @@
       <c r="AM82" s="1"/>
       <c r="AN82" s="83"/>
     </row>
-    <row r="83" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" s="22" t="s">
         <v>340</v>
       </c>
@@ -21643,7 +21644,7 @@
       <c r="AM83" s="1"/>
       <c r="AN83" s="83"/>
     </row>
-    <row r="84" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" s="22" t="s">
         <v>342</v>
       </c>
@@ -21738,7 +21739,7 @@
       <c r="AM84" s="1"/>
       <c r="AN84" s="83"/>
     </row>
-    <row r="85" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" s="22" t="s">
         <v>345</v>
       </c>
@@ -21831,7 +21832,7 @@
       <c r="AM85" s="1"/>
       <c r="AN85" s="83"/>
     </row>
-    <row r="86" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" s="22" t="s">
         <v>347</v>
       </c>
@@ -21920,7 +21921,7 @@
       <c r="AM86" s="1"/>
       <c r="AN86" s="83"/>
     </row>
-    <row r="87" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" s="22" t="s">
         <v>352</v>
       </c>
@@ -22013,7 +22014,7 @@
       <c r="AM87" s="1"/>
       <c r="AN87" s="83"/>
     </row>
-    <row r="88" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" s="22" t="s">
         <v>354</v>
       </c>
@@ -22108,7 +22109,7 @@
       <c r="AM88" s="1"/>
       <c r="AN88" s="83"/>
     </row>
-    <row r="89" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" s="22" t="s">
         <v>359</v>
       </c>
@@ -22201,7 +22202,7 @@
       <c r="AM89" s="1"/>
       <c r="AN89" s="83"/>
     </row>
-    <row r="90" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" s="22" t="s">
         <v>362</v>
       </c>
@@ -22294,7 +22295,7 @@
       <c r="AM90" s="1"/>
       <c r="AN90" s="83"/>
     </row>
-    <row r="91" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" s="22" t="s">
         <v>364</v>
       </c>
@@ -22387,7 +22388,7 @@
       <c r="AM91" s="1"/>
       <c r="AN91" s="83"/>
     </row>
-    <row r="92" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" s="22" t="s">
         <v>367</v>
       </c>
@@ -22480,7 +22481,7 @@
       <c r="AM92" s="1"/>
       <c r="AN92" s="83"/>
     </row>
-    <row r="93" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" s="22" t="s">
         <v>370</v>
       </c>
@@ -22571,7 +22572,7 @@
       <c r="AM93" s="1"/>
       <c r="AN93" s="83"/>
     </row>
-    <row r="94" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" s="22" t="s">
         <v>372</v>
       </c>
@@ -22664,7 +22665,7 @@
       <c r="AM94" s="1"/>
       <c r="AN94" s="83"/>
     </row>
-    <row r="95" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" s="15" t="s">
         <v>375</v>
       </c>
@@ -22757,7 +22758,7 @@
       <c r="AM95" s="1"/>
       <c r="AN95" s="83"/>
     </row>
-    <row r="96" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" s="22" t="s">
         <v>378</v>
       </c>
@@ -22870,7 +22871,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="97" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" s="22" t="s">
         <v>381</v>
       </c>
@@ -22957,7 +22958,7 @@
       <c r="AM97" s="1"/>
       <c r="AN97" s="83"/>
     </row>
-    <row r="98" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" s="3" t="s">
         <v>382</v>
       </c>
@@ -23052,7 +23053,7 @@
       <c r="AM98" s="1"/>
       <c r="AN98" s="83"/>
     </row>
-    <row r="99" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" s="22" t="s">
         <v>386</v>
       </c>
@@ -23147,7 +23148,7 @@
       <c r="AM99" s="1"/>
       <c r="AN99" s="83"/>
     </row>
-    <row r="100" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" s="22" t="s">
         <v>388</v>
       </c>
@@ -23240,7 +23241,7 @@
       <c r="AM100" s="1"/>
       <c r="AN100" s="83"/>
     </row>
-    <row r="101" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" s="22" t="s">
         <v>391</v>
       </c>
@@ -23333,7 +23334,7 @@
       <c r="AM101" s="1"/>
       <c r="AN101" s="83"/>
     </row>
-    <row r="102" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" s="22" t="s">
         <v>394</v>
       </c>
@@ -23422,7 +23423,7 @@
       <c r="AM102" s="1"/>
       <c r="AN102" s="83"/>
     </row>
-    <row r="103" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" s="22" t="s">
         <v>397</v>
       </c>
@@ -23515,7 +23516,7 @@
       <c r="AM103" s="1"/>
       <c r="AN103" s="83"/>
     </row>
-    <row r="104" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" s="22" t="s">
         <v>398</v>
       </c>
@@ -23610,7 +23611,7 @@
       <c r="AM104" s="1"/>
       <c r="AN104" s="83"/>
     </row>
-    <row r="105" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="22" t="s">
         <v>400</v>
       </c>
@@ -23697,7 +23698,7 @@
       <c r="AM105" s="1"/>
       <c r="AN105" s="83"/>
     </row>
-    <row r="106" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" s="22" t="s">
         <v>402</v>
       </c>
@@ -23790,7 +23791,7 @@
       <c r="AM106" s="1"/>
       <c r="AN106" s="83"/>
     </row>
-    <row r="107" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" s="15" t="s">
         <v>404</v>
       </c>
@@ -23877,7 +23878,7 @@
       <c r="AM107" s="1"/>
       <c r="AN107" s="83"/>
     </row>
-    <row r="108" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" s="22" t="s">
         <v>406</v>
       </c>
@@ -23968,7 +23969,7 @@
       <c r="AM108" s="1"/>
       <c r="AN108" s="83"/>
     </row>
-    <row r="109" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" s="22" t="s">
         <v>408</v>
       </c>
@@ -24061,7 +24062,7 @@
       <c r="AM109" s="1"/>
       <c r="AN109" s="83"/>
     </row>
-    <row r="110" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" s="22" t="s">
         <v>410</v>
       </c>
@@ -24176,7 +24177,7 @@
       </c>
       <c r="AN110" s="83"/>
     </row>
-    <row r="111" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" s="22" t="s">
         <v>414</v>
       </c>
@@ -24271,7 +24272,7 @@
       <c r="AM111" s="1"/>
       <c r="AN111" s="83"/>
     </row>
-    <row r="112" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" s="22" t="s">
         <v>416</v>
       </c>
@@ -24386,7 +24387,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="113" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" s="22" t="s">
         <v>419</v>
       </c>
@@ -24475,7 +24476,7 @@
       <c r="AM113" s="1"/>
       <c r="AN113" s="83"/>
     </row>
-    <row r="114" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" s="22" t="s">
         <v>423</v>
       </c>
@@ -24562,7 +24563,7 @@
       <c r="AM114" s="1"/>
       <c r="AN114" s="83"/>
     </row>
-    <row r="115" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" s="3" t="s">
         <v>424</v>
       </c>
@@ -24655,7 +24656,7 @@
       <c r="AM115" s="1"/>
       <c r="AN115" s="83"/>
     </row>
-    <row r="116" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" s="22" t="s">
         <v>426</v>
       </c>
@@ -24740,7 +24741,7 @@
       <c r="AM116" s="1"/>
       <c r="AN116" s="83"/>
     </row>
-    <row r="117" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" s="22" t="s">
         <v>428</v>
       </c>
@@ -24835,7 +24836,7 @@
       <c r="AM117" s="1"/>
       <c r="AN117" s="83"/>
     </row>
-    <row r="118" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" s="22" t="s">
         <v>430</v>
       </c>
@@ -24928,7 +24929,7 @@
       <c r="AM118" s="1"/>
       <c r="AN118" s="83"/>
     </row>
-    <row r="119" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" s="22" t="s">
         <v>432</v>
       </c>
@@ -25019,7 +25020,7 @@
       <c r="AM119" s="1"/>
       <c r="AN119" s="83"/>
     </row>
-    <row r="120" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" s="15" t="s">
         <v>434</v>
       </c>
@@ -25104,7 +25105,7 @@
       <c r="AM120" s="1"/>
       <c r="AN120" s="83"/>
     </row>
-    <row r="121" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" s="22" t="s">
         <v>435</v>
       </c>
@@ -25195,7 +25196,7 @@
       <c r="AM121" s="1"/>
       <c r="AN121" s="83"/>
     </row>
-    <row r="122" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" s="15" t="s">
         <v>437</v>
       </c>
@@ -25282,7 +25283,7 @@
       <c r="AM122" s="1"/>
       <c r="AN122" s="83"/>
     </row>
-    <row r="123" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" s="22" t="s">
         <v>438</v>
       </c>
@@ -25393,7 +25394,7 @@
         <v>46113</v>
       </c>
     </row>
-    <row r="124" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" s="22" t="s">
         <v>440</v>
       </c>
@@ -25478,7 +25479,7 @@
       <c r="AM124" s="1"/>
       <c r="AN124" s="83"/>
     </row>
-    <row r="125" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" s="22" t="s">
         <v>441</v>
       </c>
@@ -25573,7 +25574,7 @@
       <c r="AM125" s="1"/>
       <c r="AN125" s="83"/>
     </row>
-    <row r="126" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" s="22" t="s">
         <v>443</v>
       </c>
@@ -25662,7 +25663,7 @@
       <c r="AM126" s="1"/>
       <c r="AN126" s="83"/>
     </row>
-    <row r="127" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" s="22" t="s">
         <v>446</v>
       </c>
@@ -25755,7 +25756,7 @@
       <c r="AM127" s="1"/>
       <c r="AN127" s="83"/>
     </row>
-    <row r="128" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" s="22" t="s">
         <v>448</v>
       </c>
@@ -25844,7 +25845,7 @@
       <c r="AM128" s="1"/>
       <c r="AN128" s="83"/>
     </row>
-    <row r="129" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" s="15" t="s">
         <v>451</v>
       </c>
@@ -25937,7 +25938,7 @@
       <c r="AM129" s="1"/>
       <c r="AN129" s="83"/>
     </row>
-    <row r="130" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" s="22" t="s">
         <v>453</v>
       </c>
@@ -26020,7 +26021,7 @@
       <c r="AM130" s="1"/>
       <c r="AN130" s="83"/>
     </row>
-    <row r="131" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" s="22" t="s">
         <v>454</v>
       </c>
@@ -26103,7 +26104,7 @@
       <c r="AM131" s="1"/>
       <c r="AN131" s="83"/>
     </row>
-    <row r="132" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" s="22" t="s">
         <v>455</v>
       </c>
@@ -26196,7 +26197,7 @@
       <c r="AM132" s="1"/>
       <c r="AN132" s="83"/>
     </row>
-    <row r="133" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" s="22" t="s">
         <v>457</v>
       </c>
@@ -26291,7 +26292,7 @@
       <c r="AM133" s="1"/>
       <c r="AN133" s="83"/>
     </row>
-    <row r="134" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" s="22" t="s">
         <v>459</v>
       </c>
@@ -26382,7 +26383,7 @@
       <c r="AM134" s="1"/>
       <c r="AN134" s="83"/>
     </row>
-    <row r="135" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" s="15" t="s">
         <v>461</v>
       </c>
@@ -26471,7 +26472,7 @@
       <c r="AM135" s="1"/>
       <c r="AN135" s="83"/>
     </row>
-    <row r="136" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" s="22" t="s">
         <v>463</v>
       </c>
@@ -26562,7 +26563,7 @@
       <c r="AM136" s="1"/>
       <c r="AN136" s="83"/>
     </row>
-    <row r="137" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" s="15" t="s">
         <v>465</v>
       </c>
@@ -26647,7 +26648,7 @@
       <c r="AM137" s="1"/>
       <c r="AN137" s="83"/>
     </row>
-    <row r="138" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" s="22" t="s">
         <v>467</v>
       </c>
@@ -26738,7 +26739,7 @@
       <c r="AM138" s="1"/>
       <c r="AN138" s="83"/>
     </row>
-    <row r="139" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" s="15" t="s">
         <v>468</v>
       </c>
@@ -26825,7 +26826,7 @@
       <c r="AM139" s="1"/>
       <c r="AN139" s="83"/>
     </row>
-    <row r="140" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" s="22" t="s">
         <v>471</v>
       </c>
@@ -26916,7 +26917,7 @@
       <c r="AM140" s="1"/>
       <c r="AN140" s="83"/>
     </row>
-    <row r="141" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" s="22" t="s">
         <v>474</v>
       </c>
@@ -27001,7 +27002,7 @@
       <c r="AM141" s="1"/>
       <c r="AN141" s="83"/>
     </row>
-    <row r="142" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" s="15" t="s">
         <v>475</v>
       </c>
@@ -27092,7 +27093,7 @@
       <c r="AM142" s="1"/>
       <c r="AN142" s="83"/>
     </row>
-    <row r="143" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" s="15" t="s">
         <v>477</v>
       </c>
@@ -27179,7 +27180,7 @@
       <c r="AM143" s="1"/>
       <c r="AN143" s="83"/>
     </row>
-    <row r="144" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" s="15" t="s">
         <v>480</v>
       </c>
@@ -27274,7 +27275,7 @@
       <c r="AM144" s="1"/>
       <c r="AN144" s="83"/>
     </row>
-    <row r="145" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" s="15" t="s">
         <v>482</v>
       </c>
@@ -27361,7 +27362,7 @@
       <c r="AM145" s="1"/>
       <c r="AN145" s="83"/>
     </row>
-    <row r="146" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" s="15" t="s">
         <v>483</v>
       </c>
@@ -27446,7 +27447,7 @@
       <c r="AM146" s="1"/>
       <c r="AN146" s="83"/>
     </row>
-    <row r="147" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" s="15" t="s">
         <v>484</v>
       </c>
@@ -27527,7 +27528,7 @@
       <c r="AM147" s="1"/>
       <c r="AN147" s="83"/>
     </row>
-    <row r="148" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" s="15" t="s">
         <v>485</v>
       </c>
@@ -27620,7 +27621,7 @@
       <c r="AM148" s="1"/>
       <c r="AN148" s="83"/>
     </row>
-    <row r="149" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" s="15" t="s">
         <v>487</v>
       </c>
@@ -27711,7 +27712,7 @@
       <c r="AM149" s="1"/>
       <c r="AN149" s="83"/>
     </row>
-    <row r="150" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" s="15" t="s">
         <v>489</v>
       </c>
@@ -27792,7 +27793,7 @@
       <c r="AM150" s="1"/>
       <c r="AN150" s="83"/>
     </row>
-    <row r="151" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" s="15" t="s">
         <v>490</v>
       </c>
@@ -27879,7 +27880,7 @@
       <c r="AM151" s="1"/>
       <c r="AN151" s="83"/>
     </row>
-    <row r="152" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" s="15" t="s">
         <v>492</v>
       </c>
@@ -27970,7 +27971,7 @@
       <c r="AM152" s="1"/>
       <c r="AN152" s="83"/>
     </row>
-    <row r="153" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" s="15" t="s">
         <v>495</v>
       </c>
@@ -28057,7 +28058,7 @@
       <c r="AM153" s="1"/>
       <c r="AN153" s="83"/>
     </row>
-    <row r="154" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" s="15" t="s">
         <v>497</v>
       </c>
@@ -28144,7 +28145,7 @@
       <c r="AM154" s="1"/>
       <c r="AN154" s="83"/>
     </row>
-    <row r="155" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" s="15" t="s">
         <v>499</v>
       </c>
@@ -28231,7 +28232,7 @@
       <c r="AM155" s="1"/>
       <c r="AN155" s="83"/>
     </row>
-    <row r="156" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" s="15" t="s">
         <v>501</v>
       </c>
@@ -28320,7 +28321,7 @@
       <c r="AM156" s="1"/>
       <c r="AN156" s="83"/>
     </row>
-    <row r="157" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" s="15" t="s">
         <v>504</v>
       </c>
@@ -28407,7 +28408,7 @@
       <c r="AM157" s="1"/>
       <c r="AN157" s="83"/>
     </row>
-    <row r="158" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" s="15" t="s">
         <v>506</v>
       </c>
@@ -28494,7 +28495,7 @@
       <c r="AM158" s="1"/>
       <c r="AN158" s="83"/>
     </row>
-    <row r="159" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" s="15" t="s">
         <v>508</v>
       </c>
@@ -28583,7 +28584,7 @@
       <c r="AM159" s="1"/>
       <c r="AN159" s="83"/>
     </row>
-    <row r="160" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" s="15" t="s">
         <v>510</v>
       </c>
@@ -28670,7 +28671,7 @@
       <c r="AM160" s="1"/>
       <c r="AN160" s="83"/>
     </row>
-    <row r="161" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" s="15" t="s">
         <v>512</v>
       </c>
@@ -28757,7 +28758,7 @@
       <c r="AM161" s="1"/>
       <c r="AN161" s="83"/>
     </row>
-    <row r="162" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" s="15" t="s">
         <v>514</v>
       </c>
@@ -28848,7 +28849,7 @@
       <c r="AM162" s="1"/>
       <c r="AN162" s="83"/>
     </row>
-    <row r="163" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" s="15" t="s">
         <v>517</v>
       </c>
@@ -28935,7 +28936,7 @@
       <c r="AM163" s="1"/>
       <c r="AN163" s="83"/>
     </row>
-    <row r="164" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" s="15" t="s">
         <v>519</v>
       </c>
@@ -29022,7 +29023,7 @@
       <c r="AM164" s="1"/>
       <c r="AN164" s="83"/>
     </row>
-    <row r="165" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" s="15" t="s">
         <v>521</v>
       </c>
@@ -29111,7 +29112,7 @@
       <c r="AM165" s="1"/>
       <c r="AN165" s="83"/>
     </row>
-    <row r="166" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" s="15" t="s">
         <v>523</v>
       </c>
@@ -29200,7 +29201,7 @@
       <c r="AM166" s="1"/>
       <c r="AN166" s="83"/>
     </row>
-    <row r="167" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" s="15" t="s">
         <v>525</v>
       </c>
@@ -29289,7 +29290,7 @@
       <c r="AM167" s="1"/>
       <c r="AN167" s="83"/>
     </row>
-    <row r="168" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" s="15" t="s">
         <v>527</v>
       </c>
@@ -29378,7 +29379,7 @@
       <c r="AM168" s="1"/>
       <c r="AN168" s="83"/>
     </row>
-    <row r="169" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" s="15" t="s">
         <v>529</v>
       </c>
@@ -29465,7 +29466,7 @@
       <c r="AM169" s="1"/>
       <c r="AN169" s="83"/>
     </row>
-    <row r="170" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" s="15" t="s">
         <v>531</v>
       </c>
@@ -29554,7 +29555,7 @@
       <c r="AM170" s="1"/>
       <c r="AN170" s="83"/>
     </row>
-    <row r="171" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" s="15" t="s">
         <v>533</v>
       </c>
@@ -29643,7 +29644,7 @@
       <c r="AM171" s="1"/>
       <c r="AN171" s="83"/>
     </row>
-    <row r="172" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" s="15" t="s">
         <v>535</v>
       </c>
@@ -29730,7 +29731,7 @@
       <c r="AM172" s="1"/>
       <c r="AN172" s="83"/>
     </row>
-    <row r="173" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" s="15" t="s">
         <v>537</v>
       </c>
@@ -29819,7 +29820,7 @@
       <c r="AM173" s="1"/>
       <c r="AN173" s="83"/>
     </row>
-    <row r="174" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" s="15" t="s">
         <v>539</v>
       </c>
@@ -29908,7 +29909,7 @@
       <c r="AM174" s="1"/>
       <c r="AN174" s="83"/>
     </row>
-    <row r="175" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" s="15" t="s">
         <v>541</v>
       </c>
@@ -29981,7 +29982,7 @@
       <c r="AM175" s="1"/>
       <c r="AN175" s="83"/>
     </row>
-    <row r="176" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" s="15" t="s">
         <v>542</v>
       </c>
@@ -30068,7 +30069,7 @@
       <c r="AM176" s="1"/>
       <c r="AN176" s="83"/>
     </row>
-    <row r="177" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" s="15" t="s">
         <v>545</v>
       </c>
@@ -30153,7 +30154,7 @@
       <c r="AM177" s="1"/>
       <c r="AN177" s="83"/>
     </row>
-    <row r="178" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" s="15" t="s">
         <v>547</v>
       </c>
@@ -30244,7 +30245,7 @@
       <c r="AM178" s="1"/>
       <c r="AN178" s="83"/>
     </row>
-    <row r="179" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" s="15" t="s">
         <v>548</v>
       </c>
@@ -30331,7 +30332,7 @@
       <c r="AM179" s="1"/>
       <c r="AN179" s="83"/>
     </row>
-    <row r="180" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" s="15" t="s">
         <v>552</v>
       </c>
@@ -30446,7 +30447,7 @@
         <v>46204</v>
       </c>
     </row>
-    <row r="181" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" s="15" t="s">
         <v>557</v>
       </c>
@@ -30561,7 +30562,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="182" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" s="15" t="s">
         <v>562</v>
       </c>
@@ -30652,7 +30653,7 @@
       <c r="AM182" s="1"/>
       <c r="AN182" s="83"/>
     </row>
-    <row r="183" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" s="15" t="s">
         <v>564</v>
       </c>
@@ -30741,7 +30742,7 @@
       <c r="AM183" s="1"/>
       <c r="AN183" s="83"/>
     </row>
-    <row r="184" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" s="15" t="s">
         <v>565</v>
       </c>
@@ -30830,7 +30831,7 @@
       <c r="AM184" s="1"/>
       <c r="AN184" s="83"/>
     </row>
-    <row r="185" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185" s="15" t="s">
         <v>567</v>
       </c>
@@ -30917,7 +30918,7 @@
       <c r="AM185" s="1"/>
       <c r="AN185" s="83"/>
     </row>
-    <row r="186" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" s="15" t="s">
         <v>570</v>
       </c>
@@ -31004,7 +31005,7 @@
       <c r="AM186" s="1"/>
       <c r="AN186" s="83"/>
     </row>
-    <row r="187" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187" s="15" t="s">
         <v>572</v>
       </c>
@@ -31091,7 +31092,7 @@
       <c r="AM187" s="1"/>
       <c r="AN187" s="83"/>
     </row>
-    <row r="188" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" s="15" t="s">
         <v>575</v>
       </c>
@@ -31178,7 +31179,7 @@
       <c r="AM188" s="1"/>
       <c r="AN188" s="83"/>
     </row>
-    <row r="189" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" s="15" t="s">
         <v>578</v>
       </c>
@@ -31265,7 +31266,7 @@
       <c r="AM189" s="1"/>
       <c r="AN189" s="83"/>
     </row>
-    <row r="190" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" s="15" t="s">
         <v>580</v>
       </c>
@@ -31352,7 +31353,7 @@
       <c r="AM190" s="1"/>
       <c r="AN190" s="83"/>
     </row>
-    <row r="191" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" s="15" t="s">
         <v>582</v>
       </c>
@@ -31433,7 +31434,7 @@
       <c r="AM191" s="1"/>
       <c r="AN191" s="83"/>
     </row>
-    <row r="192" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" s="15" t="s">
         <v>584</v>
       </c>
@@ -31520,7 +31521,7 @@
       <c r="AM192" s="1"/>
       <c r="AN192" s="83"/>
     </row>
-    <row r="193" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" s="15" t="s">
         <v>586</v>
       </c>
@@ -31609,7 +31610,7 @@
       <c r="AM193" s="1"/>
       <c r="AN193" s="83"/>
     </row>
-    <row r="194" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194" s="15" t="s">
         <v>589</v>
       </c>
@@ -31696,7 +31697,7 @@
       <c r="AM194" s="1"/>
       <c r="AN194" s="83"/>
     </row>
-    <row r="195" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" s="15" t="s">
         <v>592</v>
       </c>
@@ -31783,7 +31784,7 @@
       <c r="AM195" s="1"/>
       <c r="AN195" s="83"/>
     </row>
-    <row r="196" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196" s="15" t="s">
         <v>595</v>
       </c>
@@ -31872,7 +31873,7 @@
       <c r="AM196" s="1"/>
       <c r="AN196" s="83"/>
     </row>
-    <row r="197" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" s="15" t="s">
         <v>599</v>
       </c>
@@ -31961,7 +31962,7 @@
       <c r="AM197" s="1"/>
       <c r="AN197" s="83"/>
     </row>
-    <row r="198" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A198" s="15" t="s">
         <v>601</v>
       </c>
@@ -32050,7 +32051,7 @@
       <c r="AM198" s="1"/>
       <c r="AN198" s="83"/>
     </row>
-    <row r="199" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199" s="15" t="s">
         <v>603</v>
       </c>
@@ -32137,7 +32138,7 @@
       <c r="AM199" s="1"/>
       <c r="AN199" s="83"/>
     </row>
-    <row r="200" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200" s="15" t="s">
         <v>605</v>
       </c>
@@ -32224,7 +32225,7 @@
       <c r="AM200" s="1"/>
       <c r="AN200" s="83"/>
     </row>
-    <row r="201" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" s="15" t="s">
         <v>607</v>
       </c>
@@ -32311,7 +32312,7 @@
       <c r="AM201" s="1"/>
       <c r="AN201" s="83"/>
     </row>
-    <row r="202" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" s="15" t="s">
         <v>610</v>
       </c>
@@ -32402,7 +32403,7 @@
       <c r="AM202" s="1"/>
       <c r="AN202" s="83"/>
     </row>
-    <row r="203" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" s="15" t="s">
         <v>611</v>
       </c>
@@ -32489,7 +32490,7 @@
       <c r="AM203" s="1"/>
       <c r="AN203" s="83"/>
     </row>
-    <row r="204" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204" s="15" t="s">
         <v>612</v>
       </c>
@@ -32576,7 +32577,7 @@
       <c r="AM204" s="1"/>
       <c r="AN204" s="83"/>
     </row>
-    <row r="205" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" s="15" t="s">
         <v>614</v>
       </c>
@@ -32665,7 +32666,7 @@
       <c r="AM205" s="1"/>
       <c r="AN205" s="83"/>
     </row>
-    <row r="206" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206" s="15" t="s">
         <v>615</v>
       </c>
@@ -32758,7 +32759,7 @@
       <c r="AM206" s="1"/>
       <c r="AN206" s="83"/>
     </row>
-    <row r="207" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207" s="15" t="s">
         <v>616</v>
       </c>
@@ -32845,7 +32846,7 @@
       <c r="AM207" s="1"/>
       <c r="AN207" s="83"/>
     </row>
-    <row r="208" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A208" s="15" t="s">
         <v>619</v>
       </c>
@@ -32934,7 +32935,7 @@
       <c r="AM208" s="1"/>
       <c r="AN208" s="83"/>
     </row>
-    <row r="209" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209" s="15" t="s">
         <v>621</v>
       </c>
@@ -33021,7 +33022,7 @@
       <c r="AM209" s="1"/>
       <c r="AN209" s="83"/>
     </row>
-    <row r="210" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210" s="15" t="s">
         <v>623</v>
       </c>
@@ -33108,7 +33109,7 @@
       <c r="AM210" s="1"/>
       <c r="AN210" s="83"/>
     </row>
-    <row r="211" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211" s="15" t="s">
         <v>625</v>
       </c>
@@ -33195,7 +33196,7 @@
       <c r="AM211" s="1"/>
       <c r="AN211" s="83"/>
     </row>
-    <row r="212" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A212" s="15" t="s">
         <v>627</v>
       </c>
@@ -33284,7 +33285,7 @@
       <c r="AM212" s="1"/>
       <c r="AN212" s="83"/>
     </row>
-    <row r="213" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213" s="15" t="s">
         <v>629</v>
       </c>
@@ -33371,7 +33372,7 @@
       <c r="AM213" s="1"/>
       <c r="AN213" s="83"/>
     </row>
-    <row r="214" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214" s="15" t="s">
         <v>631</v>
       </c>
@@ -33458,7 +33459,7 @@
       <c r="AM214" s="1"/>
       <c r="AN214" s="83"/>
     </row>
-    <row r="215" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" s="15" t="s">
         <v>634</v>
       </c>
@@ -33547,7 +33548,7 @@
       <c r="AM215" s="1"/>
       <c r="AN215" s="83"/>
     </row>
-    <row r="216" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A216" s="15" t="s">
         <v>637</v>
       </c>
@@ -33632,7 +33633,7 @@
       <c r="AM216" s="1"/>
       <c r="AN216" s="83"/>
     </row>
-    <row r="217" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217" s="15" t="s">
         <v>639</v>
       </c>
@@ -33719,7 +33720,7 @@
       <c r="AM217" s="1"/>
       <c r="AN217" s="83"/>
     </row>
-    <row r="218" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A218" s="15" t="s">
         <v>642</v>
       </c>
@@ -33804,7 +33805,7 @@
       <c r="AM218" s="1"/>
       <c r="AN218" s="83"/>
     </row>
-    <row r="219" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A219" s="15" t="s">
         <v>644</v>
       </c>
@@ -33889,7 +33890,7 @@
       <c r="AM219" s="1"/>
       <c r="AN219" s="83"/>
     </row>
-    <row r="220" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A220" s="15" t="s">
         <v>646</v>
       </c>
@@ -33970,7 +33971,7 @@
       <c r="AM220" s="1"/>
       <c r="AN220" s="83"/>
     </row>
-    <row r="221" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A221" s="15" t="s">
         <v>647</v>
       </c>
@@ -34055,7 +34056,7 @@
       <c r="AM221" s="1"/>
       <c r="AN221" s="83"/>
     </row>
-    <row r="222" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A222" s="15" t="s">
         <v>650</v>
       </c>
@@ -34140,7 +34141,7 @@
       <c r="AM222" s="1"/>
       <c r="AN222" s="83"/>
     </row>
-    <row r="223" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A223" s="15" t="s">
         <v>653</v>
       </c>
@@ -34225,7 +34226,7 @@
       <c r="AM223" s="1"/>
       <c r="AN223" s="83"/>
     </row>
-    <row r="224" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A224" s="15" t="s">
         <v>655</v>
       </c>
@@ -34314,7 +34315,7 @@
       <c r="AM224" s="1"/>
       <c r="AN224" s="83"/>
     </row>
-    <row r="225" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A225" s="15" t="s">
         <v>657</v>
       </c>
@@ -34397,7 +34398,7 @@
       <c r="AM225" s="1"/>
       <c r="AN225" s="83"/>
     </row>
-    <row r="226" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A226" s="15" t="s">
         <v>659</v>
       </c>
@@ -34484,7 +34485,7 @@
       <c r="AM226" s="1"/>
       <c r="AN226" s="83"/>
     </row>
-    <row r="227" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A227" s="15" t="s">
         <v>661</v>
       </c>
@@ -34571,7 +34572,7 @@
       <c r="AM227" s="1"/>
       <c r="AN227" s="83"/>
     </row>
-    <row r="228" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A228" s="15" t="s">
         <v>664</v>
       </c>
@@ -34656,7 +34657,7 @@
       <c r="AM228" s="1"/>
       <c r="AN228" s="83"/>
     </row>
-    <row r="229" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A229" s="15" t="s">
         <v>666</v>
       </c>
@@ -34739,7 +34740,7 @@
       <c r="AM229" s="1"/>
       <c r="AN229" s="83"/>
     </row>
-    <row r="230" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A230" s="15" t="s">
         <v>667</v>
       </c>
@@ -34824,7 +34825,7 @@
       <c r="AM230" s="1"/>
       <c r="AN230" s="83"/>
     </row>
-    <row r="231" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A231" s="15" t="s">
         <v>669</v>
       </c>
@@ -34909,7 +34910,7 @@
       <c r="AM231" s="1"/>
       <c r="AN231" s="83"/>
     </row>
-    <row r="232" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A232" s="15" t="s">
         <v>671</v>
       </c>
@@ -34990,7 +34991,7 @@
       <c r="AM232" s="1"/>
       <c r="AN232" s="83"/>
     </row>
-    <row r="233" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A233" s="15" t="s">
         <v>672</v>
       </c>
@@ -35075,7 +35076,7 @@
       <c r="AM233" s="1"/>
       <c r="AN233" s="83"/>
     </row>
-    <row r="234" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A234" s="15" t="s">
         <v>674</v>
       </c>
@@ -35164,7 +35165,7 @@
       <c r="AM234" s="1"/>
       <c r="AN234" s="83"/>
     </row>
-    <row r="235" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A235" s="15" t="s">
         <v>675</v>
       </c>
@@ -35251,7 +35252,7 @@
       <c r="AM235" s="1"/>
       <c r="AN235" s="83"/>
     </row>
-    <row r="236" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A236" s="15" t="s">
         <v>678</v>
       </c>
@@ -35338,7 +35339,7 @@
       <c r="AM236" s="1"/>
       <c r="AN236" s="83"/>
     </row>
-    <row r="237" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A237" s="15" t="s">
         <v>680</v>
       </c>
@@ -35425,7 +35426,7 @@
       <c r="AM237" s="1"/>
       <c r="AN237" s="83"/>
     </row>
-    <row r="238" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A238" s="15" t="s">
         <v>683</v>
       </c>
@@ -35516,7 +35517,7 @@
       <c r="AM238" s="1"/>
       <c r="AN238" s="83"/>
     </row>
-    <row r="239" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A239" s="15" t="s">
         <v>686</v>
       </c>
@@ -35607,7 +35608,7 @@
       <c r="AM239" s="1"/>
       <c r="AN239" s="83"/>
     </row>
-    <row r="240" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A240" s="15" t="s">
         <v>688</v>
       </c>
@@ -35698,7 +35699,7 @@
       <c r="AM240" s="1"/>
       <c r="AN240" s="83"/>
     </row>
-    <row r="241" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A241" s="15" t="s">
         <v>690</v>
       </c>
@@ -35787,7 +35788,7 @@
       <c r="AM241" s="1"/>
       <c r="AN241" s="83"/>
     </row>
-    <row r="242" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A242" s="15" t="s">
         <v>692</v>
       </c>
@@ -35874,7 +35875,7 @@
       <c r="AM242" s="1"/>
       <c r="AN242" s="83"/>
     </row>
-    <row r="243" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A243" s="15" t="s">
         <v>694</v>
       </c>
@@ -35967,7 +35968,7 @@
       <c r="AM243" s="1"/>
       <c r="AN243" s="83"/>
     </row>
-    <row r="244" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A244" s="15" t="s">
         <v>696</v>
       </c>
@@ -36054,7 +36055,7 @@
       <c r="AM244" s="1"/>
       <c r="AN244" s="83"/>
     </row>
-    <row r="245" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A245" s="15" t="s">
         <v>698</v>
       </c>
@@ -36139,7 +36140,7 @@
       <c r="AM245" s="1"/>
       <c r="AN245" s="83"/>
     </row>
-    <row r="246" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A246" s="15" t="s">
         <v>700</v>
       </c>
@@ -36226,7 +36227,7 @@
       <c r="AM246" s="1"/>
       <c r="AN246" s="83"/>
     </row>
-    <row r="247" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A247" s="15" t="s">
         <v>702</v>
       </c>
@@ -36313,7 +36314,7 @@
       <c r="AM247" s="1"/>
       <c r="AN247" s="83"/>
     </row>
-    <row r="248" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A248" s="15" t="s">
         <v>704</v>
       </c>
@@ -36400,7 +36401,7 @@
       <c r="AM248" s="1"/>
       <c r="AN248" s="83"/>
     </row>
-    <row r="249" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A249" s="15" t="s">
         <v>706</v>
       </c>
@@ -36487,7 +36488,7 @@
       <c r="AM249" s="1"/>
       <c r="AN249" s="83"/>
     </row>
-    <row r="250" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A250" s="15" t="s">
         <v>708</v>
       </c>
@@ -36576,7 +36577,7 @@
       <c r="AM250" s="1"/>
       <c r="AN250" s="83"/>
     </row>
-    <row r="251" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A251" s="15" t="s">
         <v>709</v>
       </c>
@@ -36661,7 +36662,7 @@
       <c r="AM251" s="1"/>
       <c r="AN251" s="83"/>
     </row>
-    <row r="252" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A252" s="15" t="s">
         <v>711</v>
       </c>
@@ -36746,7 +36747,7 @@
       <c r="AM252" s="1"/>
       <c r="AN252" s="83"/>
     </row>
-    <row r="253" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A253" s="15" t="s">
         <v>713</v>
       </c>
@@ -36831,7 +36832,7 @@
       <c r="AM253" s="1"/>
       <c r="AN253" s="83"/>
     </row>
-    <row r="254" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A254" s="15" t="s">
         <v>715</v>
       </c>
@@ -36916,7 +36917,7 @@
       <c r="AM254" s="1"/>
       <c r="AN254" s="83"/>
     </row>
-    <row r="255" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A255" s="15" t="s">
         <v>717</v>
       </c>
@@ -37003,7 +37004,7 @@
       <c r="AM255" s="1"/>
       <c r="AN255" s="83"/>
     </row>
-    <row r="256" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A256" s="15" t="s">
         <v>719</v>
       </c>
@@ -37092,7 +37093,7 @@
       <c r="AM256" s="1"/>
       <c r="AN256" s="83"/>
     </row>
-    <row r="257" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257" s="15" t="s">
         <v>721</v>
       </c>
@@ -37179,7 +37180,7 @@
       <c r="AM257" s="1"/>
       <c r="AN257" s="83"/>
     </row>
-    <row r="258" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A258" s="15" t="s">
         <v>723</v>
       </c>
@@ -37266,7 +37267,7 @@
       <c r="AM258" s="1"/>
       <c r="AN258" s="83"/>
     </row>
-    <row r="259" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A259" s="15" t="s">
         <v>725</v>
       </c>
@@ -37353,7 +37354,7 @@
       <c r="AM259" s="1"/>
       <c r="AN259" s="83"/>
     </row>
-    <row r="260" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A260" s="15" t="s">
         <v>727</v>
       </c>
@@ -37438,7 +37439,7 @@
       <c r="AM260" s="1"/>
       <c r="AN260" s="83"/>
     </row>
-    <row r="261" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A261" s="15" t="s">
         <v>728</v>
       </c>
@@ -37519,7 +37520,7 @@
       <c r="AM261" s="1"/>
       <c r="AN261" s="83"/>
     </row>
-    <row r="262" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A262" s="15" t="s">
         <v>729</v>
       </c>
@@ -37600,7 +37601,7 @@
       <c r="AM262" s="1"/>
       <c r="AN262" s="83"/>
     </row>
-    <row r="263" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A263" s="15" t="s">
         <v>730</v>
       </c>
@@ -37677,7 +37678,7 @@
       <c r="AM263" s="1"/>
       <c r="AN263" s="83"/>
     </row>
-    <row r="264" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A264" s="15" t="s">
         <v>732</v>
       </c>
@@ -37758,7 +37759,7 @@
       <c r="AM264" s="1"/>
       <c r="AN264" s="83"/>
     </row>
-    <row r="265" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A265" s="15" t="s">
         <v>733</v>
       </c>
@@ -37835,7 +37836,7 @@
       <c r="AM265" s="1"/>
       <c r="AN265" s="83"/>
     </row>
-    <row r="266" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A266" s="15" t="s">
         <v>734</v>
       </c>
@@ -37916,7 +37917,7 @@
       <c r="AM266" s="1"/>
       <c r="AN266" s="83"/>
     </row>
-    <row r="267" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A267" s="15" t="s">
         <v>735</v>
       </c>
@@ -37999,7 +38000,7 @@
       <c r="AM267" s="1"/>
       <c r="AN267" s="83"/>
     </row>
-    <row r="268" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A268" s="15" t="s">
         <v>736</v>
       </c>
@@ -38080,7 +38081,7 @@
       <c r="AM268" s="1"/>
       <c r="AN268" s="83"/>
     </row>
-    <row r="269" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A269" s="15" t="s">
         <v>738</v>
       </c>
@@ -38161,7 +38162,7 @@
       <c r="AM269" s="1"/>
       <c r="AN269" s="83"/>
     </row>
-    <row r="270" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A270" s="15" t="s">
         <v>739</v>
       </c>
@@ -38242,7 +38243,7 @@
       <c r="AM270" s="1"/>
       <c r="AN270" s="83"/>
     </row>
-    <row r="271" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A271" s="15" t="s">
         <v>740</v>
       </c>
@@ -38323,7 +38324,7 @@
       <c r="AM271" s="1"/>
       <c r="AN271" s="83"/>
     </row>
-    <row r="272" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A272" s="31" t="s">
         <v>741</v>
       </c>
@@ -38404,7 +38405,7 @@
       <c r="AM272" s="1"/>
       <c r="AN272" s="83"/>
     </row>
-    <row r="273" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A273" s="15" t="s">
         <v>742</v>
       </c>
@@ -38487,7 +38488,7 @@
       <c r="AM273" s="1"/>
       <c r="AN273" s="83"/>
     </row>
-    <row r="274" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A274" s="15" t="s">
         <v>743</v>
       </c>
@@ -38568,7 +38569,7 @@
       <c r="AM274" s="1"/>
       <c r="AN274" s="83"/>
     </row>
-    <row r="275" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A275" s="15" t="s">
         <v>744</v>
       </c>
@@ -38649,7 +38650,7 @@
       <c r="AM275" s="1"/>
       <c r="AN275" s="83"/>
     </row>
-    <row r="276" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A276" s="15" t="s">
         <v>745</v>
       </c>
@@ -38730,7 +38731,7 @@
       <c r="AM276" s="1"/>
       <c r="AN276" s="83"/>
     </row>
-    <row r="277" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A277" s="15" t="s">
         <v>746</v>
       </c>
@@ -38811,7 +38812,7 @@
       <c r="AM277" s="1"/>
       <c r="AN277" s="83"/>
     </row>
-    <row r="278" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A278" s="15" t="s">
         <v>747</v>
       </c>
@@ -57805,7 +57806,7 @@
       <c r="AM497" s="1"/>
       <c r="AN497" s="83"/>
     </row>
-    <row r="498" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="498" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="A498" s="19" t="s">
         <v>1129</v>
       </c>
@@ -57920,7 +57921,7 @@
       </c>
       <c r="AO498" s="81"/>
     </row>
-    <row r="499" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="499" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A499" s="19" t="s">
         <v>1136</v>
       </c>
@@ -58035,7 +58036,7 @@
       </c>
       <c r="AO499" s="81"/>
     </row>
-    <row r="500" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="500" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A500" s="19" t="s">
         <v>1141</v>
       </c>
@@ -58148,7 +58149,7 @@
       </c>
       <c r="AO500" s="81"/>
     </row>
-    <row r="501" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="501" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A501" s="19" t="s">
         <v>1147</v>
       </c>
@@ -58263,7 +58264,7 @@
       </c>
       <c r="AO501" s="81"/>
     </row>
-    <row r="502" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="502" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="A502" s="19" t="s">
         <v>1150</v>
       </c>
@@ -58378,7 +58379,7 @@
       </c>
       <c r="AO502" s="81"/>
     </row>
-    <row r="503" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="503" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A503" s="19" t="s">
         <v>1154</v>
       </c>
@@ -58493,7 +58494,7 @@
       </c>
       <c r="AO503" s="81"/>
     </row>
-    <row r="504" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="504" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A504" s="19" t="s">
         <v>1158</v>
       </c>
@@ -58595,7 +58596,7 @@
       <c r="AN504" s="83"/>
       <c r="AO504" s="81"/>
     </row>
-    <row r="505" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="505" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A505" s="19" t="s">
         <v>1162</v>
       </c>
@@ -58710,7 +58711,7 @@
       </c>
       <c r="AO505" s="81"/>
     </row>
-    <row r="506" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="506" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A506" s="19" t="s">
         <v>1166</v>
       </c>
@@ -58825,7 +58826,7 @@
       </c>
       <c r="AO506" s="81"/>
     </row>
-    <row r="507" spans="1:41" s="26" customFormat="1" ht="30.6" x14ac:dyDescent="0.3">
+    <row r="507" spans="1:41" s="26" customFormat="1" ht="30.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A507" s="19" t="s">
         <v>1169</v>
       </c>
@@ -58940,7 +58941,7 @@
       </c>
       <c r="AO507" s="81"/>
     </row>
-    <row r="508" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="508" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A508" s="19" t="s">
         <v>1172</v>
       </c>
@@ -59045,7 +59046,7 @@
       <c r="AN508" s="83"/>
       <c r="AO508" s="81"/>
     </row>
-    <row r="509" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="509" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A509" s="19" t="s">
         <v>1174</v>
       </c>
@@ -59160,7 +59161,7 @@
       </c>
       <c r="AO509" s="81"/>
     </row>
-    <row r="510" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="510" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A510" s="19" t="s">
         <v>1177</v>
       </c>
@@ -59266,7 +59267,7 @@
       </c>
       <c r="AO510" s="81"/>
     </row>
-    <row r="511" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="511" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A511" s="19" t="s">
         <v>1179</v>
       </c>
@@ -59369,7 +59370,7 @@
       <c r="AN511" s="83"/>
       <c r="AO511" s="81"/>
     </row>
-    <row r="512" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="512" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A512" s="19" t="s">
         <v>1181</v>
       </c>
@@ -59484,7 +59485,7 @@
       </c>
       <c r="AO512" s="81"/>
     </row>
-    <row r="513" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="513" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="A513" s="19" t="s">
         <v>1184</v>
       </c>
@@ -59599,7 +59600,7 @@
       </c>
       <c r="AO513" s="81"/>
     </row>
-    <row r="514" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="514" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A514" s="19" t="s">
         <v>1187</v>
       </c>
@@ -59714,7 +59715,7 @@
       </c>
       <c r="AO514" s="81"/>
     </row>
-    <row r="515" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="515" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A515" s="19" t="s">
         <v>1190</v>
       </c>
@@ -59829,7 +59830,7 @@
       </c>
       <c r="AO515" s="81"/>
     </row>
-    <row r="516" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="516" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A516" s="19" t="s">
         <v>1193</v>
       </c>
@@ -59942,7 +59943,7 @@
       </c>
       <c r="AO516" s="81"/>
     </row>
-    <row r="517" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="517" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="A517" s="19" t="s">
         <v>388</v>
       </c>
@@ -60209,7 +60210,7 @@
       </c>
       <c r="AO519" s="81"/>
     </row>
-    <row r="520" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="520" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A520" s="19" t="s">
         <v>1200</v>
       </c>
@@ -60324,7 +60325,7 @@
       </c>
       <c r="AO520" s="81"/>
     </row>
-    <row r="521" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="521" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A521" s="19" t="s">
         <v>1205</v>
       </c>
@@ -60435,7 +60436,7 @@
       </c>
       <c r="AO521" s="81"/>
     </row>
-    <row r="522" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="522" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="A522" s="19" t="s">
         <v>1207</v>
       </c>
@@ -60550,7 +60551,7 @@
       </c>
       <c r="AO522" s="81"/>
     </row>
-    <row r="523" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="523" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A523" s="19" t="s">
         <v>1210</v>
       </c>
@@ -60655,7 +60656,7 @@
       <c r="AN523" s="83"/>
       <c r="AO523" s="81"/>
     </row>
-    <row r="524" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="524" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A524" s="19" t="s">
         <v>1214</v>
       </c>
@@ -60768,7 +60769,7 @@
       </c>
       <c r="AO524" s="81"/>
     </row>
-    <row r="525" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="525" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A525" s="19" t="s">
         <v>1218</v>
       </c>
@@ -60869,7 +60870,7 @@
       <c r="AN525" s="83"/>
       <c r="AO525" s="81"/>
     </row>
-    <row r="526" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="526" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A526" s="19" t="s">
         <v>1221</v>
       </c>
@@ -60984,7 +60985,7 @@
       </c>
       <c r="AO526" s="81"/>
     </row>
-    <row r="527" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="527" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A527" s="19" t="s">
         <v>1224</v>
       </c>
@@ -61099,7 +61100,7 @@
       </c>
       <c r="AO527" s="81"/>
     </row>
-    <row r="528" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="528" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A528" s="19" t="s">
         <v>1228</v>
       </c>
@@ -61214,7 +61215,7 @@
       </c>
       <c r="AO528" s="81"/>
     </row>
-    <row r="529" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="529" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="A529" s="19" t="s">
         <v>1231</v>
       </c>
@@ -61330,7 +61331,7 @@
       </c>
       <c r="AO529" s="81"/>
     </row>
-    <row r="530" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="530" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A530" s="19" t="s">
         <v>723</v>
       </c>
@@ -61430,7 +61431,7 @@
       <c r="AN530" s="83"/>
       <c r="AO530" s="81"/>
     </row>
-    <row r="531" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="531" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A531" s="19" t="s">
         <v>1234</v>
       </c>
@@ -61543,7 +61544,7 @@
       </c>
       <c r="AO531" s="81"/>
     </row>
-    <row r="532" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="532" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A532" s="19" t="s">
         <v>1237</v>
       </c>
@@ -61647,7 +61648,7 @@
       <c r="AN532" s="83"/>
       <c r="AO532" s="81"/>
     </row>
-    <row r="533" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="533" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A533" s="19" t="s">
         <v>1239</v>
       </c>
@@ -61751,7 +61752,7 @@
       <c r="AN533" s="83"/>
       <c r="AO533" s="81"/>
     </row>
-    <row r="534" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="534" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A534" s="19" t="s">
         <v>1241</v>
       </c>
@@ -61866,7 +61867,7 @@
       </c>
       <c r="AO534" s="81"/>
     </row>
-    <row r="535" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="535" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A535" s="19" t="s">
         <v>1245</v>
       </c>
@@ -61977,7 +61978,7 @@
       <c r="AN535" s="83"/>
       <c r="AO535" s="81"/>
     </row>
-    <row r="536" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="536" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A536" s="19" t="s">
         <v>1247</v>
       </c>
@@ -62081,7 +62082,7 @@
       <c r="AN536" s="83"/>
       <c r="AO536" s="81"/>
     </row>
-    <row r="537" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="537" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A537" s="19" t="s">
         <v>734</v>
       </c>
@@ -62194,7 +62195,7 @@
       </c>
       <c r="AO537" s="81"/>
     </row>
-    <row r="538" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="538" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A538" s="19" t="s">
         <v>1251</v>
       </c>
@@ -62306,7 +62307,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="539" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="539" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A539" s="19" t="s">
         <v>1253</v>
       </c>
@@ -62420,7 +62421,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="540" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="540" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A540" s="19" t="s">
         <v>1256</v>
       </c>
@@ -62523,7 +62524,7 @@
       <c r="AM540" s="1"/>
       <c r="AN540" s="83"/>
     </row>
-    <row r="541" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="541" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A541" s="19" t="s">
         <v>719</v>
       </c>
@@ -62622,7 +62623,7 @@
       <c r="AM541" s="1"/>
       <c r="AN541" s="83"/>
     </row>
-    <row r="542" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="542" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A542" s="19" t="s">
         <v>1259</v>
       </c>
@@ -62736,7 +62737,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="543" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="543" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A543" s="19" t="s">
         <v>1261</v>
       </c>
@@ -62839,7 +62840,7 @@
       <c r="AM543" s="1"/>
       <c r="AN543" s="83"/>
     </row>
-    <row r="544" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="544" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A544" s="19" t="s">
         <v>1263</v>
       </c>
@@ -62953,7 +62954,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="545" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="545" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A545" s="19" t="s">
         <v>1266</v>
       </c>
@@ -63067,7 +63068,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="546" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="546" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A546" s="19" t="s">
         <v>1268</v>
       </c>
@@ -63181,7 +63182,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="547" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="547" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A547" s="19" t="s">
         <v>1270</v>
       </c>
@@ -63284,7 +63285,7 @@
       <c r="AM547" s="1"/>
       <c r="AN547" s="83"/>
     </row>
-    <row r="548" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="548" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A548" s="19" t="s">
         <v>1271</v>
       </c>
@@ -63398,7 +63399,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="549" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="549" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A549" s="19" t="s">
         <v>1274</v>
       </c>
@@ -63501,7 +63502,7 @@
       <c r="AM549" s="1"/>
       <c r="AN549" s="83"/>
     </row>
-    <row r="550" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="550" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A550" s="19" t="s">
         <v>1275</v>
       </c>
@@ -63604,7 +63605,7 @@
       <c r="AM550" s="1"/>
       <c r="AN550" s="83"/>
     </row>
-    <row r="551" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="551" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A551" s="19" t="s">
         <v>1277</v>
       </c>
@@ -63707,7 +63708,7 @@
       <c r="AM551" s="1"/>
       <c r="AN551" s="83"/>
     </row>
-    <row r="552" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="552" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A552" s="19" t="s">
         <v>738</v>
       </c>
@@ -63808,7 +63809,7 @@
       <c r="AM552" s="1"/>
       <c r="AN552" s="83"/>
     </row>
-    <row r="553" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="553" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A553" s="19" t="s">
         <v>1278</v>
       </c>
@@ -63922,7 +63923,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="554" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="554" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A554" s="19" t="s">
         <v>1282</v>
       </c>
@@ -64025,7 +64026,7 @@
       <c r="AM554" s="1"/>
       <c r="AN554" s="83"/>
     </row>
-    <row r="555" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="555" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A555" s="19" t="s">
         <v>1283</v>
       </c>
@@ -64126,7 +64127,7 @@
       <c r="AM555" s="1"/>
       <c r="AN555" s="83"/>
     </row>
-    <row r="556" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="556" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A556" s="19" t="s">
         <v>1284</v>
       </c>
@@ -64240,7 +64241,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="557" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="557" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A557" s="19" t="s">
         <v>1287</v>
       </c>
@@ -64343,7 +64344,7 @@
       <c r="AM557" s="1"/>
       <c r="AN557" s="83"/>
     </row>
-    <row r="558" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="558" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A558" s="19" t="s">
         <v>1289</v>
       </c>
@@ -64444,7 +64445,7 @@
       <c r="AM558" s="1"/>
       <c r="AN558" s="83"/>
     </row>
-    <row r="559" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="559" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A559" s="19" t="s">
         <v>1291</v>
       </c>
@@ -64545,7 +64546,7 @@
       <c r="AM559" s="1"/>
       <c r="AN559" s="83"/>
     </row>
-    <row r="560" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="560" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A560" s="19" t="s">
         <v>1293</v>
       </c>
@@ -64657,7 +64658,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="561" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="561" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A561" s="19" t="s">
         <v>586</v>
       </c>
@@ -64760,7 +64761,7 @@
       <c r="AM561" s="1"/>
       <c r="AN561" s="83"/>
     </row>
-    <row r="562" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="562" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A562" s="19" t="s">
         <v>1296</v>
       </c>
@@ -64874,7 +64875,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="563" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="563" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A563" s="19" t="s">
         <v>1298</v>
       </c>
@@ -64988,7 +64989,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="564" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="564" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A564" s="19" t="s">
         <v>1301</v>
       </c>
@@ -65100,7 +65101,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="565" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="565" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A565" s="19" t="s">
         <v>1304</v>
       </c>
@@ -65201,7 +65202,7 @@
       <c r="AM565" s="1"/>
       <c r="AN565" s="83"/>
     </row>
-    <row r="566" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="566" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A566" s="19" t="s">
         <v>1306</v>
       </c>
@@ -65304,7 +65305,7 @@
       <c r="AM566" s="1"/>
       <c r="AN566" s="83"/>
     </row>
-    <row r="567" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="567" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A567" s="32" t="s">
         <v>1308</v>
       </c>
@@ -65405,7 +65406,7 @@
       <c r="AM567" s="1"/>
       <c r="AN567" s="83"/>
     </row>
-    <row r="568" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="568" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A568" s="19" t="s">
         <v>1310</v>
       </c>
@@ -65508,7 +65509,7 @@
       <c r="AM568" s="1"/>
       <c r="AN568" s="83"/>
     </row>
-    <row r="569" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="569" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A569" s="19" t="s">
         <v>1312</v>
       </c>
@@ -65622,7 +65623,7 @@
         <v>46174</v>
       </c>
     </row>
-    <row r="570" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="570" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A570" s="19" t="s">
         <v>1315</v>
       </c>
@@ -65723,7 +65724,7 @@
       <c r="AM570" s="1"/>
       <c r="AN570" s="83"/>
     </row>
-    <row r="571" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="571" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A571" s="19" t="s">
         <v>1317</v>
       </c>
@@ -65824,7 +65825,7 @@
       <c r="AM571" s="1"/>
       <c r="AN571" s="83"/>
     </row>
-    <row r="572" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="572" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A572" s="19" t="s">
         <v>1318</v>
       </c>
@@ -65925,7 +65926,7 @@
       <c r="AM572" s="1"/>
       <c r="AN572" s="83"/>
     </row>
-    <row r="573" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="573" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A573" s="19" t="s">
         <v>1320</v>
       </c>
@@ -66028,7 +66029,7 @@
       <c r="AM573" s="1"/>
       <c r="AN573" s="83"/>
     </row>
-    <row r="574" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="574" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A574" s="19" t="s">
         <v>1322</v>
       </c>
@@ -66131,7 +66132,7 @@
       <c r="AM574" s="1"/>
       <c r="AN574" s="83"/>
     </row>
-    <row r="575" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="575" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A575" s="19" t="s">
         <v>1325</v>
       </c>
@@ -66234,7 +66235,7 @@
       <c r="AM575" s="1"/>
       <c r="AN575" s="83"/>
     </row>
-    <row r="576" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="576" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A576" s="19" t="s">
         <v>1327</v>
       </c>
@@ -66337,7 +66338,7 @@
       <c r="AM576" s="1"/>
       <c r="AN576" s="83"/>
     </row>
-    <row r="577" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="577" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A577" s="19" t="s">
         <v>1329</v>
       </c>
@@ -66440,7 +66441,7 @@
       <c r="AM577" s="1"/>
       <c r="AN577" s="83"/>
     </row>
-    <row r="578" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="578" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A578" s="19" t="s">
         <v>1331</v>
       </c>
@@ -66541,7 +66542,7 @@
       <c r="AM578" s="1"/>
       <c r="AN578" s="83"/>
     </row>
-    <row r="579" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="579" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A579" s="19" t="s">
         <v>1332</v>
       </c>
@@ -66644,7 +66645,7 @@
       <c r="AM579" s="1"/>
       <c r="AN579" s="83"/>
     </row>
-    <row r="580" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="580" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A580" s="19" t="s">
         <v>1334</v>
       </c>
@@ -66747,7 +66748,7 @@
       <c r="AM580" s="1"/>
       <c r="AN580" s="83"/>
     </row>
-    <row r="581" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="581" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A581" s="19" t="s">
         <v>1335</v>
       </c>
@@ -66850,7 +66851,7 @@
       <c r="AM581" s="1"/>
       <c r="AN581" s="83"/>
     </row>
-    <row r="582" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="582" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A582" s="19" t="s">
         <v>1337</v>
       </c>
@@ -66953,7 +66954,7 @@
       <c r="AM582" s="1"/>
       <c r="AN582" s="83"/>
     </row>
-    <row r="583" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="583" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A583" s="19" t="s">
         <v>1339</v>
       </c>
@@ -67016,7 +67017,7 @@
       <c r="AM583" s="1"/>
       <c r="AN583" s="83"/>
     </row>
-    <row r="584" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="584" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A584" s="19" t="s">
         <v>1340</v>
       </c>
@@ -67119,7 +67120,7 @@
       <c r="AM584" s="1"/>
       <c r="AN584" s="83"/>
     </row>
-    <row r="585" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="585" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A585" s="19" t="s">
         <v>1342</v>
       </c>
@@ -67222,7 +67223,7 @@
       <c r="AM585" s="1"/>
       <c r="AN585" s="83"/>
     </row>
-    <row r="586" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="586" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A586" s="19" t="s">
         <v>1344</v>
       </c>
@@ -67325,7 +67326,7 @@
       <c r="AM586" s="1"/>
       <c r="AN586" s="83"/>
     </row>
-    <row r="587" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="587" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A587" s="19" t="s">
         <v>1346</v>
       </c>
@@ -67424,7 +67425,7 @@
       <c r="AM587" s="1"/>
       <c r="AN587" s="83"/>
     </row>
-    <row r="588" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="588" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A588" s="19" t="s">
         <v>299</v>
       </c>
@@ -67523,7 +67524,7 @@
       <c r="AM588" s="1"/>
       <c r="AN588" s="83"/>
     </row>
-    <row r="589" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="589" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A589" s="19" t="s">
         <v>1349</v>
       </c>
@@ -67626,7 +67627,7 @@
       <c r="AM589" s="1"/>
       <c r="AN589" s="83"/>
     </row>
-    <row r="590" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="590" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A590" s="19" t="s">
         <v>1351</v>
       </c>
@@ -67729,7 +67730,7 @@
       <c r="AM590" s="1"/>
       <c r="AN590" s="83"/>
     </row>
-    <row r="591" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="591" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A591" s="22" t="s">
         <v>1353</v>
       </c>
@@ -67804,7 +67805,7 @@
       <c r="AM591" s="1"/>
       <c r="AN591" s="83"/>
     </row>
-    <row r="592" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="592" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A592" s="22" t="s">
         <v>1356</v>
       </c>
@@ -67877,7 +67878,7 @@
       <c r="AM592" s="1"/>
       <c r="AN592" s="83"/>
     </row>
-    <row r="593" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="593" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A593" s="22" t="s">
         <v>1359</v>
       </c>
@@ -67950,7 +67951,7 @@
       <c r="AM593" s="1"/>
       <c r="AN593" s="83"/>
     </row>
-    <row r="594" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="594" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A594" s="22" t="s">
         <v>1360</v>
       </c>
@@ -68023,7 +68024,7 @@
       <c r="AM594" s="1"/>
       <c r="AN594" s="83"/>
     </row>
-    <row r="595" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="595" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A595" s="22" t="s">
         <v>647</v>
       </c>
@@ -68096,7 +68097,7 @@
       <c r="AM595" s="1"/>
       <c r="AN595" s="83"/>
     </row>
-    <row r="596" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="596" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A596" s="22" t="s">
         <v>1363</v>
       </c>
@@ -68169,7 +68170,7 @@
       <c r="AM596" s="1"/>
       <c r="AN596" s="83"/>
     </row>
-    <row r="597" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="597" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A597" s="22" t="s">
         <v>1364</v>
       </c>
@@ -68242,7 +68243,7 @@
       <c r="AM597" s="1"/>
       <c r="AN597" s="83"/>
     </row>
-    <row r="598" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="598" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A598" s="22" t="s">
         <v>1365</v>
       </c>
@@ -68315,7 +68316,7 @@
       <c r="AM598" s="1"/>
       <c r="AN598" s="83"/>
     </row>
-    <row r="599" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="599" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A599" s="22" t="s">
         <v>1368</v>
       </c>
@@ -68388,7 +68389,7 @@
       <c r="AM599" s="1"/>
       <c r="AN599" s="83"/>
     </row>
-    <row r="600" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="600" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A600" s="22" t="s">
         <v>1369</v>
       </c>
@@ -68461,7 +68462,7 @@
       <c r="AM600" s="1"/>
       <c r="AN600" s="83"/>
     </row>
-    <row r="601" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="601" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A601" s="22" t="s">
         <v>1371</v>
       </c>
@@ -68534,7 +68535,7 @@
       <c r="AM601" s="1"/>
       <c r="AN601" s="83"/>
     </row>
-    <row r="602" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="602" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A602" s="22" t="s">
         <v>868</v>
       </c>
@@ -68607,7 +68608,7 @@
       <c r="AM602" s="1"/>
       <c r="AN602" s="83"/>
     </row>
-    <row r="603" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="603" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A603" s="22" t="s">
         <v>1373</v>
       </c>
@@ -68680,7 +68681,7 @@
       <c r="AM603" s="1"/>
       <c r="AN603" s="83"/>
     </row>
-    <row r="604" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="604" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A604" s="22" t="s">
         <v>1374</v>
       </c>
@@ -68753,7 +68754,7 @@
       <c r="AM604" s="1"/>
       <c r="AN604" s="83"/>
     </row>
-    <row r="605" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="605" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A605" s="22" t="s">
         <v>655</v>
       </c>
@@ -68826,7 +68827,7 @@
       <c r="AM605" s="1"/>
       <c r="AN605" s="83"/>
     </row>
-    <row r="606" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="606" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A606" s="22" t="s">
         <v>275</v>
       </c>
@@ -68901,7 +68902,7 @@
       <c r="AM606" s="1"/>
       <c r="AN606" s="83"/>
     </row>
-    <row r="607" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="607" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A607" s="22" t="s">
         <v>1377</v>
       </c>
@@ -68974,7 +68975,7 @@
       <c r="AM607" s="1"/>
       <c r="AN607" s="83"/>
     </row>
-    <row r="608" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="608" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A608" s="22" t="s">
         <v>1378</v>
       </c>
@@ -69047,7 +69048,7 @@
       <c r="AM608" s="1"/>
       <c r="AN608" s="83"/>
     </row>
-    <row r="609" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="609" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A609" s="22" t="s">
         <v>378</v>
       </c>
@@ -69120,7 +69121,7 @@
       <c r="AM609" s="1"/>
       <c r="AN609" s="83"/>
     </row>
-    <row r="610" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="610" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A610" s="22" t="s">
         <v>370</v>
       </c>
@@ -69193,7 +69194,7 @@
       <c r="AM610" s="1"/>
       <c r="AN610" s="83"/>
     </row>
-    <row r="611" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="611" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A611" s="22" t="s">
         <v>1379</v>
       </c>
@@ -69266,7 +69267,7 @@
       <c r="AM611" s="1"/>
       <c r="AN611" s="83"/>
     </row>
-    <row r="612" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="612" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A612" s="22" t="s">
         <v>1380</v>
       </c>
@@ -69339,7 +69340,7 @@
       <c r="AM612" s="1"/>
       <c r="AN612" s="83"/>
     </row>
-    <row r="613" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="613" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A613" s="22" t="s">
         <v>1381</v>
       </c>
@@ -69412,7 +69413,7 @@
       <c r="AM613" s="1"/>
       <c r="AN613" s="83"/>
     </row>
-    <row r="614" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="614" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A614" s="22" t="s">
         <v>1383</v>
       </c>
@@ -69485,7 +69486,7 @@
       <c r="AM614" s="1"/>
       <c r="AN614" s="83"/>
     </row>
-    <row r="615" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="615" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A615" s="22" t="s">
         <v>672</v>
       </c>
@@ -69558,7 +69559,7 @@
       <c r="AM615" s="1"/>
       <c r="AN615" s="83"/>
     </row>
-    <row r="616" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="616" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A616" s="22" t="s">
         <v>1384</v>
       </c>
@@ -69631,7 +69632,7 @@
       <c r="AM616" s="1"/>
       <c r="AN616" s="83"/>
     </row>
-    <row r="617" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="617" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A617" s="22" t="s">
         <v>1386</v>
       </c>
@@ -69704,7 +69705,7 @@
       <c r="AM617" s="1"/>
       <c r="AN617" s="83"/>
     </row>
-    <row r="618" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="618" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A618" s="22" t="s">
         <v>880</v>
       </c>
@@ -69777,7 +69778,7 @@
       <c r="AM618" s="1"/>
       <c r="AN618" s="83"/>
     </row>
-    <row r="619" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="619" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A619" s="22" t="s">
         <v>907</v>
       </c>
@@ -69850,7 +69851,7 @@
       <c r="AM619" s="1"/>
       <c r="AN619" s="83"/>
     </row>
-    <row r="620" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="620" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A620" s="22" t="s">
         <v>877</v>
       </c>
@@ -69923,7 +69924,7 @@
       <c r="AM620" s="1"/>
       <c r="AN620" s="83"/>
     </row>
-    <row r="621" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="621" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A621" s="22" t="s">
         <v>1389</v>
       </c>
@@ -69996,7 +69997,7 @@
       <c r="AM621" s="1"/>
       <c r="AN621" s="83"/>
     </row>
-    <row r="622" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="622" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A622" s="22" t="s">
         <v>1390</v>
       </c>
@@ -70069,7 +70070,7 @@
       <c r="AM622" s="1"/>
       <c r="AN622" s="83"/>
     </row>
-    <row r="623" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="623" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A623" s="22" t="s">
         <v>859</v>
       </c>
@@ -70142,7 +70143,7 @@
       <c r="AM623" s="1"/>
       <c r="AN623" s="83"/>
     </row>
-    <row r="624" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="624" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A624" s="22" t="s">
         <v>1392</v>
       </c>
@@ -70215,7 +70216,7 @@
       <c r="AM624" s="1"/>
       <c r="AN624" s="83"/>
     </row>
-    <row r="625" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="625" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A625" s="22" t="s">
         <v>1393</v>
       </c>
@@ -70288,7 +70289,7 @@
       <c r="AM625" s="1"/>
       <c r="AN625" s="83"/>
     </row>
-    <row r="626" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="626" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A626" s="22" t="s">
         <v>406</v>
       </c>
@@ -70361,7 +70362,7 @@
       <c r="AM626" s="1"/>
       <c r="AN626" s="83"/>
     </row>
-    <row r="627" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="627" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A627" s="22" t="s">
         <v>1396</v>
       </c>
@@ -70434,7 +70435,7 @@
       <c r="AM627" s="1"/>
       <c r="AN627" s="83"/>
     </row>
-    <row r="628" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="628" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A628" s="22" t="s">
         <v>921</v>
       </c>
@@ -70507,7 +70508,7 @@
       <c r="AM628" s="1"/>
       <c r="AN628" s="83"/>
     </row>
-    <row r="629" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="629" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A629" s="22" t="s">
         <v>1398</v>
       </c>
@@ -70580,7 +70581,7 @@
       <c r="AM629" s="1"/>
       <c r="AN629" s="83"/>
     </row>
-    <row r="630" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="630" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A630" s="22" t="s">
         <v>892</v>
       </c>
@@ -70653,7 +70654,7 @@
       <c r="AM630" s="1"/>
       <c r="AN630" s="83"/>
     </row>
-    <row r="631" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="631" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A631" s="22" t="s">
         <v>1400</v>
       </c>
@@ -70726,7 +70727,7 @@
       <c r="AM631" s="1"/>
       <c r="AN631" s="83"/>
     </row>
-    <row r="632" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="632" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A632" s="22" t="s">
         <v>1401</v>
       </c>
@@ -70799,7 +70800,7 @@
       <c r="AM632" s="1"/>
       <c r="AN632" s="83"/>
     </row>
-    <row r="633" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="633" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A633" s="22" t="s">
         <v>1403</v>
       </c>
@@ -70872,7 +70873,7 @@
       <c r="AM633" s="1"/>
       <c r="AN633" s="83"/>
     </row>
-    <row r="634" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="634" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A634" s="22" t="s">
         <v>1404</v>
       </c>
@@ -70945,7 +70946,7 @@
       <c r="AM634" s="1"/>
       <c r="AN634" s="83"/>
     </row>
-    <row r="635" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="635" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A635" s="22" t="s">
         <v>1405</v>
       </c>
@@ -71018,7 +71019,7 @@
       <c r="AM635" s="1"/>
       <c r="AN635" s="83"/>
     </row>
-    <row r="636" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="636" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A636" s="22" t="s">
         <v>1406</v>
       </c>
@@ -71091,7 +71092,7 @@
       <c r="AM636" s="1"/>
       <c r="AN636" s="83"/>
     </row>
-    <row r="637" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="637" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A637" s="22" t="s">
         <v>1407</v>
       </c>
@@ -71164,7 +71165,7 @@
       <c r="AM637" s="1"/>
       <c r="AN637" s="83"/>
     </row>
-    <row r="638" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="638" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A638" s="22" t="s">
         <v>1409</v>
       </c>
@@ -71237,7 +71238,7 @@
       <c r="AM638" s="1"/>
       <c r="AN638" s="83"/>
     </row>
-    <row r="639" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="639" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A639" s="22" t="s">
         <v>1410</v>
       </c>
@@ -71310,7 +71311,7 @@
       <c r="AM639" s="1"/>
       <c r="AN639" s="83"/>
     </row>
-    <row r="640" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="640" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A640" s="22" t="s">
         <v>1411</v>
       </c>
@@ -71383,7 +71384,7 @@
       <c r="AM640" s="1"/>
       <c r="AN640" s="83"/>
     </row>
-    <row r="641" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="641" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A641" s="22" t="s">
         <v>898</v>
       </c>
@@ -71456,7 +71457,7 @@
       <c r="AM641" s="1"/>
       <c r="AN641" s="83"/>
     </row>
-    <row r="642" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="642" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A642" s="22" t="s">
         <v>967</v>
       </c>
@@ -71529,7 +71530,7 @@
       <c r="AM642" s="1"/>
       <c r="AN642" s="83"/>
     </row>
-    <row r="643" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="643" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A643" s="22" t="s">
         <v>1412</v>
       </c>
@@ -71602,7 +71603,7 @@
       <c r="AM643" s="1"/>
       <c r="AN643" s="83"/>
     </row>
-    <row r="644" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="644" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A644" s="22" t="s">
         <v>1414</v>
       </c>
@@ -71675,7 +71676,7 @@
       <c r="AM644" s="1"/>
       <c r="AN644" s="83"/>
     </row>
-    <row r="645" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="645" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A645" s="22" t="s">
         <v>874</v>
       </c>
@@ -71748,7 +71749,7 @@
       <c r="AM645" s="1"/>
       <c r="AN645" s="83"/>
     </row>
-    <row r="646" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="646" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A646" s="22" t="s">
         <v>1415</v>
       </c>
@@ -71821,7 +71822,7 @@
       <c r="AM646" s="1"/>
       <c r="AN646" s="83"/>
     </row>
-    <row r="647" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="647" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A647" s="22" t="s">
         <v>946</v>
       </c>
@@ -71894,7 +71895,7 @@
       <c r="AM647" s="1"/>
       <c r="AN647" s="83"/>
     </row>
-    <row r="648" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="648" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A648" s="22" t="s">
         <v>1416</v>
       </c>
@@ -71967,7 +71968,7 @@
       <c r="AM648" s="1"/>
       <c r="AN648" s="83"/>
     </row>
-    <row r="649" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="649" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A649" s="22" t="s">
         <v>97</v>
       </c>
@@ -72042,7 +72043,7 @@
       <c r="AM649" s="1"/>
       <c r="AN649" s="83"/>
     </row>
-    <row r="650" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="650" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A650" s="22" t="s">
         <v>1419</v>
       </c>
@@ -72115,7 +72116,7 @@
       <c r="AM650" s="1"/>
       <c r="AN650" s="83"/>
     </row>
-    <row r="651" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="651" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A651" s="22" t="s">
         <v>1420</v>
       </c>
@@ -72186,7 +72187,7 @@
       <c r="AM651" s="1"/>
       <c r="AN651" s="83"/>
     </row>
-    <row r="652" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="652" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A652" s="22" t="s">
         <v>650</v>
       </c>
@@ -72259,7 +72260,7 @@
       <c r="AM652" s="1"/>
       <c r="AN652" s="83"/>
     </row>
-    <row r="653" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="653" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A653" s="22" t="s">
         <v>1421</v>
       </c>
@@ -72332,7 +72333,7 @@
       <c r="AM653" s="1"/>
       <c r="AN653" s="83"/>
     </row>
-    <row r="654" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="654" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A654" s="22" t="s">
         <v>1423</v>
       </c>
@@ -72405,7 +72406,7 @@
       <c r="AM654" s="1"/>
       <c r="AN654" s="83"/>
     </row>
-    <row r="655" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="655" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A655" s="22" t="s">
         <v>1424</v>
       </c>
@@ -72478,7 +72479,7 @@
       <c r="AM655" s="1"/>
       <c r="AN655" s="83"/>
     </row>
-    <row r="656" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="656" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A656" s="22" t="s">
         <v>1426</v>
       </c>
@@ -72551,7 +72552,7 @@
       <c r="AM656" s="1"/>
       <c r="AN656" s="83"/>
     </row>
-    <row r="657" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="657" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A657" s="22" t="s">
         <v>1427</v>
       </c>
@@ -72624,7 +72625,7 @@
       <c r="AM657" s="1"/>
       <c r="AN657" s="83"/>
     </row>
-    <row r="658" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="658" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A658" s="22" t="s">
         <v>1428</v>
       </c>
@@ -72697,7 +72698,7 @@
       <c r="AM658" s="1"/>
       <c r="AN658" s="83"/>
     </row>
-    <row r="659" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="659" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A659" s="22" t="s">
         <v>1429</v>
       </c>
@@ -72770,7 +72771,7 @@
       <c r="AM659" s="1"/>
       <c r="AN659" s="83"/>
     </row>
-    <row r="660" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="660" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A660" s="22" t="s">
         <v>1430</v>
       </c>
@@ -72843,7 +72844,7 @@
       <c r="AM660" s="1"/>
       <c r="AN660" s="83"/>
     </row>
-    <row r="661" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="661" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A661" s="22" t="s">
         <v>1431</v>
       </c>
@@ -72916,7 +72917,7 @@
       <c r="AM661" s="1"/>
       <c r="AN661" s="83"/>
     </row>
-    <row r="662" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="662" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A662" s="22" t="s">
         <v>1432</v>
       </c>
@@ -72989,7 +72990,7 @@
       <c r="AM662" s="1"/>
       <c r="AN662" s="83"/>
     </row>
-    <row r="663" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="663" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A663" s="22" t="s">
         <v>966</v>
       </c>
@@ -73062,7 +73063,7 @@
       <c r="AM663" s="1"/>
       <c r="AN663" s="83"/>
     </row>
-    <row r="664" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="664" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A664" s="22" t="s">
         <v>578</v>
       </c>
@@ -73145,7 +73146,7 @@
       <c r="AM664" s="1"/>
       <c r="AN664" s="83"/>
     </row>
-    <row r="665" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="665" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A665" s="22" t="s">
         <v>1435</v>
       </c>
@@ -73218,7 +73219,7 @@
       <c r="AM665" s="1"/>
       <c r="AN665" s="83"/>
     </row>
-    <row r="666" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="666" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A666" s="22" t="s">
         <v>1437</v>
       </c>
@@ -73291,7 +73292,7 @@
       <c r="AM666" s="1"/>
       <c r="AN666" s="83"/>
     </row>
-    <row r="667" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="667" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A667" s="22" t="s">
         <v>1439</v>
       </c>
@@ -73364,7 +73365,7 @@
       <c r="AM667" s="1"/>
       <c r="AN667" s="83"/>
     </row>
-    <row r="668" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="668" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A668" s="22" t="s">
         <v>1441</v>
       </c>
@@ -73437,7 +73438,7 @@
       <c r="AM668" s="1"/>
       <c r="AN668" s="83"/>
     </row>
-    <row r="669" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="669" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A669" s="22" t="s">
         <v>1442</v>
       </c>
@@ -73510,7 +73511,7 @@
       <c r="AM669" s="1"/>
       <c r="AN669" s="83"/>
     </row>
-    <row r="670" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="670" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A670" s="22" t="s">
         <v>1443</v>
       </c>
@@ -73583,7 +73584,7 @@
       <c r="AM670" s="1"/>
       <c r="AN670" s="83"/>
     </row>
-    <row r="671" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="671" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A671" s="22" t="s">
         <v>1445</v>
       </c>
@@ -73656,7 +73657,7 @@
       <c r="AM671" s="1"/>
       <c r="AN671" s="83"/>
     </row>
-    <row r="672" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="672" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A672" s="22" t="s">
         <v>1447</v>
       </c>
@@ -73729,7 +73730,7 @@
       <c r="AM672" s="1"/>
       <c r="AN672" s="83"/>
     </row>
-    <row r="673" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="673" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A673" s="22" t="s">
         <v>1448</v>
       </c>
@@ -73802,7 +73803,7 @@
       <c r="AM673" s="1"/>
       <c r="AN673" s="83"/>
     </row>
-    <row r="674" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="674" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A674" s="22" t="s">
         <v>1449</v>
       </c>
@@ -73873,7 +73874,7 @@
       <c r="AM674" s="1"/>
       <c r="AN674" s="83"/>
     </row>
-    <row r="675" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="675" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A675" s="22" t="s">
         <v>1450</v>
       </c>
@@ -73946,7 +73947,7 @@
       <c r="AM675" s="1"/>
       <c r="AN675" s="83"/>
     </row>
-    <row r="676" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="676" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A676" s="22" t="s">
         <v>1451</v>
       </c>
@@ -74019,7 +74020,7 @@
       <c r="AM676" s="1"/>
       <c r="AN676" s="83"/>
     </row>
-    <row r="677" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="677" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A677" s="22" t="s">
         <v>1452</v>
       </c>
@@ -74092,7 +74093,7 @@
       <c r="AM677" s="1"/>
       <c r="AN677" s="83"/>
     </row>
-    <row r="678" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="678" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A678" s="22" t="s">
         <v>1453</v>
       </c>
@@ -74165,7 +74166,7 @@
       <c r="AM678" s="1"/>
       <c r="AN678" s="83"/>
     </row>
-    <row r="679" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="679" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A679" s="22" t="s">
         <v>1454</v>
       </c>
@@ -74238,7 +74239,7 @@
       <c r="AM679" s="1"/>
       <c r="AN679" s="83"/>
     </row>
-    <row r="680" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="680" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A680" s="22" t="s">
         <v>1455</v>
       </c>
@@ -74311,7 +74312,7 @@
       <c r="AM680" s="1"/>
       <c r="AN680" s="83"/>
     </row>
-    <row r="681" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="681" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A681" s="22" t="s">
         <v>870</v>
       </c>
@@ -74384,7 +74385,7 @@
       <c r="AM681" s="1"/>
       <c r="AN681" s="83"/>
     </row>
-    <row r="682" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="682" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A682" s="22" t="s">
         <v>1456</v>
       </c>
@@ -74457,7 +74458,7 @@
       <c r="AM682" s="1"/>
       <c r="AN682" s="83"/>
     </row>
-    <row r="683" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="683" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A683" s="22" t="s">
         <v>1457</v>
       </c>
@@ -74530,7 +74531,7 @@
       <c r="AM683" s="1"/>
       <c r="AN683" s="83"/>
     </row>
-    <row r="684" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="684" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A684" s="22" t="s">
         <v>1458</v>
       </c>
@@ -74603,7 +74604,7 @@
       <c r="AM684" s="1"/>
       <c r="AN684" s="83"/>
     </row>
-    <row r="685" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="685" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A685" s="22" t="s">
         <v>1459</v>
       </c>
@@ -74676,7 +74677,7 @@
       <c r="AM685" s="1"/>
       <c r="AN685" s="83"/>
     </row>
-    <row r="686" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="686" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A686" s="22" t="s">
         <v>1460</v>
       </c>
@@ -74749,7 +74750,7 @@
       <c r="AM686" s="1"/>
       <c r="AN686" s="83"/>
     </row>
-    <row r="687" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="687" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A687" s="22" t="s">
         <v>1461</v>
       </c>
@@ -74822,7 +74823,7 @@
       <c r="AM687" s="1"/>
       <c r="AN687" s="83"/>
     </row>
-    <row r="688" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="688" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A688" s="22" t="s">
         <v>1462</v>
       </c>
@@ -74895,7 +74896,7 @@
       <c r="AM688" s="1"/>
       <c r="AN688" s="83"/>
     </row>
-    <row r="689" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="689" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A689" s="22" t="s">
         <v>1463</v>
       </c>
@@ -74968,7 +74969,7 @@
       <c r="AM689" s="1"/>
       <c r="AN689" s="83"/>
     </row>
-    <row r="690" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="690" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A690" s="22" t="s">
         <v>1464</v>
       </c>
@@ -75041,7 +75042,7 @@
       <c r="AM690" s="1"/>
       <c r="AN690" s="83"/>
     </row>
-    <row r="691" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="691" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A691" s="22" t="s">
         <v>1465</v>
       </c>
@@ -75114,7 +75115,7 @@
       <c r="AM691" s="1"/>
       <c r="AN691" s="83"/>
     </row>
-    <row r="692" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="692" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A692" s="22" t="s">
         <v>1466</v>
       </c>
@@ -75187,7 +75188,7 @@
       <c r="AM692" s="1"/>
       <c r="AN692" s="83"/>
     </row>
-    <row r="693" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="693" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A693" s="22" t="s">
         <v>1467</v>
       </c>
@@ -75260,7 +75261,7 @@
       <c r="AM693" s="1"/>
       <c r="AN693" s="83"/>
     </row>
-    <row r="694" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="694" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A694" s="22" t="s">
         <v>1468</v>
       </c>
@@ -75333,7 +75334,7 @@
       <c r="AM694" s="1"/>
       <c r="AN694" s="83"/>
     </row>
-    <row r="695" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="695" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A695" s="22" t="s">
         <v>1469</v>
       </c>
@@ -75406,7 +75407,7 @@
       <c r="AM695" s="1"/>
       <c r="AN695" s="83"/>
     </row>
-    <row r="696" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="696" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A696" s="22" t="s">
         <v>1470</v>
       </c>
@@ -75479,7 +75480,7 @@
       <c r="AM696" s="1"/>
       <c r="AN696" s="83"/>
     </row>
-    <row r="697" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="697" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A697" s="22" t="s">
         <v>1081</v>
       </c>
@@ -75552,7 +75553,7 @@
       <c r="AM697" s="1"/>
       <c r="AN697" s="83"/>
     </row>
-    <row r="698" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="698" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A698" s="22" t="s">
         <v>1472</v>
       </c>
@@ -75625,7 +75626,7 @@
       <c r="AM698" s="1"/>
       <c r="AN698" s="83"/>
     </row>
-    <row r="699" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="699" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A699" s="22" t="s">
         <v>1473</v>
       </c>
@@ -75698,7 +75699,7 @@
       <c r="AM699" s="1"/>
       <c r="AN699" s="83"/>
     </row>
-    <row r="700" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="700" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A700" s="22" t="s">
         <v>1474</v>
       </c>
@@ -75771,7 +75772,7 @@
       <c r="AM700" s="1"/>
       <c r="AN700" s="83"/>
     </row>
-    <row r="701" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="701" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A701" s="22" t="s">
         <v>1475</v>
       </c>
@@ -75844,7 +75845,7 @@
       <c r="AM701" s="1"/>
       <c r="AN701" s="83"/>
     </row>
-    <row r="702" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="702" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A702" s="22" t="s">
         <v>1476</v>
       </c>
@@ -75917,7 +75918,7 @@
       <c r="AM702" s="1"/>
       <c r="AN702" s="83"/>
     </row>
-    <row r="703" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="703" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A703" s="22" t="s">
         <v>1477</v>
       </c>
@@ -75990,7 +75991,7 @@
       <c r="AM703" s="1"/>
       <c r="AN703" s="83"/>
     </row>
-    <row r="704" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="704" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A704" s="22" t="s">
         <v>1109</v>
       </c>
@@ -76063,7 +76064,7 @@
       <c r="AM704" s="1"/>
       <c r="AN704" s="83"/>
     </row>
-    <row r="705" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="705" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A705" s="22" t="s">
         <v>1478</v>
       </c>
@@ -76136,7 +76137,7 @@
       <c r="AM705" s="1"/>
       <c r="AN705" s="83"/>
     </row>
-    <row r="706" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="706" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A706" s="22" t="s">
         <v>1479</v>
       </c>
@@ -76209,7 +76210,7 @@
       <c r="AM706" s="1"/>
       <c r="AN706" s="83"/>
     </row>
-    <row r="707" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="707" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A707" s="22" t="s">
         <v>1480</v>
       </c>
@@ -76282,7 +76283,7 @@
       <c r="AM707" s="1"/>
       <c r="AN707" s="83"/>
     </row>
-    <row r="708" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="708" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A708" s="22" t="s">
         <v>1481</v>
       </c>
@@ -76355,7 +76356,7 @@
       <c r="AM708" s="1"/>
       <c r="AN708" s="83"/>
     </row>
-    <row r="709" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="709" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A709" s="22" t="s">
         <v>1482</v>
       </c>
@@ -76428,7 +76429,7 @@
       <c r="AM709" s="1"/>
       <c r="AN709" s="83"/>
     </row>
-    <row r="710" spans="1:40" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="710" spans="1:40" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A710" s="22" t="s">
         <v>1483</v>
       </c>
@@ -76590,7 +76591,7 @@
       <c r="AB720" s="73"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AN710" xr:uid="{2AA437EE-405D-4A43-9EB9-23F1BEB36011}"/>
+  <autoFilter ref="A2:AN711" xr:uid="{2AA437EE-405D-4A43-9EB9-23F1BEB36011}"/>
   <conditionalFormatting sqref="A193:A213 A4:A95 A97:A118">
     <cfRule type="duplicateValues" dxfId="4" priority="12"/>
   </conditionalFormatting>
@@ -77768,9 +77769,15 @@
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE495743-F761-4961-A762-7A3D120C6961}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="c06ce65c-ed18-47f4-a957-afd315448c9c"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="f5ab1930-d403-4c69-b2cd-8cc48f527d10"/>
-    <ds:schemaRef ds:uri="c06ce65c-ed18-47f4-a957-afd315448c9c"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Atualização de dados: Controle Resumo - Base BSW (31).xlsx (20/05/2026 10:38)
</commit_message>
<xml_diff>
--- a/data/dados_atuais.xlsx
+++ b/data/dados_atuais.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://delgadiadema.sharepoint.com/sites/GestoEstratgica/Documentos Compartilhados/Controle Master/BSW/Novo controle (Em processo)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2108" documentId="1_{DDE4A242-D13A-46DE-8B65-653B9F6ECEB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{168F0F45-6497-47F3-9ED0-64BF8C3F1EC5}"/>
+  <xr:revisionPtr revIDLastSave="2121" documentId="1_{DDE4A242-D13A-46DE-8B65-653B9F6ECEB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E2C8DB98-9027-4611-BF89-9C238FB9BC56}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3E398004-7492-4AA0-94C2-EA9B761AAA49}"/>
   </bookViews>
@@ -322,7 +322,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7134" uniqueCount="1504">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7139" uniqueCount="1504">
   <si>
     <t>Código
 Bobina Mâe</t>
@@ -5037,10 +5037,10 @@
     <t>Material em análise (Thiago Cardoso). Aguardando produção do produto para acompanhamento.</t>
   </si>
   <si>
-    <t>Material em análise (Izaias Claro). Aguardando produção do produto para acompanhamento.</t>
-  </si>
-  <si>
     <t>Material em análise (Edson Lupis). Aguardando produção do produto para acompanhamento.</t>
+  </si>
+  <si>
+    <t>Material em análise (Izaias Claro). Possibilidade na redução da largura da bobina / chapa.</t>
   </si>
 </sst>
 </file>
@@ -14826,7 +14826,7 @@
       </c>
       <c r="AL13" s="1"/>
       <c r="AM13" s="1" t="s">
-        <v>1503</v>
+        <v>1502</v>
       </c>
       <c r="AN13" s="83"/>
     </row>
@@ -15010,16 +15010,26 @@
         <f t="shared" si="0"/>
         <v>31.757323800000005</v>
       </c>
-      <c r="Z15" s="10"/>
+      <c r="Z15" s="10" t="s">
+        <v>50</v>
+      </c>
       <c r="AA15" s="10"/>
-      <c r="AB15" s="10"/>
-      <c r="AC15" s="10"/>
-      <c r="AD15" s="10"/>
+      <c r="AB15" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="AC15" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="AD15" s="10" t="s">
+        <v>50</v>
+      </c>
       <c r="AE15" s="10"/>
-      <c r="AF15" s="10"/>
+      <c r="AF15" s="10" t="s">
+        <v>50</v>
+      </c>
       <c r="AG15" s="38">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="AH15" s="51" t="str">
         <f t="shared" si="2"/>
@@ -15036,7 +15046,7 @@
       </c>
       <c r="AL15" s="1"/>
       <c r="AM15" s="1" t="s">
-        <v>1502</v>
+        <v>1503</v>
       </c>
       <c r="AN15" s="83"/>
     </row>

</xml_diff>

<commit_message>
Atualização de dados: Controle Resumo - Base BSW (36).xlsx (26/05/2026 20:52)
</commit_message>
<xml_diff>
--- a/data/dados_atuais.xlsx
+++ b/data/dados_atuais.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr codeName="EsteLivro"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr codeName="EsteLivro" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://delgadiadema.sharepoint.com/sites/GestoEstratgica/Documentos Compartilhados/Controle Master/BSW/Novo controle (Em processo)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2228" documentId="1_{DDE4A242-D13A-46DE-8B65-653B9F6ECEB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5CA87258-A579-4031-A157-959517B13604}"/>
+  <xr:revisionPtr revIDLastSave="2234" documentId="1_{DDE4A242-D13A-46DE-8B65-653B9F6ECEB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E07EDBF8-507D-4903-B295-279546C99279}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3E398004-7492-4AA0-94C2-EA9B761AAA49}"/>
   </bookViews>
@@ -321,7 +321,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7181" uniqueCount="1515">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7185" uniqueCount="1515">
   <si>
     <t>Código
 Bobina Mâe</t>
@@ -13119,10 +13119,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/namedSheetViews/namedSheetView1.xml><?xml version="1.0" encoding="utf-8"?>
-<namedSheetViews xmlns="http://schemas.microsoft.com/office/spreadsheetml/2019/namedsheetviews" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14"/>
-</file>
-
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <person displayName="Eric da Silva Maia" id="{D9E3AE94-B136-43DC-991E-9F5A8D1687A6}" userId="S::eric.maia@delga.com.br::43e774bf-1d7b-4030-aa96-fdc0a837fc3b" providerId="AD"/>
@@ -13634,7 +13630,7 @@
         <v>1513</v>
       </c>
     </row>
-    <row r="3" spans="1:41" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:41" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
         <v>40</v>
       </c>
@@ -13750,7 +13746,7 @@
       <c r="AN3" s="82"/>
       <c r="AO3" s="82"/>
     </row>
-    <row r="4" spans="1:41" s="26" customFormat="1" ht="132.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:41" s="26" customFormat="1" ht="132.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
         <v>52</v>
       </c>
@@ -13870,7 +13866,7 @@
         <v>1514</v>
       </c>
     </row>
-    <row r="5" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
         <v>62</v>
       </c>
@@ -13990,7 +13986,7 @@
         <v>1514</v>
       </c>
     </row>
-    <row r="6" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
         <v>69</v>
       </c>
@@ -14100,7 +14096,7 @@
       <c r="AN6" s="82"/>
       <c r="AO6" s="82"/>
     </row>
-    <row r="7" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
         <v>77</v>
       </c>
@@ -14216,7 +14212,7 @@
       <c r="AN7" s="82"/>
       <c r="AO7" s="82"/>
     </row>
-    <row r="8" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
         <v>84</v>
       </c>
@@ -14330,7 +14326,7 @@
       <c r="AN8" s="82"/>
       <c r="AO8" s="82"/>
     </row>
-    <row r="9" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
         <v>89</v>
       </c>
@@ -14450,7 +14446,7 @@
         <v>1514</v>
       </c>
     </row>
-    <row r="10" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>96</v>
       </c>
@@ -14570,7 +14566,7 @@
         <v>1514</v>
       </c>
     </row>
-    <row r="11" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
         <v>102</v>
       </c>
@@ -14688,7 +14684,7 @@
       </c>
       <c r="AO11" s="82"/>
     </row>
-    <row r="12" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
         <v>107</v>
       </c>
@@ -14804,7 +14800,7 @@
       </c>
       <c r="AO12" s="82"/>
     </row>
-    <row r="13" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
         <v>110</v>
       </c>
@@ -14903,7 +14899,7 @@
       <c r="AN13" s="82"/>
       <c r="AO13" s="82"/>
     </row>
-    <row r="14" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
         <v>114</v>
       </c>
@@ -15017,7 +15013,7 @@
       </c>
       <c r="AO14" s="82"/>
     </row>
-    <row r="15" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
         <v>117</v>
       </c>
@@ -15127,7 +15123,7 @@
       <c r="AN15" s="82"/>
       <c r="AO15" s="82"/>
     </row>
-    <row r="16" spans="1:41" s="26" customFormat="1" ht="30.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:41" s="26" customFormat="1" ht="30.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
         <v>121</v>
       </c>
@@ -15245,7 +15241,7 @@
       </c>
       <c r="AO16" s="82"/>
     </row>
-    <row r="17" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
         <v>126</v>
       </c>
@@ -15345,7 +15341,7 @@
       <c r="AN17" s="82"/>
       <c r="AO17" s="82"/>
     </row>
-    <row r="18" spans="1:41" s="26" customFormat="1" ht="51" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:41" s="26" customFormat="1" ht="51" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
         <v>131</v>
       </c>
@@ -15453,7 +15449,7 @@
       <c r="AN18" s="82"/>
       <c r="AO18" s="82"/>
     </row>
-    <row r="19" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
         <v>136</v>
       </c>
@@ -15569,7 +15565,7 @@
       </c>
       <c r="AO19" s="82"/>
     </row>
-    <row r="20" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
         <v>141</v>
       </c>
@@ -15669,7 +15665,7 @@
       <c r="AN20" s="82"/>
       <c r="AO20" s="82"/>
     </row>
-    <row r="21" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
         <v>146</v>
       </c>
@@ -15787,7 +15783,7 @@
       </c>
       <c r="AO21" s="82"/>
     </row>
-    <row r="22" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
         <v>153</v>
       </c>
@@ -15887,7 +15883,7 @@
       <c r="AN22" s="82"/>
       <c r="AO22" s="82"/>
     </row>
-    <row r="23" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
         <v>155</v>
       </c>
@@ -16003,7 +15999,7 @@
       </c>
       <c r="AO23" s="82"/>
     </row>
-    <row r="24" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="22" t="s">
         <v>159</v>
       </c>
@@ -16101,7 +16097,7 @@
       <c r="AN24" s="82"/>
       <c r="AO24" s="82"/>
     </row>
-    <row r="25" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="22" t="s">
         <v>160</v>
       </c>
@@ -16199,7 +16195,7 @@
       <c r="AN25" s="82"/>
       <c r="AO25" s="82"/>
     </row>
-    <row r="26" spans="1:41" s="26" customFormat="1" ht="30.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:41" s="26" customFormat="1" ht="30.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="22" t="s">
         <v>162</v>
       </c>
@@ -16295,7 +16291,7 @@
       <c r="AN26" s="82"/>
       <c r="AO26" s="82"/>
     </row>
-    <row r="27" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="22" t="s">
         <v>165</v>
       </c>
@@ -16393,7 +16389,7 @@
       <c r="AN27" s="82"/>
       <c r="AO27" s="82"/>
     </row>
-    <row r="28" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="22" t="s">
         <v>168</v>
       </c>
@@ -16509,7 +16505,7 @@
       <c r="AN28" s="82"/>
       <c r="AO28" s="82"/>
     </row>
-    <row r="29" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="22" t="s">
         <v>171</v>
       </c>
@@ -16607,7 +16603,7 @@
       <c r="AN29" s="82"/>
       <c r="AO29" s="82"/>
     </row>
-    <row r="30" spans="1:41" s="26" customFormat="1" ht="30.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:41" s="26" customFormat="1" ht="30.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="22" t="s">
         <v>174</v>
       </c>
@@ -16705,7 +16701,7 @@
       <c r="AN30" s="82"/>
       <c r="AO30" s="82"/>
     </row>
-    <row r="31" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="22" t="s">
         <v>178</v>
       </c>
@@ -16797,7 +16793,7 @@
       <c r="AN31" s="82"/>
       <c r="AO31" s="82"/>
     </row>
-    <row r="32" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="22" t="s">
         <v>180</v>
       </c>
@@ -16915,7 +16911,7 @@
       </c>
       <c r="AO32" s="82"/>
     </row>
-    <row r="33" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="22" t="s">
         <v>183</v>
       </c>
@@ -17031,7 +17027,7 @@
       </c>
       <c r="AO33" s="82"/>
     </row>
-    <row r="34" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="22" t="s">
         <v>189</v>
       </c>
@@ -17125,7 +17121,7 @@
       <c r="AN34" s="82"/>
       <c r="AO34" s="82"/>
     </row>
-    <row r="35" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="22" t="s">
         <v>193</v>
       </c>
@@ -17243,7 +17239,7 @@
       </c>
       <c r="AO35" s="82"/>
     </row>
-    <row r="36" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="22" t="s">
         <v>199</v>
       </c>
@@ -17339,7 +17335,7 @@
       <c r="AN36" s="82"/>
       <c r="AO36" s="82"/>
     </row>
-    <row r="37" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="22" t="s">
         <v>200</v>
       </c>
@@ -17427,7 +17423,7 @@
       <c r="AN37" s="82"/>
       <c r="AO37" s="82"/>
     </row>
-    <row r="38" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="22" t="s">
         <v>203</v>
       </c>
@@ -17529,7 +17525,7 @@
       <c r="AN38" s="82"/>
       <c r="AO38" s="82"/>
     </row>
-    <row r="39" spans="1:41" s="26" customFormat="1" ht="71.400000000000006" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:41" s="26" customFormat="1" ht="71.400000000000006" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" s="22" t="s">
         <v>206</v>
       </c>
@@ -17649,7 +17645,7 @@
       </c>
       <c r="AO39" s="82"/>
     </row>
-    <row r="40" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="22" t="s">
         <v>210</v>
       </c>
@@ -17743,7 +17739,7 @@
       <c r="AN40" s="82"/>
       <c r="AO40" s="82"/>
     </row>
-    <row r="41" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="22" t="s">
         <v>213</v>
       </c>
@@ -17837,7 +17833,7 @@
       <c r="AN41" s="82"/>
       <c r="AO41" s="82"/>
     </row>
-    <row r="42" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="22" t="s">
         <v>216</v>
       </c>
@@ -17931,7 +17927,7 @@
       <c r="AN42" s="82"/>
       <c r="AO42" s="82"/>
     </row>
-    <row r="43" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="22" t="s">
         <v>220</v>
       </c>
@@ -18025,7 +18021,7 @@
       <c r="AN43" s="82"/>
       <c r="AO43" s="82"/>
     </row>
-    <row r="44" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="22" t="s">
         <v>224</v>
       </c>
@@ -18143,7 +18139,7 @@
       </c>
       <c r="AO44" s="82"/>
     </row>
-    <row r="45" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="22" t="s">
         <v>229</v>
       </c>
@@ -18257,7 +18253,7 @@
       </c>
       <c r="AO45" s="82"/>
     </row>
-    <row r="46" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="22" t="s">
         <v>233</v>
       </c>
@@ -18351,7 +18347,7 @@
       <c r="AN46" s="82"/>
       <c r="AO46" s="82"/>
     </row>
-    <row r="47" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="22" t="s">
         <v>240</v>
       </c>
@@ -18445,7 +18441,7 @@
       <c r="AN47" s="82"/>
       <c r="AO47" s="82"/>
     </row>
-    <row r="48" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="22" t="s">
         <v>243</v>
       </c>
@@ -18539,7 +18535,7 @@
       <c r="AN48" s="82"/>
       <c r="AO48" s="82"/>
     </row>
-    <row r="49" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="22" t="s">
         <v>245</v>
       </c>
@@ -18633,7 +18629,7 @@
       <c r="AN49" s="82"/>
       <c r="AO49" s="82"/>
     </row>
-    <row r="50" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="22" t="s">
         <v>247</v>
       </c>
@@ -18727,7 +18723,7 @@
       <c r="AN50" s="82"/>
       <c r="AO50" s="82"/>
     </row>
-    <row r="51" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="22" t="s">
         <v>250</v>
       </c>
@@ -18821,7 +18817,7 @@
       <c r="AN51" s="82"/>
       <c r="AO51" s="82"/>
     </row>
-    <row r="52" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="22" t="s">
         <v>253</v>
       </c>
@@ -18915,7 +18911,7 @@
       <c r="AN52" s="82"/>
       <c r="AO52" s="82"/>
     </row>
-    <row r="53" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="22" t="s">
         <v>256</v>
       </c>
@@ -19009,7 +19005,7 @@
       <c r="AN53" s="82"/>
       <c r="AO53" s="82"/>
     </row>
-    <row r="54" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="22" t="s">
         <v>258</v>
       </c>
@@ -19103,7 +19099,7 @@
       <c r="AN54" s="82"/>
       <c r="AO54" s="82"/>
     </row>
-    <row r="55" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="22" t="s">
         <v>262</v>
       </c>
@@ -19197,7 +19193,7 @@
       <c r="AN55" s="82"/>
       <c r="AO55" s="82"/>
     </row>
-    <row r="56" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="22" t="s">
         <v>265</v>
       </c>
@@ -19315,7 +19311,7 @@
       </c>
       <c r="AO56" s="82"/>
     </row>
-    <row r="57" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="22" t="s">
         <v>269</v>
       </c>
@@ -19409,7 +19405,7 @@
       <c r="AN57" s="82"/>
       <c r="AO57" s="82"/>
     </row>
-    <row r="58" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="22" t="s">
         <v>270</v>
       </c>
@@ -19503,7 +19499,7 @@
       <c r="AN58" s="82"/>
       <c r="AO58" s="82"/>
     </row>
-    <row r="59" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="22" t="s">
         <v>272</v>
       </c>
@@ -19597,7 +19593,7 @@
       <c r="AN59" s="82"/>
       <c r="AO59" s="82"/>
     </row>
-    <row r="60" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="22" t="s">
         <v>274</v>
       </c>
@@ -19709,7 +19705,7 @@
       <c r="AN60" s="82"/>
       <c r="AO60" s="82"/>
     </row>
-    <row r="61" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="22" t="s">
         <v>280</v>
       </c>
@@ -19823,7 +19819,7 @@
       </c>
       <c r="AO61" s="82"/>
     </row>
-    <row r="62" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="22" t="s">
         <v>286</v>
       </c>
@@ -19917,7 +19913,7 @@
       <c r="AN62" s="82"/>
       <c r="AO62" s="82"/>
     </row>
-    <row r="63" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="22" t="s">
         <v>288</v>
       </c>
@@ -20011,7 +20007,7 @@
       <c r="AN63" s="82"/>
       <c r="AO63" s="82"/>
     </row>
-    <row r="64" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="22" t="s">
         <v>291</v>
       </c>
@@ -20105,7 +20101,7 @@
       <c r="AN64" s="82"/>
       <c r="AO64" s="82"/>
     </row>
-    <row r="65" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" s="22" t="s">
         <v>293</v>
       </c>
@@ -20201,7 +20197,7 @@
       <c r="AN65" s="82"/>
       <c r="AO65" s="82"/>
     </row>
-    <row r="66" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="22" t="s">
         <v>295</v>
       </c>
@@ -20297,7 +20293,7 @@
       <c r="AN66" s="82"/>
       <c r="AO66" s="82"/>
     </row>
-    <row r="67" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="22" t="s">
         <v>297</v>
       </c>
@@ -20387,7 +20383,7 @@
       <c r="AN67" s="82"/>
       <c r="AO67" s="82"/>
     </row>
-    <row r="68" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="22" t="s">
         <v>298</v>
       </c>
@@ -20481,7 +20477,7 @@
       <c r="AN68" s="82"/>
       <c r="AO68" s="82"/>
     </row>
-    <row r="69" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="22" t="s">
         <v>300</v>
       </c>
@@ -20577,7 +20573,7 @@
       <c r="AN69" s="82"/>
       <c r="AO69" s="82"/>
     </row>
-    <row r="70" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="22" t="s">
         <v>303</v>
       </c>
@@ -20671,7 +20667,7 @@
       <c r="AN70" s="82"/>
       <c r="AO70" s="82"/>
     </row>
-    <row r="71" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="22" t="s">
         <v>305</v>
       </c>
@@ -20765,7 +20761,7 @@
       <c r="AN71" s="82"/>
       <c r="AO71" s="82"/>
     </row>
-    <row r="72" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="22" t="s">
         <v>308</v>
       </c>
@@ -20861,7 +20857,7 @@
       <c r="AN72" s="82"/>
       <c r="AO72" s="82"/>
     </row>
-    <row r="73" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="22" t="s">
         <v>311</v>
       </c>
@@ -20955,7 +20951,7 @@
       <c r="AN73" s="82"/>
       <c r="AO73" s="82"/>
     </row>
-    <row r="74" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" s="22" t="s">
         <v>313</v>
       </c>
@@ -21049,7 +21045,7 @@
       <c r="AN74" s="82"/>
       <c r="AO74" s="82"/>
     </row>
-    <row r="75" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" s="22" t="s">
         <v>315</v>
       </c>
@@ -21141,7 +21137,7 @@
       <c r="AN75" s="82"/>
       <c r="AO75" s="82"/>
     </row>
-    <row r="76" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" s="22" t="s">
         <v>318</v>
       </c>
@@ -21235,7 +21231,7 @@
       <c r="AN76" s="82"/>
       <c r="AO76" s="82"/>
     </row>
-    <row r="77" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" s="22" t="s">
         <v>322</v>
       </c>
@@ -21327,7 +21323,7 @@
       <c r="AN77" s="82"/>
       <c r="AO77" s="82"/>
     </row>
-    <row r="78" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" s="22" t="s">
         <v>324</v>
       </c>
@@ -21441,7 +21437,7 @@
       </c>
       <c r="AO78" s="82"/>
     </row>
-    <row r="79" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" s="22" t="s">
         <v>328</v>
       </c>
@@ -21535,7 +21531,7 @@
       <c r="AN79" s="82"/>
       <c r="AO79" s="82"/>
     </row>
-    <row r="80" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" s="22" t="s">
         <v>331</v>
       </c>
@@ -21649,7 +21645,7 @@
       </c>
       <c r="AO80" s="82"/>
     </row>
-    <row r="81" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="22" t="s">
         <v>335</v>
       </c>
@@ -21745,7 +21741,7 @@
       <c r="AN81" s="82"/>
       <c r="AO81" s="82"/>
     </row>
-    <row r="82" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" s="22" t="s">
         <v>337</v>
       </c>
@@ -21839,7 +21835,7 @@
       <c r="AN82" s="82"/>
       <c r="AO82" s="82"/>
     </row>
-    <row r="83" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" s="22" t="s">
         <v>339</v>
       </c>
@@ -21933,7 +21929,7 @@
       <c r="AN83" s="82"/>
       <c r="AO83" s="82"/>
     </row>
-    <row r="84" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" s="22" t="s">
         <v>341</v>
       </c>
@@ -22029,7 +22025,7 @@
       <c r="AN84" s="82"/>
       <c r="AO84" s="82"/>
     </row>
-    <row r="85" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" s="22" t="s">
         <v>344</v>
       </c>
@@ -22123,7 +22119,7 @@
       <c r="AN85" s="82"/>
       <c r="AO85" s="82"/>
     </row>
-    <row r="86" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" s="22" t="s">
         <v>346</v>
       </c>
@@ -22213,7 +22209,7 @@
       <c r="AN86" s="82"/>
       <c r="AO86" s="82"/>
     </row>
-    <row r="87" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" s="22" t="s">
         <v>351</v>
       </c>
@@ -22307,7 +22303,7 @@
       <c r="AN87" s="82"/>
       <c r="AO87" s="82"/>
     </row>
-    <row r="88" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" s="22" t="s">
         <v>353</v>
       </c>
@@ -22403,7 +22399,7 @@
       <c r="AN88" s="82"/>
       <c r="AO88" s="82"/>
     </row>
-    <row r="89" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" s="22" t="s">
         <v>358</v>
       </c>
@@ -22497,7 +22493,7 @@
       <c r="AN89" s="82"/>
       <c r="AO89" s="82"/>
     </row>
-    <row r="90" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" s="22" t="s">
         <v>361</v>
       </c>
@@ -22591,7 +22587,7 @@
       <c r="AN90" s="82"/>
       <c r="AO90" s="82"/>
     </row>
-    <row r="91" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" s="22" t="s">
         <v>363</v>
       </c>
@@ -22685,7 +22681,7 @@
       <c r="AN91" s="82"/>
       <c r="AO91" s="82"/>
     </row>
-    <row r="92" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" s="22" t="s">
         <v>366</v>
       </c>
@@ -22779,7 +22775,7 @@
       <c r="AN92" s="82"/>
       <c r="AO92" s="82"/>
     </row>
-    <row r="93" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" s="22" t="s">
         <v>369</v>
       </c>
@@ -22871,7 +22867,7 @@
       <c r="AN93" s="82"/>
       <c r="AO93" s="82"/>
     </row>
-    <row r="94" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" s="22" t="s">
         <v>371</v>
       </c>
@@ -22965,7 +22961,7 @@
       <c r="AN94" s="82"/>
       <c r="AO94" s="82"/>
     </row>
-    <row r="95" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" s="15" t="s">
         <v>374</v>
       </c>
@@ -23059,7 +23055,7 @@
       <c r="AN95" s="82"/>
       <c r="AO95" s="82"/>
     </row>
-    <row r="96" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" s="22" t="s">
         <v>377</v>
       </c>
@@ -23173,7 +23169,7 @@
       </c>
       <c r="AO96" s="82"/>
     </row>
-    <row r="97" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" s="22" t="s">
         <v>380</v>
       </c>
@@ -23261,7 +23257,7 @@
       <c r="AN97" s="82"/>
       <c r="AO97" s="82"/>
     </row>
-    <row r="98" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" s="3" t="s">
         <v>381</v>
       </c>
@@ -23357,7 +23353,7 @@
       <c r="AN98" s="82"/>
       <c r="AO98" s="82"/>
     </row>
-    <row r="99" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" s="22" t="s">
         <v>385</v>
       </c>
@@ -23453,7 +23449,7 @@
       <c r="AN99" s="82"/>
       <c r="AO99" s="82"/>
     </row>
-    <row r="100" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" s="22" t="s">
         <v>387</v>
       </c>
@@ -23547,7 +23543,7 @@
       <c r="AN100" s="82"/>
       <c r="AO100" s="82"/>
     </row>
-    <row r="101" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" s="22" t="s">
         <v>390</v>
       </c>
@@ -23641,7 +23637,7 @@
       <c r="AN101" s="82"/>
       <c r="AO101" s="82"/>
     </row>
-    <row r="102" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" s="22" t="s">
         <v>393</v>
       </c>
@@ -23731,7 +23727,7 @@
       <c r="AN102" s="82"/>
       <c r="AO102" s="82"/>
     </row>
-    <row r="103" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" s="22" t="s">
         <v>396</v>
       </c>
@@ -23825,7 +23821,7 @@
       <c r="AN103" s="82"/>
       <c r="AO103" s="82"/>
     </row>
-    <row r="104" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" s="22" t="s">
         <v>397</v>
       </c>
@@ -23921,7 +23917,7 @@
       <c r="AN104" s="82"/>
       <c r="AO104" s="82"/>
     </row>
-    <row r="105" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="22" t="s">
         <v>399</v>
       </c>
@@ -24009,7 +24005,7 @@
       <c r="AN105" s="82"/>
       <c r="AO105" s="82"/>
     </row>
-    <row r="106" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" s="22" t="s">
         <v>401</v>
       </c>
@@ -24103,7 +24099,7 @@
       <c r="AN106" s="82"/>
       <c r="AO106" s="82"/>
     </row>
-    <row r="107" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" s="15" t="s">
         <v>403</v>
       </c>
@@ -24191,7 +24187,7 @@
       <c r="AN107" s="82"/>
       <c r="AO107" s="82"/>
     </row>
-    <row r="108" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" s="22" t="s">
         <v>405</v>
       </c>
@@ -24283,7 +24279,7 @@
       <c r="AN108" s="82"/>
       <c r="AO108" s="82"/>
     </row>
-    <row r="109" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" s="22" t="s">
         <v>407</v>
       </c>
@@ -24377,7 +24373,7 @@
       <c r="AN109" s="82"/>
       <c r="AO109" s="82"/>
     </row>
-    <row r="110" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" s="22" t="s">
         <v>409</v>
       </c>
@@ -24493,7 +24489,7 @@
       <c r="AN110" s="82"/>
       <c r="AO110" s="82"/>
     </row>
-    <row r="111" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" s="22" t="s">
         <v>413</v>
       </c>
@@ -24589,7 +24585,7 @@
       <c r="AN111" s="82"/>
       <c r="AO111" s="82"/>
     </row>
-    <row r="112" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" s="22" t="s">
         <v>415</v>
       </c>
@@ -24705,7 +24701,7 @@
       </c>
       <c r="AO112" s="82"/>
     </row>
-    <row r="113" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" s="22" t="s">
         <v>418</v>
       </c>
@@ -24795,7 +24791,7 @@
       <c r="AN113" s="82"/>
       <c r="AO113" s="82"/>
     </row>
-    <row r="114" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" s="22" t="s">
         <v>422</v>
       </c>
@@ -24883,7 +24879,7 @@
       <c r="AN114" s="82"/>
       <c r="AO114" s="82"/>
     </row>
-    <row r="115" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" s="3" t="s">
         <v>423</v>
       </c>
@@ -24977,7 +24973,7 @@
       <c r="AN115" s="82"/>
       <c r="AO115" s="82"/>
     </row>
-    <row r="116" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" s="22" t="s">
         <v>425</v>
       </c>
@@ -25063,7 +25059,7 @@
       <c r="AN116" s="82"/>
       <c r="AO116" s="82"/>
     </row>
-    <row r="117" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" s="22" t="s">
         <v>427</v>
       </c>
@@ -25159,7 +25155,7 @@
       <c r="AN117" s="82"/>
       <c r="AO117" s="82"/>
     </row>
-    <row r="118" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" s="22" t="s">
         <v>429</v>
       </c>
@@ -25253,7 +25249,7 @@
       <c r="AN118" s="82"/>
       <c r="AO118" s="82"/>
     </row>
-    <row r="119" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" s="22" t="s">
         <v>431</v>
       </c>
@@ -25345,7 +25341,7 @@
       <c r="AN119" s="82"/>
       <c r="AO119" s="82"/>
     </row>
-    <row r="120" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" s="15" t="s">
         <v>433</v>
       </c>
@@ -25431,7 +25427,7 @@
       <c r="AN120" s="82"/>
       <c r="AO120" s="82"/>
     </row>
-    <row r="121" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" s="22" t="s">
         <v>434</v>
       </c>
@@ -25523,7 +25519,7 @@
       <c r="AN121" s="82"/>
       <c r="AO121" s="82"/>
     </row>
-    <row r="122" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" s="15" t="s">
         <v>436</v>
       </c>
@@ -25611,7 +25607,7 @@
       <c r="AN122" s="82"/>
       <c r="AO122" s="82"/>
     </row>
-    <row r="123" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" s="22" t="s">
         <v>437</v>
       </c>
@@ -25723,7 +25719,7 @@
       </c>
       <c r="AO123" s="82"/>
     </row>
-    <row r="124" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" s="22" t="s">
         <v>439</v>
       </c>
@@ -25809,7 +25805,7 @@
       <c r="AN124" s="82"/>
       <c r="AO124" s="82"/>
     </row>
-    <row r="125" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" s="22" t="s">
         <v>440</v>
       </c>
@@ -25905,7 +25901,7 @@
       <c r="AN125" s="82"/>
       <c r="AO125" s="82"/>
     </row>
-    <row r="126" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" s="22" t="s">
         <v>442</v>
       </c>
@@ -25995,7 +25991,7 @@
       <c r="AN126" s="82"/>
       <c r="AO126" s="82"/>
     </row>
-    <row r="127" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" s="22" t="s">
         <v>445</v>
       </c>
@@ -26089,7 +26085,7 @@
       <c r="AN127" s="82"/>
       <c r="AO127" s="82"/>
     </row>
-    <row r="128" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" s="22" t="s">
         <v>447</v>
       </c>
@@ -26179,7 +26175,7 @@
       <c r="AN128" s="82"/>
       <c r="AO128" s="82"/>
     </row>
-    <row r="129" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" s="15" t="s">
         <v>450</v>
       </c>
@@ -26273,7 +26269,7 @@
       <c r="AN129" s="82"/>
       <c r="AO129" s="82"/>
     </row>
-    <row r="130" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" s="22" t="s">
         <v>452</v>
       </c>
@@ -26357,7 +26353,7 @@
       <c r="AN130" s="82"/>
       <c r="AO130" s="82"/>
     </row>
-    <row r="131" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" s="22" t="s">
         <v>453</v>
       </c>
@@ -26441,7 +26437,7 @@
       <c r="AN131" s="82"/>
       <c r="AO131" s="82"/>
     </row>
-    <row r="132" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" s="22" t="s">
         <v>454</v>
       </c>
@@ -26535,7 +26531,7 @@
       <c r="AN132" s="82"/>
       <c r="AO132" s="82"/>
     </row>
-    <row r="133" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" s="22" t="s">
         <v>456</v>
       </c>
@@ -26631,7 +26627,7 @@
       <c r="AN133" s="82"/>
       <c r="AO133" s="82"/>
     </row>
-    <row r="134" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" s="22" t="s">
         <v>458</v>
       </c>
@@ -26723,7 +26719,7 @@
       <c r="AN134" s="82"/>
       <c r="AO134" s="82"/>
     </row>
-    <row r="135" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" s="15" t="s">
         <v>460</v>
       </c>
@@ -26813,7 +26809,7 @@
       <c r="AN135" s="82"/>
       <c r="AO135" s="82"/>
     </row>
-    <row r="136" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" s="22" t="s">
         <v>462</v>
       </c>
@@ -26905,7 +26901,7 @@
       <c r="AN136" s="82"/>
       <c r="AO136" s="82"/>
     </row>
-    <row r="137" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" s="15" t="s">
         <v>464</v>
       </c>
@@ -26991,7 +26987,7 @@
       <c r="AN137" s="82"/>
       <c r="AO137" s="82"/>
     </row>
-    <row r="138" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" s="22" t="s">
         <v>466</v>
       </c>
@@ -27083,7 +27079,7 @@
       <c r="AN138" s="82"/>
       <c r="AO138" s="82"/>
     </row>
-    <row r="139" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" s="15" t="s">
         <v>467</v>
       </c>
@@ -27171,7 +27167,7 @@
       <c r="AN139" s="82"/>
       <c r="AO139" s="82"/>
     </row>
-    <row r="140" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" s="22" t="s">
         <v>470</v>
       </c>
@@ -27263,7 +27259,7 @@
       <c r="AN140" s="82"/>
       <c r="AO140" s="82"/>
     </row>
-    <row r="141" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" s="22" t="s">
         <v>473</v>
       </c>
@@ -27349,7 +27345,7 @@
       <c r="AN141" s="82"/>
       <c r="AO141" s="82"/>
     </row>
-    <row r="142" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" s="15" t="s">
         <v>474</v>
       </c>
@@ -27441,7 +27437,7 @@
       <c r="AN142" s="82"/>
       <c r="AO142" s="82"/>
     </row>
-    <row r="143" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" s="15" t="s">
         <v>476</v>
       </c>
@@ -27529,7 +27525,7 @@
       <c r="AN143" s="82"/>
       <c r="AO143" s="82"/>
     </row>
-    <row r="144" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" s="15" t="s">
         <v>479</v>
       </c>
@@ -27625,7 +27621,7 @@
       <c r="AN144" s="82"/>
       <c r="AO144" s="82"/>
     </row>
-    <row r="145" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" s="15" t="s">
         <v>481</v>
       </c>
@@ -27713,7 +27709,7 @@
       <c r="AN145" s="82"/>
       <c r="AO145" s="82"/>
     </row>
-    <row r="146" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" s="15" t="s">
         <v>482</v>
       </c>
@@ -27799,7 +27795,7 @@
       <c r="AN146" s="82"/>
       <c r="AO146" s="82"/>
     </row>
-    <row r="147" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" s="15" t="s">
         <v>483</v>
       </c>
@@ -27881,7 +27877,7 @@
       <c r="AN147" s="82"/>
       <c r="AO147" s="82"/>
     </row>
-    <row r="148" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" s="15" t="s">
         <v>484</v>
       </c>
@@ -27975,7 +27971,7 @@
       <c r="AN148" s="82"/>
       <c r="AO148" s="82"/>
     </row>
-    <row r="149" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" s="15" t="s">
         <v>486</v>
       </c>
@@ -28067,7 +28063,7 @@
       <c r="AN149" s="82"/>
       <c r="AO149" s="82"/>
     </row>
-    <row r="150" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" s="15" t="s">
         <v>488</v>
       </c>
@@ -28149,7 +28145,7 @@
       <c r="AN150" s="82"/>
       <c r="AO150" s="82"/>
     </row>
-    <row r="151" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" s="15" t="s">
         <v>489</v>
       </c>
@@ -28237,7 +28233,7 @@
       <c r="AN151" s="82"/>
       <c r="AO151" s="82"/>
     </row>
-    <row r="152" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" s="15" t="s">
         <v>491</v>
       </c>
@@ -28329,7 +28325,7 @@
       <c r="AN152" s="82"/>
       <c r="AO152" s="82"/>
     </row>
-    <row r="153" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" s="15" t="s">
         <v>494</v>
       </c>
@@ -28417,7 +28413,7 @@
       <c r="AN153" s="82"/>
       <c r="AO153" s="82"/>
     </row>
-    <row r="154" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" s="15" t="s">
         <v>496</v>
       </c>
@@ -28505,7 +28501,7 @@
       <c r="AN154" s="82"/>
       <c r="AO154" s="82"/>
     </row>
-    <row r="155" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" s="15" t="s">
         <v>498</v>
       </c>
@@ -28593,7 +28589,7 @@
       <c r="AN155" s="82"/>
       <c r="AO155" s="82"/>
     </row>
-    <row r="156" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" s="15" t="s">
         <v>500</v>
       </c>
@@ -28683,7 +28679,7 @@
       <c r="AN156" s="82"/>
       <c r="AO156" s="82"/>
     </row>
-    <row r="157" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" s="15" t="s">
         <v>503</v>
       </c>
@@ -28771,7 +28767,7 @@
       <c r="AN157" s="82"/>
       <c r="AO157" s="82"/>
     </row>
-    <row r="158" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" s="15" t="s">
         <v>505</v>
       </c>
@@ -28859,7 +28855,7 @@
       <c r="AN158" s="82"/>
       <c r="AO158" s="82"/>
     </row>
-    <row r="159" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" s="15" t="s">
         <v>507</v>
       </c>
@@ -28949,7 +28945,7 @@
       <c r="AN159" s="82"/>
       <c r="AO159" s="82"/>
     </row>
-    <row r="160" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" s="15" t="s">
         <v>509</v>
       </c>
@@ -29037,7 +29033,7 @@
       <c r="AN160" s="82"/>
       <c r="AO160" s="82"/>
     </row>
-    <row r="161" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" s="15" t="s">
         <v>511</v>
       </c>
@@ -29125,7 +29121,7 @@
       <c r="AN161" s="82"/>
       <c r="AO161" s="82"/>
     </row>
-    <row r="162" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" s="15" t="s">
         <v>513</v>
       </c>
@@ -29217,7 +29213,7 @@
       <c r="AN162" s="82"/>
       <c r="AO162" s="82"/>
     </row>
-    <row r="163" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" s="15" t="s">
         <v>516</v>
       </c>
@@ -29305,7 +29301,7 @@
       <c r="AN163" s="82"/>
       <c r="AO163" s="82"/>
     </row>
-    <row r="164" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" s="15" t="s">
         <v>518</v>
       </c>
@@ -29393,7 +29389,7 @@
       <c r="AN164" s="82"/>
       <c r="AO164" s="82"/>
     </row>
-    <row r="165" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" s="15" t="s">
         <v>520</v>
       </c>
@@ -29483,7 +29479,7 @@
       <c r="AN165" s="82"/>
       <c r="AO165" s="82"/>
     </row>
-    <row r="166" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" s="15" t="s">
         <v>522</v>
       </c>
@@ -29573,7 +29569,7 @@
       <c r="AN166" s="82"/>
       <c r="AO166" s="82"/>
     </row>
-    <row r="167" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" s="15" t="s">
         <v>524</v>
       </c>
@@ -29663,7 +29659,7 @@
       <c r="AN167" s="82"/>
       <c r="AO167" s="82"/>
     </row>
-    <row r="168" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" s="15" t="s">
         <v>526</v>
       </c>
@@ -29753,7 +29749,7 @@
       <c r="AN168" s="82"/>
       <c r="AO168" s="82"/>
     </row>
-    <row r="169" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" s="15" t="s">
         <v>528</v>
       </c>
@@ -29841,7 +29837,7 @@
       <c r="AN169" s="82"/>
       <c r="AO169" s="82"/>
     </row>
-    <row r="170" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" s="15" t="s">
         <v>530</v>
       </c>
@@ -29931,7 +29927,7 @@
       <c r="AN170" s="82"/>
       <c r="AO170" s="82"/>
     </row>
-    <row r="171" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" s="15" t="s">
         <v>532</v>
       </c>
@@ -30021,7 +30017,7 @@
       <c r="AN171" s="82"/>
       <c r="AO171" s="82"/>
     </row>
-    <row r="172" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" s="15" t="s">
         <v>534</v>
       </c>
@@ -30109,7 +30105,7 @@
       <c r="AN172" s="82"/>
       <c r="AO172" s="82"/>
     </row>
-    <row r="173" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" s="15" t="s">
         <v>536</v>
       </c>
@@ -30199,7 +30195,7 @@
       <c r="AN173" s="82"/>
       <c r="AO173" s="82"/>
     </row>
-    <row r="174" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" s="15" t="s">
         <v>538</v>
       </c>
@@ -30289,7 +30285,7 @@
       <c r="AN174" s="82"/>
       <c r="AO174" s="82"/>
     </row>
-    <row r="175" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" s="15" t="s">
         <v>540</v>
       </c>
@@ -30363,7 +30359,7 @@
       <c r="AN175" s="82"/>
       <c r="AO175" s="82"/>
     </row>
-    <row r="176" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" s="15" t="s">
         <v>541</v>
       </c>
@@ -30451,7 +30447,7 @@
       <c r="AN176" s="82"/>
       <c r="AO176" s="82"/>
     </row>
-    <row r="177" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" s="15" t="s">
         <v>544</v>
       </c>
@@ -30537,7 +30533,7 @@
       <c r="AN177" s="82"/>
       <c r="AO177" s="82"/>
     </row>
-    <row r="178" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" s="15" t="s">
         <v>546</v>
       </c>
@@ -30629,7 +30625,7 @@
       <c r="AN178" s="82"/>
       <c r="AO178" s="82"/>
     </row>
-    <row r="179" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" s="15" t="s">
         <v>547</v>
       </c>
@@ -30717,7 +30713,7 @@
       <c r="AN179" s="82"/>
       <c r="AO179" s="82"/>
     </row>
-    <row r="180" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" s="15" t="s">
         <v>551</v>
       </c>
@@ -30833,7 +30829,7 @@
       </c>
       <c r="AO180" s="82"/>
     </row>
-    <row r="181" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" s="15" t="s">
         <v>556</v>
       </c>
@@ -30949,7 +30945,7 @@
       </c>
       <c r="AO181" s="82"/>
     </row>
-    <row r="182" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" s="15" t="s">
         <v>561</v>
       </c>
@@ -31041,7 +31037,7 @@
       <c r="AN182" s="82"/>
       <c r="AO182" s="82"/>
     </row>
-    <row r="183" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" s="15" t="s">
         <v>563</v>
       </c>
@@ -31131,7 +31127,7 @@
       <c r="AN183" s="82"/>
       <c r="AO183" s="82"/>
     </row>
-    <row r="184" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" s="15" t="s">
         <v>564</v>
       </c>
@@ -31221,7 +31217,7 @@
       <c r="AN184" s="82"/>
       <c r="AO184" s="82"/>
     </row>
-    <row r="185" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185" s="15" t="s">
         <v>566</v>
       </c>
@@ -31309,7 +31305,7 @@
       <c r="AN185" s="82"/>
       <c r="AO185" s="82"/>
     </row>
-    <row r="186" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" s="15" t="s">
         <v>569</v>
       </c>
@@ -31397,7 +31393,7 @@
       <c r="AN186" s="82"/>
       <c r="AO186" s="82"/>
     </row>
-    <row r="187" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187" s="15" t="s">
         <v>571</v>
       </c>
@@ -31485,7 +31481,7 @@
       <c r="AN187" s="82"/>
       <c r="AO187" s="82"/>
     </row>
-    <row r="188" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" s="15" t="s">
         <v>574</v>
       </c>
@@ -31573,7 +31569,7 @@
       <c r="AN188" s="82"/>
       <c r="AO188" s="82"/>
     </row>
-    <row r="189" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" s="15" t="s">
         <v>577</v>
       </c>
@@ -31661,7 +31657,7 @@
       <c r="AN189" s="82"/>
       <c r="AO189" s="82"/>
     </row>
-    <row r="190" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" s="15" t="s">
         <v>579</v>
       </c>
@@ -31749,7 +31745,7 @@
       <c r="AN190" s="82"/>
       <c r="AO190" s="82"/>
     </row>
-    <row r="191" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" s="15" t="s">
         <v>581</v>
       </c>
@@ -31831,7 +31827,7 @@
       <c r="AN191" s="82"/>
       <c r="AO191" s="82"/>
     </row>
-    <row r="192" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" s="15" t="s">
         <v>583</v>
       </c>
@@ -31919,7 +31915,7 @@
       <c r="AN192" s="82"/>
       <c r="AO192" s="82"/>
     </row>
-    <row r="193" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" s="15" t="s">
         <v>585</v>
       </c>
@@ -32009,7 +32005,7 @@
       <c r="AN193" s="82"/>
       <c r="AO193" s="82"/>
     </row>
-    <row r="194" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194" s="15" t="s">
         <v>588</v>
       </c>
@@ -32097,7 +32093,7 @@
       <c r="AN194" s="82"/>
       <c r="AO194" s="82"/>
     </row>
-    <row r="195" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" s="15" t="s">
         <v>591</v>
       </c>
@@ -32185,7 +32181,7 @@
       <c r="AN195" s="82"/>
       <c r="AO195" s="82"/>
     </row>
-    <row r="196" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196" s="15" t="s">
         <v>594</v>
       </c>
@@ -32275,7 +32271,7 @@
       <c r="AN196" s="82"/>
       <c r="AO196" s="82"/>
     </row>
-    <row r="197" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" s="15" t="s">
         <v>598</v>
       </c>
@@ -32365,7 +32361,7 @@
       <c r="AN197" s="82"/>
       <c r="AO197" s="82"/>
     </row>
-    <row r="198" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A198" s="15" t="s">
         <v>600</v>
       </c>
@@ -32455,7 +32451,7 @@
       <c r="AN198" s="82"/>
       <c r="AO198" s="82"/>
     </row>
-    <row r="199" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199" s="15" t="s">
         <v>602</v>
       </c>
@@ -32543,7 +32539,7 @@
       <c r="AN199" s="82"/>
       <c r="AO199" s="82"/>
     </row>
-    <row r="200" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200" s="15" t="s">
         <v>604</v>
       </c>
@@ -32631,7 +32627,7 @@
       <c r="AN200" s="82"/>
       <c r="AO200" s="82"/>
     </row>
-    <row r="201" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" s="15" t="s">
         <v>606</v>
       </c>
@@ -32719,7 +32715,7 @@
       <c r="AN201" s="82"/>
       <c r="AO201" s="82"/>
     </row>
-    <row r="202" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" s="15" t="s">
         <v>609</v>
       </c>
@@ -32811,7 +32807,7 @@
       <c r="AN202" s="82"/>
       <c r="AO202" s="82"/>
     </row>
-    <row r="203" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" s="15" t="s">
         <v>610</v>
       </c>
@@ -32899,7 +32895,7 @@
       <c r="AN203" s="82"/>
       <c r="AO203" s="82"/>
     </row>
-    <row r="204" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204" s="15" t="s">
         <v>611</v>
       </c>
@@ -32987,7 +32983,7 @@
       <c r="AN204" s="82"/>
       <c r="AO204" s="82"/>
     </row>
-    <row r="205" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" s="15" t="s">
         <v>613</v>
       </c>
@@ -33077,7 +33073,7 @@
       <c r="AN205" s="82"/>
       <c r="AO205" s="82"/>
     </row>
-    <row r="206" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206" s="15" t="s">
         <v>614</v>
       </c>
@@ -33171,7 +33167,7 @@
       <c r="AN206" s="82"/>
       <c r="AO206" s="82"/>
     </row>
-    <row r="207" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207" s="15" t="s">
         <v>615</v>
       </c>
@@ -33259,7 +33255,7 @@
       <c r="AN207" s="82"/>
       <c r="AO207" s="82"/>
     </row>
-    <row r="208" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A208" s="15" t="s">
         <v>618</v>
       </c>
@@ -33349,7 +33345,7 @@
       <c r="AN208" s="82"/>
       <c r="AO208" s="82"/>
     </row>
-    <row r="209" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209" s="15" t="s">
         <v>620</v>
       </c>
@@ -33437,7 +33433,7 @@
       <c r="AN209" s="82"/>
       <c r="AO209" s="82"/>
     </row>
-    <row r="210" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210" s="15" t="s">
         <v>622</v>
       </c>
@@ -33525,7 +33521,7 @@
       <c r="AN210" s="82"/>
       <c r="AO210" s="82"/>
     </row>
-    <row r="211" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211" s="15" t="s">
         <v>624</v>
       </c>
@@ -33613,7 +33609,7 @@
       <c r="AN211" s="82"/>
       <c r="AO211" s="82"/>
     </row>
-    <row r="212" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A212" s="15" t="s">
         <v>626</v>
       </c>
@@ -33703,7 +33699,7 @@
       <c r="AN212" s="82"/>
       <c r="AO212" s="82"/>
     </row>
-    <row r="213" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213" s="15" t="s">
         <v>628</v>
       </c>
@@ -33791,7 +33787,7 @@
       <c r="AN213" s="82"/>
       <c r="AO213" s="82"/>
     </row>
-    <row r="214" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214" s="15" t="s">
         <v>630</v>
       </c>
@@ -33879,7 +33875,7 @@
       <c r="AN214" s="82"/>
       <c r="AO214" s="82"/>
     </row>
-    <row r="215" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" s="15" t="s">
         <v>633</v>
       </c>
@@ -33969,7 +33965,7 @@
       <c r="AN215" s="82"/>
       <c r="AO215" s="82"/>
     </row>
-    <row r="216" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A216" s="15" t="s">
         <v>636</v>
       </c>
@@ -34055,7 +34051,7 @@
       <c r="AN216" s="82"/>
       <c r="AO216" s="82"/>
     </row>
-    <row r="217" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217" s="15" t="s">
         <v>638</v>
       </c>
@@ -34143,7 +34139,7 @@
       <c r="AN217" s="82"/>
       <c r="AO217" s="82"/>
     </row>
-    <row r="218" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A218" s="15" t="s">
         <v>641</v>
       </c>
@@ -34229,7 +34225,7 @@
       <c r="AN218" s="82"/>
       <c r="AO218" s="82"/>
     </row>
-    <row r="219" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A219" s="15" t="s">
         <v>643</v>
       </c>
@@ -34315,7 +34311,7 @@
       <c r="AN219" s="82"/>
       <c r="AO219" s="82"/>
     </row>
-    <row r="220" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A220" s="15" t="s">
         <v>645</v>
       </c>
@@ -34397,7 +34393,7 @@
       <c r="AN220" s="82"/>
       <c r="AO220" s="82"/>
     </row>
-    <row r="221" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A221" s="15" t="s">
         <v>646</v>
       </c>
@@ -34483,7 +34479,7 @@
       <c r="AN221" s="82"/>
       <c r="AO221" s="82"/>
     </row>
-    <row r="222" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A222" s="15" t="s">
         <v>649</v>
       </c>
@@ -34569,7 +34565,7 @@
       <c r="AN222" s="82"/>
       <c r="AO222" s="82"/>
     </row>
-    <row r="223" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A223" s="15" t="s">
         <v>652</v>
       </c>
@@ -34655,7 +34651,7 @@
       <c r="AN223" s="82"/>
       <c r="AO223" s="82"/>
     </row>
-    <row r="224" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A224" s="15" t="s">
         <v>654</v>
       </c>
@@ -34745,7 +34741,7 @@
       <c r="AN224" s="82"/>
       <c r="AO224" s="82"/>
     </row>
-    <row r="225" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A225" s="15" t="s">
         <v>656</v>
       </c>
@@ -34829,7 +34825,7 @@
       <c r="AN225" s="82"/>
       <c r="AO225" s="82"/>
     </row>
-    <row r="226" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A226" s="15" t="s">
         <v>658</v>
       </c>
@@ -34917,7 +34913,7 @@
       <c r="AN226" s="82"/>
       <c r="AO226" s="82"/>
     </row>
-    <row r="227" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A227" s="15" t="s">
         <v>660</v>
       </c>
@@ -35005,7 +35001,7 @@
       <c r="AN227" s="82"/>
       <c r="AO227" s="82"/>
     </row>
-    <row r="228" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A228" s="15" t="s">
         <v>663</v>
       </c>
@@ -35091,7 +35087,7 @@
       <c r="AN228" s="82"/>
       <c r="AO228" s="82"/>
     </row>
-    <row r="229" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A229" s="15" t="s">
         <v>665</v>
       </c>
@@ -35175,7 +35171,7 @@
       <c r="AN229" s="82"/>
       <c r="AO229" s="82"/>
     </row>
-    <row r="230" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A230" s="15" t="s">
         <v>666</v>
       </c>
@@ -35261,7 +35257,7 @@
       <c r="AN230" s="82"/>
       <c r="AO230" s="82"/>
     </row>
-    <row r="231" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A231" s="15" t="s">
         <v>668</v>
       </c>
@@ -35347,7 +35343,7 @@
       <c r="AN231" s="82"/>
       <c r="AO231" s="82"/>
     </row>
-    <row r="232" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A232" s="15" t="s">
         <v>670</v>
       </c>
@@ -35429,7 +35425,7 @@
       <c r="AN232" s="82"/>
       <c r="AO232" s="82"/>
     </row>
-    <row r="233" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A233" s="15" t="s">
         <v>671</v>
       </c>
@@ -35515,7 +35511,7 @@
       <c r="AN233" s="82"/>
       <c r="AO233" s="82"/>
     </row>
-    <row r="234" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A234" s="15" t="s">
         <v>673</v>
       </c>
@@ -35605,7 +35601,7 @@
       <c r="AN234" s="82"/>
       <c r="AO234" s="82"/>
     </row>
-    <row r="235" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A235" s="15" t="s">
         <v>674</v>
       </c>
@@ -35693,7 +35689,7 @@
       <c r="AN235" s="82"/>
       <c r="AO235" s="82"/>
     </row>
-    <row r="236" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A236" s="15" t="s">
         <v>677</v>
       </c>
@@ -35781,7 +35777,7 @@
       <c r="AN236" s="82"/>
       <c r="AO236" s="82"/>
     </row>
-    <row r="237" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A237" s="15" t="s">
         <v>679</v>
       </c>
@@ -35869,7 +35865,7 @@
       <c r="AN237" s="82"/>
       <c r="AO237" s="82"/>
     </row>
-    <row r="238" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A238" s="15" t="s">
         <v>682</v>
       </c>
@@ -35961,7 +35957,7 @@
       <c r="AN238" s="82"/>
       <c r="AO238" s="82"/>
     </row>
-    <row r="239" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A239" s="15" t="s">
         <v>685</v>
       </c>
@@ -36053,7 +36049,7 @@
       <c r="AN239" s="82"/>
       <c r="AO239" s="82"/>
     </row>
-    <row r="240" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A240" s="15" t="s">
         <v>687</v>
       </c>
@@ -36145,7 +36141,7 @@
       <c r="AN240" s="82"/>
       <c r="AO240" s="82"/>
     </row>
-    <row r="241" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A241" s="15" t="s">
         <v>689</v>
       </c>
@@ -36235,7 +36231,7 @@
       <c r="AN241" s="82"/>
       <c r="AO241" s="82"/>
     </row>
-    <row r="242" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A242" s="15" t="s">
         <v>691</v>
       </c>
@@ -36323,7 +36319,7 @@
       <c r="AN242" s="82"/>
       <c r="AO242" s="82"/>
     </row>
-    <row r="243" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A243" s="15" t="s">
         <v>693</v>
       </c>
@@ -36417,7 +36413,7 @@
       <c r="AN243" s="82"/>
       <c r="AO243" s="82"/>
     </row>
-    <row r="244" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A244" s="15" t="s">
         <v>695</v>
       </c>
@@ -36505,7 +36501,7 @@
       <c r="AN244" s="82"/>
       <c r="AO244" s="82"/>
     </row>
-    <row r="245" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A245" s="15" t="s">
         <v>697</v>
       </c>
@@ -36591,7 +36587,7 @@
       <c r="AN245" s="82"/>
       <c r="AO245" s="82"/>
     </row>
-    <row r="246" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A246" s="15" t="s">
         <v>699</v>
       </c>
@@ -36679,7 +36675,7 @@
       <c r="AN246" s="82"/>
       <c r="AO246" s="82"/>
     </row>
-    <row r="247" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A247" s="15" t="s">
         <v>701</v>
       </c>
@@ -36767,7 +36763,7 @@
       <c r="AN247" s="82"/>
       <c r="AO247" s="82"/>
     </row>
-    <row r="248" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A248" s="15" t="s">
         <v>703</v>
       </c>
@@ -36855,7 +36851,7 @@
       <c r="AN248" s="82"/>
       <c r="AO248" s="82"/>
     </row>
-    <row r="249" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A249" s="15" t="s">
         <v>705</v>
       </c>
@@ -36943,7 +36939,7 @@
       <c r="AN249" s="82"/>
       <c r="AO249" s="82"/>
     </row>
-    <row r="250" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A250" s="15" t="s">
         <v>707</v>
       </c>
@@ -37033,7 +37029,7 @@
       <c r="AN250" s="82"/>
       <c r="AO250" s="82"/>
     </row>
-    <row r="251" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A251" s="15" t="s">
         <v>708</v>
       </c>
@@ -37119,7 +37115,7 @@
       <c r="AN251" s="82"/>
       <c r="AO251" s="82"/>
     </row>
-    <row r="252" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A252" s="15" t="s">
         <v>710</v>
       </c>
@@ -37205,7 +37201,7 @@
       <c r="AN252" s="82"/>
       <c r="AO252" s="82"/>
     </row>
-    <row r="253" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A253" s="15" t="s">
         <v>712</v>
       </c>
@@ -37291,7 +37287,7 @@
       <c r="AN253" s="82"/>
       <c r="AO253" s="82"/>
     </row>
-    <row r="254" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A254" s="15" t="s">
         <v>714</v>
       </c>
@@ -37377,7 +37373,7 @@
       <c r="AN254" s="82"/>
       <c r="AO254" s="82"/>
     </row>
-    <row r="255" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A255" s="15" t="s">
         <v>716</v>
       </c>
@@ -37465,7 +37461,7 @@
       <c r="AN255" s="82"/>
       <c r="AO255" s="82"/>
     </row>
-    <row r="256" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A256" s="15" t="s">
         <v>718</v>
       </c>
@@ -37555,7 +37551,7 @@
       <c r="AN256" s="82"/>
       <c r="AO256" s="82"/>
     </row>
-    <row r="257" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257" s="15" t="s">
         <v>720</v>
       </c>
@@ -37643,7 +37639,7 @@
       <c r="AN257" s="82"/>
       <c r="AO257" s="82"/>
     </row>
-    <row r="258" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A258" s="15" t="s">
         <v>722</v>
       </c>
@@ -37731,7 +37727,7 @@
       <c r="AN258" s="82"/>
       <c r="AO258" s="82"/>
     </row>
-    <row r="259" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A259" s="15" t="s">
         <v>724</v>
       </c>
@@ -37819,7 +37815,7 @@
       <c r="AN259" s="82"/>
       <c r="AO259" s="82"/>
     </row>
-    <row r="260" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A260" s="15" t="s">
         <v>726</v>
       </c>
@@ -37905,7 +37901,7 @@
       <c r="AN260" s="82"/>
       <c r="AO260" s="82"/>
     </row>
-    <row r="261" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A261" s="15" t="s">
         <v>727</v>
       </c>
@@ -37987,7 +37983,7 @@
       <c r="AN261" s="82"/>
       <c r="AO261" s="82"/>
     </row>
-    <row r="262" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A262" s="15" t="s">
         <v>728</v>
       </c>
@@ -38069,7 +38065,7 @@
       <c r="AN262" s="82"/>
       <c r="AO262" s="82"/>
     </row>
-    <row r="263" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A263" s="15" t="s">
         <v>729</v>
       </c>
@@ -38147,7 +38143,7 @@
       <c r="AN263" s="82"/>
       <c r="AO263" s="82"/>
     </row>
-    <row r="264" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A264" s="15" t="s">
         <v>731</v>
       </c>
@@ -38229,7 +38225,7 @@
       <c r="AN264" s="82"/>
       <c r="AO264" s="82"/>
     </row>
-    <row r="265" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A265" s="15" t="s">
         <v>732</v>
       </c>
@@ -38307,7 +38303,7 @@
       <c r="AN265" s="82"/>
       <c r="AO265" s="82"/>
     </row>
-    <row r="266" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A266" s="15" t="s">
         <v>733</v>
       </c>
@@ -38389,7 +38385,7 @@
       <c r="AN266" s="82"/>
       <c r="AO266" s="82"/>
     </row>
-    <row r="267" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A267" s="15" t="s">
         <v>734</v>
       </c>
@@ -38473,7 +38469,7 @@
       <c r="AN267" s="82"/>
       <c r="AO267" s="82"/>
     </row>
-    <row r="268" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A268" s="15" t="s">
         <v>735</v>
       </c>
@@ -38555,7 +38551,7 @@
       <c r="AN268" s="82"/>
       <c r="AO268" s="82"/>
     </row>
-    <row r="269" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A269" s="15" t="s">
         <v>737</v>
       </c>
@@ -38637,7 +38633,7 @@
       <c r="AN269" s="82"/>
       <c r="AO269" s="82"/>
     </row>
-    <row r="270" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A270" s="15" t="s">
         <v>738</v>
       </c>
@@ -38719,7 +38715,7 @@
       <c r="AN270" s="82"/>
       <c r="AO270" s="82"/>
     </row>
-    <row r="271" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A271" s="15" t="s">
         <v>739</v>
       </c>
@@ -38801,7 +38797,7 @@
       <c r="AN271" s="82"/>
       <c r="AO271" s="82"/>
     </row>
-    <row r="272" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A272" s="31" t="s">
         <v>740</v>
       </c>
@@ -38883,7 +38879,7 @@
       <c r="AN272" s="82"/>
       <c r="AO272" s="82"/>
     </row>
-    <row r="273" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A273" s="15" t="s">
         <v>741</v>
       </c>
@@ -38967,7 +38963,7 @@
       <c r="AN273" s="82"/>
       <c r="AO273" s="82"/>
     </row>
-    <row r="274" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A274" s="15" t="s">
         <v>742</v>
       </c>
@@ -39049,7 +39045,7 @@
       <c r="AN274" s="82"/>
       <c r="AO274" s="82"/>
     </row>
-    <row r="275" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A275" s="15" t="s">
         <v>743</v>
       </c>
@@ -39131,7 +39127,7 @@
       <c r="AN275" s="82"/>
       <c r="AO275" s="82"/>
     </row>
-    <row r="276" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A276" s="15" t="s">
         <v>744</v>
       </c>
@@ -39213,7 +39209,7 @@
       <c r="AN276" s="82"/>
       <c r="AO276" s="82"/>
     </row>
-    <row r="277" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A277" s="15" t="s">
         <v>745</v>
       </c>
@@ -39295,7 +39291,7 @@
       <c r="AN277" s="82"/>
       <c r="AO277" s="82"/>
     </row>
-    <row r="278" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A278" s="15" t="s">
         <v>746</v>
       </c>
@@ -39377,7 +39373,7 @@
       <c r="AN278" s="82"/>
       <c r="AO278" s="82"/>
     </row>
-    <row r="279" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A279" s="22" t="s">
         <v>747</v>
       </c>
@@ -39493,9 +39489,11 @@
       <c r="AN279" s="82">
         <v>46266</v>
       </c>
-      <c r="AO279" s="82"/>
+      <c r="AO279" s="82" t="s">
+        <v>1514</v>
+      </c>
     </row>
-    <row r="280" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A280" s="22" t="s">
         <v>757</v>
       </c>
@@ -39609,9 +39607,11 @@
       <c r="AN280" s="82">
         <v>46266</v>
       </c>
-      <c r="AO280" s="82"/>
+      <c r="AO280" s="82" t="s">
+        <v>1514</v>
+      </c>
     </row>
-    <row r="281" spans="1:41" s="26" customFormat="1" ht="122.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:41" s="26" customFormat="1" ht="122.4" x14ac:dyDescent="0.3">
       <c r="A281" s="22" t="s">
         <v>759</v>
       </c>
@@ -39727,9 +39727,11 @@
       <c r="AN281" s="82">
         <v>46266</v>
       </c>
-      <c r="AO281" s="82"/>
+      <c r="AO281" s="82" t="s">
+        <v>1514</v>
+      </c>
     </row>
-    <row r="282" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A282" s="22" t="s">
         <v>767</v>
       </c>
@@ -39843,7 +39845,7 @@
       <c r="AN282" s="82"/>
       <c r="AO282" s="82"/>
     </row>
-    <row r="283" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A283" s="22" t="s">
         <v>561</v>
       </c>
@@ -39957,9 +39959,11 @@
       <c r="AN283" s="82">
         <v>46235</v>
       </c>
-      <c r="AO283" s="82"/>
+      <c r="AO283" s="82" t="s">
+        <v>1514</v>
+      </c>
     </row>
-    <row r="284" spans="1:41" s="26" customFormat="1" ht="81.599999999999994" hidden="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:41" s="26" customFormat="1" ht="81.599999999999994" x14ac:dyDescent="0.3">
       <c r="A284" s="22" t="s">
         <v>777</v>
       </c>
@@ -40075,7 +40079,7 @@
       <c r="AN284" s="82"/>
       <c r="AO284" s="82"/>
     </row>
-    <row r="285" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A285" s="22" t="s">
         <v>781</v>
       </c>
@@ -40191,7 +40195,7 @@
       <c r="AN285" s="82"/>
       <c r="AO285" s="82"/>
     </row>
-    <row r="286" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A286" s="22" t="s">
         <v>785</v>
       </c>
@@ -40307,7 +40311,7 @@
       <c r="AN286" s="82"/>
       <c r="AO286" s="82"/>
     </row>
-    <row r="287" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" hidden="1" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:41" s="26" customFormat="1" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A287" s="22" t="s">
         <v>789</v>
       </c>
@@ -40423,7 +40427,7 @@
       <c r="AN287" s="82"/>
       <c r="AO287" s="82"/>
     </row>
-    <row r="288" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A288" s="22" t="s">
         <v>791</v>
       </c>
@@ -40539,7 +40543,7 @@
       <c r="AN288" s="82"/>
       <c r="AO288" s="82"/>
     </row>
-    <row r="289" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A289" s="22" t="s">
         <v>794</v>
       </c>
@@ -40655,7 +40659,7 @@
       <c r="AN289" s="82"/>
       <c r="AO289" s="82"/>
     </row>
-    <row r="290" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A290" s="22" t="s">
         <v>206</v>
       </c>
@@ -40753,7 +40757,7 @@
       <c r="AN290" s="82"/>
       <c r="AO290" s="82"/>
     </row>
-    <row r="291" spans="1:41" s="26" customFormat="1" ht="30.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:41" s="26" customFormat="1" ht="30.6" x14ac:dyDescent="0.3">
       <c r="A291" s="22" t="s">
         <v>803</v>
       </c>
@@ -40867,7 +40871,7 @@
       <c r="AN291" s="82"/>
       <c r="AO291" s="82"/>
     </row>
-    <row r="292" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A292" s="22" t="s">
         <v>808</v>
       </c>
@@ -40963,7 +40967,7 @@
       <c r="AN292" s="82"/>
       <c r="AO292" s="82"/>
     </row>
-    <row r="293" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A293" s="22" t="s">
         <v>811</v>
       </c>
@@ -41053,7 +41057,7 @@
       <c r="AN293" s="82"/>
       <c r="AO293" s="82"/>
     </row>
-    <row r="294" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A294" s="22" t="s">
         <v>814</v>
       </c>
@@ -41145,7 +41149,7 @@
       <c r="AN294" s="82"/>
       <c r="AO294" s="82"/>
     </row>
-    <row r="295" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A295" s="22" t="s">
         <v>816</v>
       </c>
@@ -41231,7 +41235,7 @@
       <c r="AN295" s="82"/>
       <c r="AO295" s="82"/>
     </row>
-    <row r="296" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A296" s="22" t="s">
         <v>820</v>
       </c>
@@ -41323,7 +41327,7 @@
       <c r="AN296" s="82"/>
       <c r="AO296" s="82"/>
     </row>
-    <row r="297" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A297" s="22" t="s">
         <v>727</v>
       </c>
@@ -41415,7 +41419,7 @@
       <c r="AN297" s="82"/>
       <c r="AO297" s="82"/>
     </row>
-    <row r="298" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A298" s="22" t="s">
         <v>155</v>
       </c>
@@ -41505,7 +41509,7 @@
       <c r="AN298" s="82"/>
       <c r="AO298" s="82"/>
     </row>
-    <row r="299" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A299" s="22" t="s">
         <v>827</v>
       </c>
@@ -41597,7 +41601,7 @@
       <c r="AN299" s="82"/>
       <c r="AO299" s="82"/>
     </row>
-    <row r="300" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A300" s="22" t="s">
         <v>828</v>
       </c>
@@ -41687,7 +41691,7 @@
       <c r="AN300" s="82"/>
       <c r="AO300" s="82"/>
     </row>
-    <row r="301" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A301" s="22" t="s">
         <v>390</v>
       </c>
@@ -41779,7 +41783,7 @@
       <c r="AN301" s="82"/>
       <c r="AO301" s="82"/>
     </row>
-    <row r="302" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A302" s="22" t="s">
         <v>265</v>
       </c>
@@ -41869,7 +41873,7 @@
       <c r="AN302" s="82"/>
       <c r="AO302" s="82"/>
     </row>
-    <row r="303" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A303" s="22" t="s">
         <v>835</v>
       </c>
@@ -41961,7 +41965,7 @@
       <c r="AN303" s="82"/>
       <c r="AO303" s="82"/>
     </row>
-    <row r="304" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A304" s="22" t="s">
         <v>838</v>
       </c>
@@ -42053,7 +42057,7 @@
       <c r="AN304" s="82"/>
       <c r="AO304" s="82"/>
     </row>
-    <row r="305" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A305" s="22" t="s">
         <v>52</v>
       </c>
@@ -42145,7 +42149,7 @@
       <c r="AN305" s="82"/>
       <c r="AO305" s="82"/>
     </row>
-    <row r="306" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A306" s="22" t="s">
         <v>842</v>
       </c>
@@ -42229,7 +42233,7 @@
       <c r="AN306" s="82"/>
       <c r="AO306" s="82"/>
     </row>
-    <row r="307" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A307" s="22" t="s">
         <v>844</v>
       </c>
@@ -42321,7 +42325,7 @@
       <c r="AN307" s="82"/>
       <c r="AO307" s="82"/>
     </row>
-    <row r="308" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A308" s="22" t="s">
         <v>846</v>
       </c>
@@ -42411,7 +42415,7 @@
       <c r="AN308" s="82"/>
       <c r="AO308" s="82"/>
     </row>
-    <row r="309" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A309" s="22" t="s">
         <v>847</v>
       </c>
@@ -42503,7 +42507,7 @@
       <c r="AN309" s="82"/>
       <c r="AO309" s="82"/>
     </row>
-    <row r="310" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A310" s="22" t="s">
         <v>649</v>
       </c>
@@ -42589,7 +42593,7 @@
       <c r="AN310" s="82"/>
       <c r="AO310" s="82"/>
     </row>
-    <row r="311" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A311" s="22" t="s">
         <v>738</v>
       </c>
@@ -42681,7 +42685,7 @@
       <c r="AN311" s="82"/>
       <c r="AO311" s="82"/>
     </row>
-    <row r="312" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A312" s="22" t="s">
         <v>117</v>
       </c>
@@ -42771,7 +42775,7 @@
       <c r="AN312" s="82"/>
       <c r="AO312" s="82"/>
     </row>
-    <row r="313" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A313" s="22">
         <v>98451</v>
       </c>
@@ -42845,7 +42849,7 @@
       <c r="AN313" s="82"/>
       <c r="AO313" s="82"/>
     </row>
-    <row r="314" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A314" s="22" t="s">
         <v>853</v>
       </c>
@@ -42941,7 +42945,7 @@
       <c r="AN314" s="82"/>
       <c r="AO314" s="82"/>
     </row>
-    <row r="315" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A315" s="22" t="s">
         <v>856</v>
       </c>
@@ -43033,7 +43037,7 @@
       <c r="AN315" s="82"/>
       <c r="AO315" s="82"/>
     </row>
-    <row r="316" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A316" s="3" t="s">
         <v>858</v>
       </c>
@@ -43121,7 +43125,7 @@
       <c r="AN316" s="82"/>
       <c r="AO316" s="82"/>
     </row>
-    <row r="317" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A317" s="22" t="s">
         <v>643</v>
       </c>
@@ -43207,7 +43211,7 @@
       <c r="AN317" s="82"/>
       <c r="AO317" s="82"/>
     </row>
-    <row r="318" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A318" s="22" t="s">
         <v>861</v>
       </c>
@@ -43299,7 +43303,7 @@
       <c r="AN318" s="82"/>
       <c r="AO318" s="82"/>
     </row>
-    <row r="319" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A319" s="22" t="s">
         <v>863</v>
       </c>
@@ -43395,7 +43399,7 @@
       <c r="AN319" s="82"/>
       <c r="AO319" s="82"/>
     </row>
-    <row r="320" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A320" s="22" t="s">
         <v>324</v>
       </c>
@@ -43485,7 +43489,7 @@
       <c r="AN320" s="82"/>
       <c r="AO320" s="82"/>
     </row>
-    <row r="321" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A321" s="22" t="s">
         <v>865</v>
       </c>
@@ -43567,7 +43571,7 @@
       <c r="AN321" s="82"/>
       <c r="AO321" s="82"/>
     </row>
-    <row r="322" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A322" s="3" t="s">
         <v>867</v>
       </c>
@@ -43655,7 +43659,7 @@
       <c r="AN322" s="82"/>
       <c r="AO322" s="82"/>
     </row>
-    <row r="323" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A323" s="22" t="s">
         <v>868</v>
       </c>
@@ -43743,7 +43747,7 @@
       <c r="AN323" s="82"/>
       <c r="AO323" s="82"/>
     </row>
-    <row r="324" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A324" s="22" t="s">
         <v>869</v>
       </c>
@@ -43827,7 +43831,7 @@
       <c r="AN324" s="82"/>
       <c r="AO324" s="82"/>
     </row>
-    <row r="325" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A325" s="22" t="s">
         <v>131</v>
       </c>
@@ -43917,7 +43921,7 @@
       <c r="AN325" s="82"/>
       <c r="AO325" s="82"/>
     </row>
-    <row r="326" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A326" s="3" t="s">
         <v>873</v>
       </c>
@@ -44007,7 +44011,7 @@
       <c r="AN326" s="82"/>
       <c r="AO326" s="82"/>
     </row>
-    <row r="327" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A327" s="22" t="s">
         <v>645</v>
       </c>
@@ -44093,7 +44097,7 @@
       <c r="AN327" s="82"/>
       <c r="AO327" s="82"/>
     </row>
-    <row r="328" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A328" s="3" t="s">
         <v>875</v>
       </c>
@@ -44181,7 +44185,7 @@
       <c r="AN328" s="82"/>
       <c r="AO328" s="82"/>
     </row>
-    <row r="329" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A329" s="3" t="s">
         <v>876</v>
       </c>
@@ -44269,7 +44273,7 @@
       <c r="AN329" s="82"/>
       <c r="AO329" s="82"/>
     </row>
-    <row r="330" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A330" s="3" t="s">
         <v>877</v>
       </c>
@@ -44357,7 +44361,7 @@
       <c r="AN330" s="82"/>
       <c r="AO330" s="82"/>
     </row>
-    <row r="331" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A331" s="3" t="s">
         <v>879</v>
       </c>
@@ -44441,7 +44445,7 @@
       <c r="AN331" s="82"/>
       <c r="AO331" s="82"/>
     </row>
-    <row r="332" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A332" s="3" t="s">
         <v>882</v>
       </c>
@@ -44525,7 +44529,7 @@
       <c r="AN332" s="82"/>
       <c r="AO332" s="82"/>
     </row>
-    <row r="333" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A333" s="3" t="s">
         <v>885</v>
       </c>
@@ -44613,7 +44617,7 @@
       <c r="AN333" s="82"/>
       <c r="AO333" s="82"/>
     </row>
-    <row r="334" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A334" s="22" t="s">
         <v>886</v>
       </c>
@@ -44705,7 +44709,7 @@
       <c r="AN334" s="82"/>
       <c r="AO334" s="82"/>
     </row>
-    <row r="335" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A335" s="22" t="s">
         <v>889</v>
       </c>
@@ -44789,7 +44793,7 @@
       <c r="AN335" s="82"/>
       <c r="AO335" s="82"/>
     </row>
-    <row r="336" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A336" s="3" t="s">
         <v>274</v>
       </c>
@@ -44867,7 +44871,7 @@
       <c r="AN336" s="82"/>
       <c r="AO336" s="82"/>
     </row>
-    <row r="337" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A337" s="22" t="s">
         <v>891</v>
       </c>
@@ -44959,7 +44963,7 @@
       <c r="AN337" s="82"/>
       <c r="AO337" s="82"/>
     </row>
-    <row r="338" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A338" s="3" t="s">
         <v>663</v>
       </c>
@@ -45043,7 +45047,7 @@
       <c r="AN338" s="82"/>
       <c r="AO338" s="82"/>
     </row>
-    <row r="339" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A339" s="22" t="s">
         <v>894</v>
       </c>
@@ -45127,7 +45131,7 @@
       <c r="AN339" s="82"/>
       <c r="AO339" s="82"/>
     </row>
-    <row r="340" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A340" s="3" t="s">
         <v>897</v>
       </c>
@@ -45211,7 +45215,7 @@
       <c r="AN340" s="82"/>
       <c r="AO340" s="82"/>
     </row>
-    <row r="341" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A341" s="22" t="s">
         <v>899</v>
       </c>
@@ -45295,7 +45299,7 @@
       <c r="AN341" s="82"/>
       <c r="AO341" s="82"/>
     </row>
-    <row r="342" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A342" s="22" t="s">
         <v>901</v>
       </c>
@@ -45379,7 +45383,7 @@
       <c r="AN342" s="82"/>
       <c r="AO342" s="82"/>
     </row>
-    <row r="343" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A343" s="3" t="s">
         <v>903</v>
       </c>
@@ -45469,7 +45473,7 @@
       <c r="AN343" s="82"/>
       <c r="AO343" s="82"/>
     </row>
-    <row r="344" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A344" s="22" t="s">
         <v>904</v>
       </c>
@@ -45557,7 +45561,7 @@
       <c r="AN344" s="82"/>
       <c r="AO344" s="82"/>
     </row>
-    <row r="345" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A345" s="3" t="s">
         <v>906</v>
       </c>
@@ -45645,7 +45649,7 @@
       <c r="AN345" s="82"/>
       <c r="AO345" s="82"/>
     </row>
-    <row r="346" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A346" s="3" t="s">
         <v>654</v>
       </c>
@@ -45733,7 +45737,7 @@
       <c r="AN346" s="82"/>
       <c r="AO346" s="82"/>
     </row>
-    <row r="347" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A347" s="22" t="s">
         <v>908</v>
       </c>
@@ -45813,7 +45817,7 @@
       <c r="AN347" s="82"/>
       <c r="AO347" s="82"/>
     </row>
-    <row r="348" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A348" s="3" t="s">
         <v>911</v>
       </c>
@@ -45901,7 +45905,7 @@
       <c r="AN348" s="82"/>
       <c r="AO348" s="82"/>
     </row>
-    <row r="349" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A349" s="22" t="s">
         <v>912</v>
       </c>
@@ -45989,7 +45993,7 @@
       <c r="AN349" s="82"/>
       <c r="AO349" s="82"/>
     </row>
-    <row r="350" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A350" s="3" t="s">
         <v>914</v>
       </c>
@@ -46073,7 +46077,7 @@
       <c r="AN350" s="82"/>
       <c r="AO350" s="82"/>
     </row>
-    <row r="351" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A351" s="22" t="s">
         <v>916</v>
       </c>
@@ -46165,7 +46169,7 @@
       <c r="AN351" s="82"/>
       <c r="AO351" s="82"/>
     </row>
-    <row r="352" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A352" s="22" t="s">
         <v>917</v>
       </c>
@@ -46249,7 +46253,7 @@
       <c r="AN352" s="82"/>
       <c r="AO352" s="82"/>
     </row>
-    <row r="353" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A353" s="3" t="s">
         <v>919</v>
       </c>
@@ -46337,7 +46341,7 @@
       <c r="AN353" s="82"/>
       <c r="AO353" s="82"/>
     </row>
-    <row r="354" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A354" s="3" t="s">
         <v>920</v>
       </c>
@@ -46421,7 +46425,7 @@
       <c r="AN354" s="82"/>
       <c r="AO354" s="82"/>
     </row>
-    <row r="355" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A355" s="22" t="s">
         <v>921</v>
       </c>
@@ -46513,7 +46517,7 @@
       <c r="AN355" s="82"/>
       <c r="AO355" s="82"/>
     </row>
-    <row r="356" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A356" s="3" t="s">
         <v>393</v>
       </c>
@@ -46597,7 +46601,7 @@
       <c r="AN356" s="82"/>
       <c r="AO356" s="82"/>
     </row>
-    <row r="357" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A357" s="22" t="s">
         <v>922</v>
       </c>
@@ -46681,7 +46685,7 @@
       <c r="AN357" s="82"/>
       <c r="AO357" s="82"/>
     </row>
-    <row r="358" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A358" s="22" t="s">
         <v>926</v>
       </c>
@@ -46765,7 +46769,7 @@
       <c r="AN358" s="82"/>
       <c r="AO358" s="82"/>
     </row>
-    <row r="359" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A359" s="3" t="s">
         <v>927</v>
       </c>
@@ -46853,7 +46857,7 @@
       <c r="AN359" s="82"/>
       <c r="AO359" s="82"/>
     </row>
-    <row r="360" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A360" s="22" t="s">
         <v>928</v>
       </c>
@@ -46945,7 +46949,7 @@
       <c r="AN360" s="82"/>
       <c r="AO360" s="82"/>
     </row>
-    <row r="361" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A361" s="3" t="s">
         <v>369</v>
       </c>
@@ -47029,7 +47033,7 @@
       <c r="AN361" s="82"/>
       <c r="AO361" s="82"/>
     </row>
-    <row r="362" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A362" s="3" t="s">
         <v>929</v>
       </c>
@@ -47117,7 +47121,7 @@
       <c r="AN362" s="82"/>
       <c r="AO362" s="82"/>
     </row>
-    <row r="363" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A363" s="22" t="s">
         <v>931</v>
       </c>
@@ -47201,7 +47205,7 @@
       <c r="AN363" s="82"/>
       <c r="AO363" s="82"/>
     </row>
-    <row r="364" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A364" s="3" t="s">
         <v>658</v>
       </c>
@@ -47285,7 +47289,7 @@
       <c r="AN364" s="82"/>
       <c r="AO364" s="82"/>
     </row>
-    <row r="365" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A365" s="22" t="s">
         <v>932</v>
       </c>
@@ -47369,7 +47373,7 @@
       <c r="AN365" s="82"/>
       <c r="AO365" s="82"/>
     </row>
-    <row r="366" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A366" s="3" t="s">
         <v>933</v>
       </c>
@@ -47453,7 +47457,7 @@
       <c r="AN366" s="82"/>
       <c r="AO366" s="82"/>
     </row>
-    <row r="367" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A367" s="3" t="s">
         <v>739</v>
       </c>
@@ -47537,7 +47541,7 @@
       <c r="AN367" s="82"/>
       <c r="AO367" s="82"/>
     </row>
-    <row r="368" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A368" s="3" t="s">
         <v>673</v>
       </c>
@@ -47621,7 +47625,7 @@
       <c r="AN368" s="82"/>
       <c r="AO368" s="82"/>
     </row>
-    <row r="369" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A369" s="3" t="s">
         <v>937</v>
       </c>
@@ -47705,7 +47709,7 @@
       <c r="AN369" s="82"/>
       <c r="AO369" s="82"/>
     </row>
-    <row r="370" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A370" s="22" t="s">
         <v>939</v>
       </c>
@@ -47789,7 +47793,7 @@
       <c r="AN370" s="82"/>
       <c r="AO370" s="82"/>
     </row>
-    <row r="371" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A371" s="22" t="s">
         <v>942</v>
       </c>
@@ -47873,7 +47877,7 @@
       <c r="AN371" s="82"/>
       <c r="AO371" s="82"/>
     </row>
-    <row r="372" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A372" s="22" t="s">
         <v>944</v>
       </c>
@@ -47957,7 +47961,7 @@
       <c r="AN372" s="82"/>
       <c r="AO372" s="82"/>
     </row>
-    <row r="373" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A373" s="3" t="s">
         <v>945</v>
       </c>
@@ -48041,7 +48045,7 @@
       <c r="AN373" s="82"/>
       <c r="AO373" s="82"/>
     </row>
-    <row r="374" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A374" s="3" t="s">
         <v>947</v>
       </c>
@@ -48125,7 +48129,7 @@
       <c r="AN374" s="82"/>
       <c r="AO374" s="82"/>
     </row>
-    <row r="375" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A375" s="22" t="s">
         <v>948</v>
       </c>
@@ -48209,7 +48213,7 @@
       <c r="AN375" s="82"/>
       <c r="AO375" s="82"/>
     </row>
-    <row r="376" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A376" s="3" t="s">
         <v>949</v>
       </c>
@@ -48293,7 +48297,7 @@
       <c r="AN376" s="82"/>
       <c r="AO376" s="82"/>
     </row>
-    <row r="377" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A377" s="22" t="s">
         <v>950</v>
       </c>
@@ -48377,7 +48381,7 @@
       <c r="AN377" s="82"/>
       <c r="AO377" s="82"/>
     </row>
-    <row r="378" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A378" s="22" t="s">
         <v>952</v>
       </c>
@@ -48461,7 +48465,7 @@
       <c r="AN378" s="82"/>
       <c r="AO378" s="82"/>
     </row>
-    <row r="379" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A379" s="22" t="s">
         <v>955</v>
       </c>
@@ -48545,7 +48549,7 @@
       <c r="AN379" s="82"/>
       <c r="AO379" s="82"/>
     </row>
-    <row r="380" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A380" s="22" t="s">
         <v>957</v>
       </c>
@@ -48629,7 +48633,7 @@
       <c r="AN380" s="82"/>
       <c r="AO380" s="82"/>
     </row>
-    <row r="381" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A381" s="22" t="s">
         <v>961</v>
       </c>
@@ -48717,7 +48721,7 @@
       <c r="AN381" s="82"/>
       <c r="AO381" s="82"/>
     </row>
-    <row r="382" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A382" s="3" t="s">
         <v>963</v>
       </c>
@@ -48797,7 +48801,7 @@
       <c r="AN382" s="82"/>
       <c r="AO382" s="82"/>
     </row>
-    <row r="383" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A383" s="22" t="s">
         <v>965</v>
       </c>
@@ -48881,7 +48885,7 @@
       <c r="AN383" s="82"/>
       <c r="AO383" s="82"/>
     </row>
-    <row r="384" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A384" s="22" t="s">
         <v>322</v>
       </c>
@@ -48965,7 +48969,7 @@
       <c r="AN384" s="82"/>
       <c r="AO384" s="82"/>
     </row>
-    <row r="385" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A385" s="3" t="s">
         <v>966</v>
       </c>
@@ -49053,7 +49057,7 @@
       <c r="AN385" s="82"/>
       <c r="AO385" s="82"/>
     </row>
-    <row r="386" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A386" s="22" t="s">
         <v>470</v>
       </c>
@@ -49137,7 +49141,7 @@
       <c r="AN386" s="82"/>
       <c r="AO386" s="82"/>
     </row>
-    <row r="387" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A387" s="22" t="s">
         <v>315</v>
       </c>
@@ -49221,7 +49225,7 @@
       <c r="AN387" s="82"/>
       <c r="AO387" s="82"/>
     </row>
-    <row r="388" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A388" s="3" t="s">
         <v>970</v>
       </c>
@@ -49305,7 +49309,7 @@
       <c r="AN388" s="82"/>
       <c r="AO388" s="82"/>
     </row>
-    <row r="389" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A389" s="22" t="s">
         <v>971</v>
       </c>
@@ -49397,7 +49401,7 @@
       <c r="AN389" s="82"/>
       <c r="AO389" s="82"/>
     </row>
-    <row r="390" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A390" s="22" t="s">
         <v>972</v>
       </c>
@@ -49489,7 +49493,7 @@
       <c r="AN390" s="82"/>
       <c r="AO390" s="82"/>
     </row>
-    <row r="391" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="391" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A391" s="22" t="s">
         <v>973</v>
       </c>
@@ -49573,7 +49577,7 @@
       <c r="AN391" s="82"/>
       <c r="AO391" s="82"/>
     </row>
-    <row r="392" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A392" s="22" t="s">
         <v>974</v>
       </c>
@@ -49657,7 +49661,7 @@
       <c r="AN392" s="82"/>
       <c r="AO392" s="82"/>
     </row>
-    <row r="393" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A393" s="22" t="s">
         <v>976</v>
       </c>
@@ -49749,7 +49753,7 @@
       <c r="AN393" s="82"/>
       <c r="AO393" s="82"/>
     </row>
-    <row r="394" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A394" s="22" t="s">
         <v>445</v>
       </c>
@@ -49833,7 +49837,7 @@
       <c r="AN394" s="82"/>
       <c r="AO394" s="82"/>
     </row>
-    <row r="395" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="395" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A395" s="22" t="s">
         <v>978</v>
       </c>
@@ -49925,7 +49929,7 @@
       <c r="AN395" s="82"/>
       <c r="AO395" s="82"/>
     </row>
-    <row r="396" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A396" s="22" t="s">
         <v>481</v>
       </c>
@@ -50009,7 +50013,7 @@
       <c r="AN396" s="82"/>
       <c r="AO396" s="82"/>
     </row>
-    <row r="397" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A397" s="22" t="s">
         <v>981</v>
       </c>
@@ -50093,7 +50097,7 @@
       <c r="AN397" s="82"/>
       <c r="AO397" s="82"/>
     </row>
-    <row r="398" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="398" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A398" s="22" t="s">
         <v>982</v>
       </c>
@@ -50177,7 +50181,7 @@
       <c r="AN398" s="82"/>
       <c r="AO398" s="82"/>
     </row>
-    <row r="399" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="399" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A399" s="22" t="s">
         <v>984</v>
       </c>
@@ -50261,7 +50265,7 @@
       <c r="AN399" s="82"/>
       <c r="AO399" s="82"/>
     </row>
-    <row r="400" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A400" s="3" t="s">
         <v>985</v>
       </c>
@@ -50345,7 +50349,7 @@
       <c r="AN400" s="82"/>
       <c r="AO400" s="82"/>
     </row>
-    <row r="401" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A401" s="3" t="s">
         <v>986</v>
       </c>
@@ -50433,7 +50437,7 @@
       <c r="AN401" s="82"/>
       <c r="AO401" s="82"/>
     </row>
-    <row r="402" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A402" s="22" t="s">
         <v>987</v>
       </c>
@@ -50517,7 +50521,7 @@
       <c r="AN402" s="82"/>
       <c r="AO402" s="82"/>
     </row>
-    <row r="403" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A403" s="22" t="s">
         <v>988</v>
       </c>
@@ -50601,7 +50605,7 @@
       <c r="AN403" s="82"/>
       <c r="AO403" s="82"/>
     </row>
-    <row r="404" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A404" s="22" t="s">
         <v>991</v>
       </c>
@@ -50691,7 +50695,7 @@
       <c r="AN404" s="82"/>
       <c r="AO404" s="82"/>
     </row>
-    <row r="405" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="405" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A405" s="22" t="s">
         <v>992</v>
       </c>
@@ -50783,7 +50787,7 @@
       <c r="AN405" s="82"/>
       <c r="AO405" s="82"/>
     </row>
-    <row r="406" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A406" s="3" t="s">
         <v>994</v>
       </c>
@@ -50871,7 +50875,7 @@
       <c r="AN406" s="82"/>
       <c r="AO406" s="82"/>
     </row>
-    <row r="407" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="407" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A407" s="22" t="s">
         <v>996</v>
       </c>
@@ -50963,7 +50967,7 @@
       <c r="AN407" s="82"/>
       <c r="AO407" s="82"/>
     </row>
-    <row r="408" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="408" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A408" s="22" t="s">
         <v>998</v>
       </c>
@@ -51047,7 +51051,7 @@
       <c r="AN408" s="82"/>
       <c r="AO408" s="82"/>
     </row>
-    <row r="409" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="409" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A409" s="22" t="s">
         <v>1000</v>
       </c>
@@ -51131,7 +51135,7 @@
       <c r="AN409" s="82"/>
       <c r="AO409" s="82"/>
     </row>
-    <row r="410" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="410" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A410" s="22" t="s">
         <v>1002</v>
       </c>
@@ -51215,7 +51219,7 @@
       <c r="AN410" s="82"/>
       <c r="AO410" s="82"/>
     </row>
-    <row r="411" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="411" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A411" s="22" t="s">
         <v>413</v>
       </c>
@@ -51299,7 +51303,7 @@
       <c r="AN411" s="82"/>
       <c r="AO411" s="82"/>
     </row>
-    <row r="412" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="412" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A412" s="22" t="s">
         <v>1004</v>
       </c>
@@ -51383,7 +51387,7 @@
       <c r="AN412" s="82"/>
       <c r="AO412" s="82"/>
     </row>
-    <row r="413" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="413" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A413" s="22" t="s">
         <v>1005</v>
       </c>
@@ -51467,7 +51471,7 @@
       <c r="AN413" s="82"/>
       <c r="AO413" s="82"/>
     </row>
-    <row r="414" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="414" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A414" s="22" t="s">
         <v>1007</v>
       </c>
@@ -51551,7 +51555,7 @@
       <c r="AN414" s="82"/>
       <c r="AO414" s="82"/>
     </row>
-    <row r="415" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="415" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A415" s="22" t="s">
         <v>1009</v>
       </c>
@@ -51641,7 +51645,7 @@
       <c r="AN415" s="82"/>
       <c r="AO415" s="82"/>
     </row>
-    <row r="416" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="416" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A416" s="22" t="s">
         <v>1010</v>
       </c>
@@ -51733,7 +51737,7 @@
       <c r="AN416" s="82"/>
       <c r="AO416" s="82"/>
     </row>
-    <row r="417" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A417" s="22" t="s">
         <v>1011</v>
       </c>
@@ -51825,7 +51829,7 @@
       <c r="AN417" s="82"/>
       <c r="AO417" s="82"/>
     </row>
-    <row r="418" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="418" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A418" s="22" t="s">
         <v>1012</v>
       </c>
@@ -51915,7 +51919,7 @@
       <c r="AN418" s="82"/>
       <c r="AO418" s="82"/>
     </row>
-    <row r="419" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="419" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A419" s="22" t="s">
         <v>1013</v>
       </c>
@@ -52007,7 +52011,7 @@
       <c r="AN419" s="82"/>
       <c r="AO419" s="82"/>
     </row>
-    <row r="420" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="420" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A420" s="22" t="s">
         <v>1014</v>
       </c>
@@ -52091,7 +52095,7 @@
       <c r="AN420" s="82"/>
       <c r="AO420" s="82"/>
     </row>
-    <row r="421" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="421" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A421" s="22" t="s">
         <v>1016</v>
       </c>
@@ -52175,7 +52179,7 @@
       <c r="AN421" s="82"/>
       <c r="AO421" s="82"/>
     </row>
-    <row r="422" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="422" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A422" s="22" t="s">
         <v>1018</v>
       </c>
@@ -52259,7 +52263,7 @@
       <c r="AN422" s="82"/>
       <c r="AO422" s="82"/>
     </row>
-    <row r="423" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="423" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A423" s="22" t="s">
         <v>1020</v>
       </c>
@@ -52343,7 +52347,7 @@
       <c r="AN423" s="82"/>
       <c r="AO423" s="82"/>
     </row>
-    <row r="424" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="424" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A424" s="22" t="s">
         <v>1023</v>
       </c>
@@ -52427,7 +52431,7 @@
       <c r="AN424" s="82"/>
       <c r="AO424" s="82"/>
     </row>
-    <row r="425" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="425" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A425" s="22" t="s">
         <v>1025</v>
       </c>
@@ -52511,7 +52515,7 @@
       <c r="AN425" s="82"/>
       <c r="AO425" s="82"/>
     </row>
-    <row r="426" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="426" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A426" s="22" t="s">
         <v>1027</v>
       </c>
@@ -52595,7 +52599,7 @@
       <c r="AN426" s="82"/>
       <c r="AO426" s="82"/>
     </row>
-    <row r="427" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="427" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A427" s="22" t="s">
         <v>1028</v>
       </c>
@@ -52679,7 +52683,7 @@
       <c r="AN427" s="82"/>
       <c r="AO427" s="82"/>
     </row>
-    <row r="428" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="428" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A428" s="22" t="s">
         <v>1029</v>
       </c>
@@ -52763,7 +52767,7 @@
       <c r="AN428" s="82"/>
       <c r="AO428" s="82"/>
     </row>
-    <row r="429" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="429" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A429" s="22" t="s">
         <v>1031</v>
       </c>
@@ -52847,7 +52851,7 @@
       <c r="AN429" s="82"/>
       <c r="AO429" s="82"/>
     </row>
-    <row r="430" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="430" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A430" s="22" t="s">
         <v>1033</v>
       </c>
@@ -52931,7 +52935,7 @@
       <c r="AN430" s="82"/>
       <c r="AO430" s="82"/>
     </row>
-    <row r="431" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="431" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A431" s="22" t="s">
         <v>1035</v>
       </c>
@@ -53015,7 +53019,7 @@
       <c r="AN431" s="82"/>
       <c r="AO431" s="82"/>
     </row>
-    <row r="432" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="432" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A432" s="22" t="s">
         <v>641</v>
       </c>
@@ -53099,7 +53103,7 @@
       <c r="AN432" s="82"/>
       <c r="AO432" s="82"/>
     </row>
-    <row r="433" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="433" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A433" s="22" t="s">
         <v>1040</v>
       </c>
@@ -53183,7 +53187,7 @@
       <c r="AN433" s="82"/>
       <c r="AO433" s="82"/>
     </row>
-    <row r="434" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="434" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A434" s="22" t="s">
         <v>1042</v>
       </c>
@@ -53267,7 +53271,7 @@
       <c r="AN434" s="82"/>
       <c r="AO434" s="82"/>
     </row>
-    <row r="435" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="435" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A435" s="22" t="s">
         <v>1043</v>
       </c>
@@ -53351,7 +53355,7 @@
       <c r="AN435" s="82"/>
       <c r="AO435" s="82"/>
     </row>
-    <row r="436" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="436" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A436" s="22" t="s">
         <v>1045</v>
       </c>
@@ -53435,7 +53439,7 @@
       <c r="AN436" s="82"/>
       <c r="AO436" s="82"/>
     </row>
-    <row r="437" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="437" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A437" s="22" t="s">
         <v>1047</v>
       </c>
@@ -53519,7 +53523,7 @@
       <c r="AN437" s="82"/>
       <c r="AO437" s="82"/>
     </row>
-    <row r="438" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="438" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A438" s="22" t="s">
         <v>397</v>
       </c>
@@ -53603,7 +53607,7 @@
       <c r="AN438" s="82"/>
       <c r="AO438" s="82"/>
     </row>
-    <row r="439" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="439" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A439" s="22" t="s">
         <v>744</v>
       </c>
@@ -53687,7 +53691,7 @@
       <c r="AN439" s="82"/>
       <c r="AO439" s="82"/>
     </row>
-    <row r="440" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="440" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A440" s="22" t="s">
         <v>1052</v>
       </c>
@@ -53771,7 +53775,7 @@
       <c r="AN440" s="82"/>
       <c r="AO440" s="82"/>
     </row>
-    <row r="441" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="441" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A441" s="22" t="s">
         <v>1053</v>
       </c>
@@ -53855,7 +53859,7 @@
       <c r="AN441" s="82"/>
       <c r="AO441" s="82"/>
     </row>
-    <row r="442" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="442" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A442" s="22" t="s">
         <v>1054</v>
       </c>
@@ -53939,7 +53943,7 @@
       <c r="AN442" s="82"/>
       <c r="AO442" s="82"/>
     </row>
-    <row r="443" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="443" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A443" s="22" t="s">
         <v>1056</v>
       </c>
@@ -54023,7 +54027,7 @@
       <c r="AN443" s="82"/>
       <c r="AO443" s="82"/>
     </row>
-    <row r="444" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="444" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A444" s="22" t="s">
         <v>1058</v>
       </c>
@@ -54107,7 +54111,7 @@
       <c r="AN444" s="82"/>
       <c r="AO444" s="82"/>
     </row>
-    <row r="445" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="445" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A445" s="22" t="s">
         <v>1061</v>
       </c>
@@ -54191,7 +54195,7 @@
       <c r="AN445" s="82"/>
       <c r="AO445" s="82"/>
     </row>
-    <row r="446" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="446" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A446" s="22" t="s">
         <v>1062</v>
       </c>
@@ -54275,7 +54279,7 @@
       <c r="AN446" s="82"/>
       <c r="AO446" s="82"/>
     </row>
-    <row r="447" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="447" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A447" s="3" t="s">
         <v>652</v>
       </c>
@@ -54351,7 +54355,7 @@
       <c r="AN447" s="82"/>
       <c r="AO447" s="82"/>
     </row>
-    <row r="448" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="448" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A448" s="3" t="s">
         <v>1063</v>
       </c>
@@ -54435,7 +54439,7 @@
       <c r="AN448" s="82"/>
       <c r="AO448" s="82"/>
     </row>
-    <row r="449" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="449" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A449" s="3" t="s">
         <v>1064</v>
       </c>
@@ -54519,7 +54523,7 @@
       <c r="AN449" s="82"/>
       <c r="AO449" s="82"/>
     </row>
-    <row r="450" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="450" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A450" s="3" t="s">
         <v>1065</v>
       </c>
@@ -54603,7 +54607,7 @@
       <c r="AN450" s="82"/>
       <c r="AO450" s="82"/>
     </row>
-    <row r="451" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="451" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A451" s="3" t="s">
         <v>1066</v>
       </c>
@@ -54687,7 +54691,7 @@
       <c r="AN451" s="82"/>
       <c r="AO451" s="82"/>
     </row>
-    <row r="452" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="452" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A452" s="3" t="s">
         <v>1067</v>
       </c>
@@ -54771,7 +54775,7 @@
       <c r="AN452" s="82"/>
       <c r="AO452" s="82"/>
     </row>
-    <row r="453" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="453" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A453" s="3" t="s">
         <v>1068</v>
       </c>
@@ -54855,7 +54859,7 @@
       <c r="AN453" s="82"/>
       <c r="AO453" s="82"/>
     </row>
-    <row r="454" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="454" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A454" s="3" t="s">
         <v>1069</v>
       </c>
@@ -54939,7 +54943,7 @@
       <c r="AN454" s="82"/>
       <c r="AO454" s="82"/>
     </row>
-    <row r="455" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="455" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A455" s="3" t="s">
         <v>1070</v>
       </c>
@@ -55023,7 +55027,7 @@
       <c r="AN455" s="82"/>
       <c r="AO455" s="82"/>
     </row>
-    <row r="456" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="456" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A456" s="3" t="s">
         <v>1071</v>
       </c>
@@ -55107,7 +55111,7 @@
       <c r="AN456" s="82"/>
       <c r="AO456" s="82"/>
     </row>
-    <row r="457" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="457" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A457" s="3" t="s">
         <v>1073</v>
       </c>
@@ -55191,7 +55195,7 @@
       <c r="AN457" s="82"/>
       <c r="AO457" s="82"/>
     </row>
-    <row r="458" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="458" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A458" s="3" t="s">
         <v>1074</v>
       </c>
@@ -55275,7 +55279,7 @@
       <c r="AN458" s="82"/>
       <c r="AO458" s="82"/>
     </row>
-    <row r="459" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="459" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A459" s="3" t="s">
         <v>1075</v>
       </c>
@@ -55359,7 +55363,7 @@
       <c r="AN459" s="82"/>
       <c r="AO459" s="82"/>
     </row>
-    <row r="460" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="460" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A460" s="3" t="s">
         <v>1077</v>
       </c>
@@ -55443,7 +55447,7 @@
       <c r="AN460" s="82"/>
       <c r="AO460" s="82"/>
     </row>
-    <row r="461" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="461" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A461" s="3" t="s">
         <v>1078</v>
       </c>
@@ -55527,7 +55531,7 @@
       <c r="AN461" s="82"/>
       <c r="AO461" s="82"/>
     </row>
-    <row r="462" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="462" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A462" s="3" t="s">
         <v>1079</v>
       </c>
@@ -55611,7 +55615,7 @@
       <c r="AN462" s="82"/>
       <c r="AO462" s="82"/>
     </row>
-    <row r="463" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="463" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A463" s="3" t="s">
         <v>1080</v>
       </c>
@@ -55699,7 +55703,7 @@
       <c r="AN463" s="82"/>
       <c r="AO463" s="82"/>
     </row>
-    <row r="464" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="464" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A464" s="3" t="s">
         <v>1081</v>
       </c>
@@ -55783,7 +55787,7 @@
       <c r="AN464" s="82"/>
       <c r="AO464" s="82"/>
     </row>
-    <row r="465" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="465" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A465" s="3" t="s">
         <v>1082</v>
       </c>
@@ -55867,7 +55871,7 @@
       <c r="AN465" s="82"/>
       <c r="AO465" s="82"/>
     </row>
-    <row r="466" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="466" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A466" s="3" t="s">
         <v>1083</v>
       </c>
@@ -55951,7 +55955,7 @@
       <c r="AN466" s="82"/>
       <c r="AO466" s="82"/>
     </row>
-    <row r="467" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="467" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A467" s="3" t="s">
         <v>1085</v>
       </c>
@@ -56035,7 +56039,7 @@
       <c r="AN467" s="82"/>
       <c r="AO467" s="82"/>
     </row>
-    <row r="468" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="468" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A468" s="3" t="s">
         <v>1087</v>
       </c>
@@ -56119,7 +56123,7 @@
       <c r="AN468" s="82"/>
       <c r="AO468" s="82"/>
     </row>
-    <row r="469" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="469" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A469" s="3" t="s">
         <v>1089</v>
       </c>
@@ -56203,7 +56207,7 @@
       <c r="AN469" s="82"/>
       <c r="AO469" s="82"/>
     </row>
-    <row r="470" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="470" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A470" s="3" t="s">
         <v>1090</v>
       </c>
@@ -56287,7 +56291,7 @@
       <c r="AN470" s="82"/>
       <c r="AO470" s="82"/>
     </row>
-    <row r="471" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="471" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A471" s="3" t="s">
         <v>1091</v>
       </c>
@@ -56371,7 +56375,7 @@
       <c r="AN471" s="82"/>
       <c r="AO471" s="82"/>
     </row>
-    <row r="472" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="472" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A472" s="3" t="s">
         <v>1092</v>
       </c>
@@ -56455,7 +56459,7 @@
       <c r="AN472" s="82"/>
       <c r="AO472" s="82"/>
     </row>
-    <row r="473" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="473" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A473" s="3" t="s">
         <v>1094</v>
       </c>
@@ -56539,7 +56543,7 @@
       <c r="AN473" s="82"/>
       <c r="AO473" s="82"/>
     </row>
-    <row r="474" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="474" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A474" s="3" t="s">
         <v>1096</v>
       </c>
@@ -56623,7 +56627,7 @@
       <c r="AN474" s="82"/>
       <c r="AO474" s="82"/>
     </row>
-    <row r="475" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="475" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A475" s="3" t="s">
         <v>1098</v>
       </c>
@@ -56707,7 +56711,7 @@
       <c r="AN475" s="82"/>
       <c r="AO475" s="82"/>
     </row>
-    <row r="476" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="476" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A476" s="3" t="s">
         <v>1100</v>
       </c>
@@ -56791,7 +56795,7 @@
       <c r="AN476" s="82"/>
       <c r="AO476" s="82"/>
     </row>
-    <row r="477" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="477" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A477" s="3" t="s">
         <v>1102</v>
       </c>
@@ -56879,7 +56883,7 @@
       <c r="AN477" s="82"/>
       <c r="AO477" s="82"/>
     </row>
-    <row r="478" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="478" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A478" s="3" t="s">
         <v>1103</v>
       </c>
@@ -56967,7 +56971,7 @@
       <c r="AN478" s="82"/>
       <c r="AO478" s="82"/>
     </row>
-    <row r="479" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="479" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A479" s="3" t="s">
         <v>1104</v>
       </c>
@@ -57055,7 +57059,7 @@
       <c r="AN479" s="82"/>
       <c r="AO479" s="82"/>
     </row>
-    <row r="480" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="480" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A480" s="3" t="s">
         <v>1105</v>
       </c>
@@ -57139,7 +57143,7 @@
       <c r="AN480" s="82"/>
       <c r="AO480" s="82"/>
     </row>
-    <row r="481" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="481" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A481" s="3" t="s">
         <v>1107</v>
       </c>
@@ -57223,7 +57227,7 @@
       <c r="AN481" s="82"/>
       <c r="AO481" s="82"/>
     </row>
-    <row r="482" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="482" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A482" s="3" t="s">
         <v>1108</v>
       </c>
@@ -57307,7 +57311,7 @@
       <c r="AN482" s="82"/>
       <c r="AO482" s="82"/>
     </row>
-    <row r="483" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="483" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A483" s="3" t="s">
         <v>1109</v>
       </c>
@@ -57395,7 +57399,7 @@
       <c r="AN483" s="82"/>
       <c r="AO483" s="82"/>
     </row>
-    <row r="484" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="484" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A484" s="3" t="s">
         <v>1110</v>
       </c>
@@ -57483,7 +57487,7 @@
       <c r="AN484" s="82"/>
       <c r="AO484" s="82"/>
     </row>
-    <row r="485" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="485" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A485" s="3" t="s">
         <v>1111</v>
       </c>
@@ -57567,7 +57571,7 @@
       <c r="AN485" s="82"/>
       <c r="AO485" s="82"/>
     </row>
-    <row r="486" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="486" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A486" s="22" t="s">
         <v>1113</v>
       </c>
@@ -57651,7 +57655,7 @@
       <c r="AN486" s="82"/>
       <c r="AO486" s="82"/>
     </row>
-    <row r="487" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="487" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A487" s="22" t="s">
         <v>1114</v>
       </c>
@@ -57735,7 +57739,7 @@
       <c r="AN487" s="82"/>
       <c r="AO487" s="82"/>
     </row>
-    <row r="488" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="488" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A488" s="22" t="s">
         <v>1116</v>
       </c>
@@ -57819,7 +57823,7 @@
       <c r="AN488" s="82"/>
       <c r="AO488" s="82"/>
     </row>
-    <row r="489" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="489" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A489" s="22" t="s">
         <v>1117</v>
       </c>
@@ -57903,7 +57907,7 @@
       <c r="AN489" s="82"/>
       <c r="AO489" s="82"/>
     </row>
-    <row r="490" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="490" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A490" s="22" t="s">
         <v>1118</v>
       </c>
@@ -57987,7 +57991,7 @@
       <c r="AN490" s="82"/>
       <c r="AO490" s="82"/>
     </row>
-    <row r="491" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="491" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A491" s="22" t="s">
         <v>1119</v>
       </c>
@@ -58079,7 +58083,7 @@
       <c r="AN491" s="82"/>
       <c r="AO491" s="82"/>
     </row>
-    <row r="492" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="492" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A492" s="22" t="s">
         <v>452</v>
       </c>
@@ -58159,7 +58163,7 @@
       <c r="AN492" s="82"/>
       <c r="AO492" s="82"/>
     </row>
-    <row r="493" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="493" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A493" s="22" t="s">
         <v>1122</v>
       </c>
@@ -58229,7 +58233,7 @@
       <c r="AN493" s="82"/>
       <c r="AO493" s="82"/>
     </row>
-    <row r="494" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="494" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A494" s="22" t="s">
         <v>1124</v>
       </c>
@@ -58299,7 +58303,7 @@
       <c r="AN494" s="82"/>
       <c r="AO494" s="82"/>
     </row>
-    <row r="495" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="495" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A495" s="22" t="s">
         <v>1125</v>
       </c>
@@ -58369,7 +58373,7 @@
       <c r="AN495" s="82"/>
       <c r="AO495" s="82"/>
     </row>
-    <row r="496" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="496" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A496" s="22" t="s">
         <v>1126</v>
       </c>
@@ -58439,7 +58443,7 @@
       <c r="AN496" s="82"/>
       <c r="AO496" s="82"/>
     </row>
-    <row r="497" spans="1:41" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
+    <row r="497" spans="1:41" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A497" s="22" t="s">
         <v>1127</v>
       </c>
@@ -77475,7 +77479,7 @@
   <autoFilter ref="A2:AO710" xr:uid="{2AA437EE-405D-4A43-9EB9-23F1BEB36011}">
     <filterColumn colId="17">
       <filters>
-        <filter val="Diadema"/>
+        <filter val="Ferraz"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -78441,15 +78445,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="f5ab1930-d403-4c69-b2cd-8cc48f527d10" xsi:nil="true"/>
@@ -78458,6 +78453,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -78656,26 +78660,26 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5AE26D3A-03CC-4B3D-9F98-6F77A1AEA74E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE495743-F761-4961-A762-7A3D120C6961}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f5ab1930-d403-4c69-b2cd-8cc48f527d10"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="c06ce65c-ed18-47f4-a957-afd315448c9c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE495743-F761-4961-A762-7A3D120C6961}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5AE26D3A-03CC-4B3D-9F98-6F77A1AEA74E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="f5ab1930-d403-4c69-b2cd-8cc48f527d10"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c06ce65c-ed18-47f4-a957-afd315448c9c"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>